<commit_message>
chore: update competitor intelligence data
</commit_message>
<xml_diff>
--- a/competitor_campaigns_latest.xlsx
+++ b/competitor_campaigns_latest.xlsx
@@ -6012,17 +6012,17 @@
       </x:c>
       <x:c r="O10" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://www.instagram.com/reel/DbJTohBs04q/</x:t>
+          <x:t xml:space="preserve">https://www.instagram.com/p/Db5ZNugDGsU</x:t>
         </x:is>
       </x:c>
       <x:c r="P10" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://x.com/stcbank_ksa/status/2071588243682832478</x:t>
+          <x:t xml:space="preserve">https://x.com/stcbank_ksa/status/2087125864437998021</x:t>
         </x:is>
       </x:c>
       <x:c r="Q10" s="63" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://www.facebook.com/share/v/1BoJpH5Xnd/</x:t>
+          <x:t xml:space="preserve">https://m.facebook.com/stcbank/posts/pfbid0z3FCbNVN2HZG9xUqpxyvHVrGnKCksURgXzJ2hd58fy55RpZ7wptbLuVAkAGrMfesl</x:t>
         </x:is>
       </x:c>
       <x:c r="R10" s="4"/>
@@ -7162,7 +7162,7 @@
       </x:c>
       <x:c r="C26" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Valid until 18 Sep 2026 15% discount from SQUATWOLF! Enjoy your purchases from SQUATWOLF using STC Bank Visa cards.</x:t>
+          <x:t xml:space="preserve">Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from Roasting House, in addition to 10% off all products in branches using…</x:t>
         </x:is>
       </x:c>
       <x:c r="D26" s="4" t="inlineStr">
@@ -7187,7 +7187,7 @@
       </x:c>
       <x:c r="N26" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/squatwolf</x:t>
+          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/roastinghouse2</x:t>
         </x:is>
       </x:c>
       <x:c r="O26" s="4"/>
@@ -7211,7 +7211,7 @@
       </x:c>
       <x:c r="C27" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Valid until 27 Dec 2027 10% off from GrintaHub Enjoy an exclusive 10% off offer on the GrintaHub website and app with all STC Bank cards.</x:t>
+          <x:t xml:space="preserve">Valid until 18 Sep 2026 15% discount from SQUATWOLF! Enjoy your purchases from SQUATWOLF using STC Bank Visa cards.</x:t>
         </x:is>
       </x:c>
       <x:c r="D27" s="4" t="inlineStr">
@@ -7236,7 +7236,7 @@
       </x:c>
       <x:c r="N27" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/grintahub</x:t>
+          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/squatwolf</x:t>
         </x:is>
       </x:c>
       <x:c r="O27" s="4"/>
@@ -7260,7 +7260,7 @@
       </x:c>
       <x:c r="C28" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Valid until 30 Sep 2026 15% discount from Madame Tussauds Walk around Madame Tussauds London using STC Bank Visa cards.</x:t>
+          <x:t xml:space="preserve">Valid until 19 Oct 2026 75% off on car repair services from MisMar Your safety matters to us. We offer you a 75% discount on the MisMar app using all STC Bank cards.</x:t>
         </x:is>
       </x:c>
       <x:c r="D28" s="4" t="inlineStr">
@@ -7285,7 +7285,7 @@
       </x:c>
       <x:c r="N28" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/madame-tussauds</x:t>
+          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/cars-replacement</x:t>
         </x:is>
       </x:c>
       <x:c r="O28" s="4"/>
@@ -7309,7 +7309,7 @@
       </x:c>
       <x:c r="C29" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Valid until 30 Sep 2026 15% off on London Eye tickets! Enjoy a London Eye visit with 15% off on tickets using Visa payment cards and Credit cards from STC Bank.</x:t>
+          <x:t xml:space="preserve">Valid until 2 Oct 2026 Indulge in fine dining around UAE! Enjoy the most delicious dishes with up to 25% off at various restaurants using STC Bank Visa cards.</x:t>
         </x:is>
       </x:c>
       <x:c r="D29" s="4" t="inlineStr">
@@ -7334,7 +7334,7 @@
       </x:c>
       <x:c r="N29" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/london-eye</x:t>
+          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/indulge-in-fine-dining-around-uae</x:t>
         </x:is>
       </x:c>
       <x:c r="O29" s="4"/>
@@ -7358,7 +7358,7 @@
       </x:c>
       <x:c r="C30" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Valid until 31 Dec 2027 10% discount on The Bicester Collection Luxurious shopping in The Bicester Collection in the UK using STC Bank Visa cards.</x:t>
+          <x:t xml:space="preserve">Valid until 21 Dec 2026 15% off on coffee products from Roasting House Make your own coffee with a 15% off from Roasting House using all STC Bank cards.</x:t>
         </x:is>
       </x:c>
       <x:c r="D30" s="4" t="inlineStr">
@@ -7383,7 +7383,7 @@
       </x:c>
       <x:c r="N30" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/the-bicester</x:t>
+          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/roasting-house</x:t>
         </x:is>
       </x:c>
       <x:c r="O30" s="4"/>
@@ -7407,7 +7407,7 @@
       </x:c>
       <x:c r="C31" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Valid until 31 Dec 2027 15% discount from Legoland Make enjoyable memories with Legoland in the UK using STC Bank Visa cards.</x:t>
+          <x:t xml:space="preserve">Valid until 27 Dec 2027 10% off from GrintaHub Enjoy an exclusive 10% off offer on the GrintaHub website and app with all STC Bank cards.</x:t>
         </x:is>
       </x:c>
       <x:c r="D31" s="4" t="inlineStr">
@@ -7432,7 +7432,7 @@
       </x:c>
       <x:c r="N31" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/legoland</x:t>
+          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/grintahub</x:t>
         </x:is>
       </x:c>
       <x:c r="O31" s="4"/>
@@ -7456,7 +7456,7 @@
       </x:c>
       <x:c r="C32" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Valid until 31 Dec 2027 A Unique Experience at the Musée du Louvre! Enjoy priority entry to the Louvre Museum, plus entry for up to 3 guests, with your STC Bank Infinite Credit Ca…</x:t>
+          <x:t xml:space="preserve">Valid until 30 Dec 2027 10% off on perfumes from Golden Scent Order your Eid perfumes from Golden Scent with 10% discount using all STC Bank cards.</x:t>
         </x:is>
       </x:c>
       <x:c r="D32" s="4" t="inlineStr">
@@ -7481,7 +7481,7 @@
       </x:c>
       <x:c r="N32" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/du-louvre</x:t>
+          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/goldenscent</x:t>
         </x:is>
       </x:c>
       <x:c r="O32" s="4"/>
@@ -7505,7 +7505,7 @@
       </x:c>
       <x:c r="C33" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Valid until 31 Dec 2027 A Unique Shopping Experience at La Vallée Village! Enjoy 12% off purchases from tax-free (via Global Blue), €5 refreshment vouchers and hands-free shopping…</x:t>
+          <x:t xml:space="preserve">Valid until 30 Sep 2026 15% discount from Madame Tussauds Walk around Madame Tussauds London using STC Bank Visa cards.</x:t>
         </x:is>
       </x:c>
       <x:c r="D33" s="4" t="inlineStr">
@@ -7530,7 +7530,7 @@
       </x:c>
       <x:c r="N33" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/la-vallee</x:t>
+          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/madame-tussauds</x:t>
         </x:is>
       </x:c>
       <x:c r="O33" s="4"/>
@@ -7554,7 +7554,7 @@
       </x:c>
       <x:c r="C34" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Valid until 31 Dec 2027 A luxurious shopping in Printemps Haussmann, Paris Enjoy shopping with unique services using STC Bank Visa cards.</x:t>
+          <x:t xml:space="preserve">Valid until 30 Sep 2026 15% off on London Eye tickets! Enjoy a London Eye visit with 15% off on tickets using Visa payment cards and Credit cards from STC Bank.</x:t>
         </x:is>
       </x:c>
       <x:c r="D34" s="4" t="inlineStr">
@@ -7579,7 +7579,7 @@
       </x:c>
       <x:c r="N34" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/printemps-haussmann</x:t>
+          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/london-eye</x:t>
         </x:is>
       </x:c>
       <x:c r="O34" s="4"/>
@@ -7603,17 +7603,15 @@
       </x:c>
       <x:c r="C35" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">قهوة الأربعاء بهللة وحدة بس من بيت التحميص 😍#اكسبلور #STCBank #explore</x:t>
+          <x:t xml:space="preserve">Valid until 31 Aug 2026 15% discount from Ladeena Renew your care routine with Ladeena products with refreshing and different scents.</x:t>
         </x:is>
       </x:c>
       <x:c r="D35" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">قهوة الأربعاء بهللة وحدة بس من بيت التحميص 😍#اكسبلور #STCBank #explore ♬ original sound - STC Bank</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E35" s="5" t="n">
-        <x:v>46245.859085648146</x:v>
-      </x:c>
+          <x:t xml:space="preserve">Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from Roasting House, in addition to 10% off all products in branches using all STC Bank cards. Valid until 2 Oct 2026 Earn cash amount on international purchases! Exclusively for selected customers, earn a cash amount on international purchases using Visa payment cards from STC Bank. Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from…</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E35" s="5"/>
       <x:c r="F35" s="5"/>
       <x:c r="G35" s="5"/>
       <x:c r="H35" s="7" t="str">
@@ -7628,15 +7626,15 @@
       <x:c r="M35" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N35" s="4"/>
+      <x:c r="N35" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/ladeena</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O35" s="4"/>
       <x:c r="P35" s="4"/>
       <x:c r="Q35" s="4"/>
-      <x:c r="R35" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.tiktok.com/@stcbank_ksa/video/7672875813536091412</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="R35" s="4"/>
       <x:c r="S35" s="4"/>
       <x:c r="T35" s="5"/>
       <x:c r="U35" s="35" t="str">
@@ -7654,17 +7652,15 @@
       </x:c>
       <x:c r="C36" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">هللة وش تجيب لك؟ 👀</x:t>
+          <x:t xml:space="preserve">Valid until 31 Dec 2027 10% discount on The Bicester Collection Luxurious shopping in The Bicester Collection in the UK using STC Bank Visa cards.</x:t>
         </x:is>
       </x:c>
       <x:c r="D36" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">هللة وش تجيب لك؟ 👀 — STC Bank (@stcbank_ksa) Aug 11, 2026</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E36" s="5" t="n">
-        <x:v>46245.84652777778</x:v>
-      </x:c>
+          <x:t xml:space="preserve">Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from Roasting House, in addition to 10% off all products in branches using all STC Bank cards. Valid until 2 Oct 2026 Earn cash amount on international purchases! Exclusively for selected customers, earn a cash amount on international purchases using Visa payment cards from STC Bank. Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from…</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E36" s="5"/>
       <x:c r="F36" s="5"/>
       <x:c r="G36" s="5"/>
       <x:c r="H36" s="7" t="str">
@@ -7679,13 +7675,13 @@
       <x:c r="M36" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N36" s="4"/>
+      <x:c r="N36" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/the-bicester</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O36" s="4"/>
-      <x:c r="P36" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://x.com/stcbank_ksa/status/2087272653434339756</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="P36" s="4"/>
       <x:c r="Q36" s="4"/>
       <x:c r="R36" s="4"/>
       <x:c r="S36" s="4"/>
@@ -7698,9 +7694,21 @@
       <x:c r="A37" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B37" s="4"/>
-      <x:c r="C37" s="4"/>
-      <x:c r="D37" s="4"/>
+      <x:c r="B37" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C37" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Valid until 31 Dec 2027 15% discount from Legoland Make enjoyable memories with Legoland in the UK using STC Bank Visa cards.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D37" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from Roasting House, in addition to 10% off all products in branches using all STC Bank cards. Valid until 2 Oct 2026 Earn cash amount on international purchases! Exclusively for selected customers, earn a cash amount on international purchases using Visa payment cards from STC Bank. Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from…</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E37" s="5"/>
       <x:c r="F37" s="5"/>
       <x:c r="G37" s="5"/>
@@ -7716,7 +7724,11 @@
       <x:c r="M37" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N37" s="4"/>
+      <x:c r="N37" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/legoland</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O37" s="4"/>
       <x:c r="P37" s="4"/>
       <x:c r="Q37" s="4"/>
@@ -7731,9 +7743,21 @@
       <x:c r="A38" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B38" s="4"/>
-      <x:c r="C38" s="4"/>
-      <x:c r="D38" s="4"/>
+      <x:c r="B38" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C38" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Valid until 31 Dec 2027 20% off with 4 Wheel Station for cars Enjoy up to 20% off with 4 Wheel Station using STC Bank cards.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D38" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from Roasting House, in addition to 10% off all products in branches using all STC Bank cards. Valid until 2 Oct 2026 Earn cash amount on international purchases! Exclusively for selected customers, earn a cash amount on international purchases using Visa payment cards from STC Bank. Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from…</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E38" s="5"/>
       <x:c r="F38" s="5"/>
       <x:c r="G38" s="5"/>
@@ -7749,7 +7773,11 @@
       <x:c r="M38" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N38" s="4"/>
+      <x:c r="N38" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/4-wheel</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O38" s="4"/>
       <x:c r="P38" s="4"/>
       <x:c r="Q38" s="4"/>
@@ -7764,9 +7792,21 @@
       <x:c r="A39" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B39" s="4"/>
-      <x:c r="C39" s="4"/>
-      <x:c r="D39" s="4"/>
+      <x:c r="B39" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C39" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Valid until 31 Dec 2027 50% off on Ultra Shield car services Enjoy a 50% discount on Ultra Shield services to protect your car from heat and scratches.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D39" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from Roasting House, in addition to 10% off all products in branches using all STC Bank cards. Valid until 2 Oct 2026 Earn cash amount on international purchases! Exclusively for selected customers, earn a cash amount on international purchases using Visa payment cards from STC Bank. Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from…</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E39" s="5"/>
       <x:c r="F39" s="5"/>
       <x:c r="G39" s="5"/>
@@ -7782,7 +7822,11 @@
       <x:c r="M39" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N39" s="4"/>
+      <x:c r="N39" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/scratches</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O39" s="4"/>
       <x:c r="P39" s="4"/>
       <x:c r="Q39" s="4"/>
@@ -7797,9 +7841,21 @@
       <x:c r="A40" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B40" s="4"/>
-      <x:c r="C40" s="4"/>
-      <x:c r="D40" s="4"/>
+      <x:c r="B40" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C40" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Valid until 31 Dec 2027 A Unique Experience at Galeries Lafayette! Enjoy free premium lounge access alongside refreshments, fast-track tax refunds and hands-free shopping with Vis…</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D40" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from Roasting House, in addition to 10% off all products in branches using all STC Bank cards. Valid until 2 Oct 2026 Earn cash amount on international purchases! Exclusively for selected customers, earn a cash amount on international purchases using Visa payment cards from STC Bank. Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from…</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E40" s="5"/>
       <x:c r="F40" s="5"/>
       <x:c r="G40" s="5"/>
@@ -7815,7 +7871,11 @@
       <x:c r="M40" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N40" s="4"/>
+      <x:c r="N40" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/galeries</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O40" s="4"/>
       <x:c r="P40" s="4"/>
       <x:c r="Q40" s="4"/>
@@ -7830,9 +7890,21 @@
       <x:c r="A41" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B41" s="4"/>
-      <x:c r="C41" s="4"/>
-      <x:c r="D41" s="4"/>
+      <x:c r="B41" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C41" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Valid until 31 Dec 2027 A Unique Experience at the Musée du Louvre! Enjoy priority entry to the Louvre Museum, plus entry for up to 3 guests, with your STC Bank Infinite Credit Ca…</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D41" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from Roasting House, in addition to 10% off all products in branches using all STC Bank cards. Valid until 2 Oct 2026 Earn cash amount on international purchases! Exclusively for selected customers, earn a cash amount on international purchases using Visa payment cards from STC Bank. Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from…</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E41" s="5"/>
       <x:c r="F41" s="5"/>
       <x:c r="G41" s="5"/>
@@ -7848,7 +7920,11 @@
       <x:c r="M41" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N41" s="4"/>
+      <x:c r="N41" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/du-louvre</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O41" s="4"/>
       <x:c r="P41" s="4"/>
       <x:c r="Q41" s="4"/>
@@ -7863,9 +7939,21 @@
       <x:c r="A42" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B42" s="4"/>
-      <x:c r="C42" s="4"/>
-      <x:c r="D42" s="4"/>
+      <x:c r="B42" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C42" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Valid until 31 Dec 2027 A Unique Shopping Experience at La Vallée Village! Enjoy 12% off purchases from tax-free (via Global Blue), €5 refreshment vouchers and hands-free shopping…</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D42" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from Roasting House, in addition to 10% off all products in branches using all STC Bank cards. Valid until 2 Oct 2026 Earn cash amount on international purchases! Exclusively for selected customers, earn a cash amount on international purchases using Visa payment cards from STC Bank. Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from…</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E42" s="5"/>
       <x:c r="F42" s="5"/>
       <x:c r="G42" s="5"/>
@@ -7881,7 +7969,11 @@
       <x:c r="M42" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N42" s="4"/>
+      <x:c r="N42" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/la-vallee</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O42" s="4"/>
       <x:c r="P42" s="4"/>
       <x:c r="Q42" s="4"/>
@@ -7896,9 +7988,21 @@
       <x:c r="A43" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B43" s="4"/>
-      <x:c r="C43" s="4"/>
-      <x:c r="D43" s="4"/>
+      <x:c r="B43" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C43" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Valid until 31 Dec 2027 A luxurious shopping in Printemps Haussmann, Paris Enjoy shopping with unique services using STC Bank Visa cards.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D43" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from Roasting House, in addition to 10% off all products in branches using all STC Bank cards. Valid until 2 Oct 2026 Earn cash amount on international purchases! Exclusively for selected customers, earn a cash amount on international purchases using Visa payment cards from STC Bank. Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from…</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E43" s="5"/>
       <x:c r="F43" s="5"/>
       <x:c r="G43" s="5"/>
@@ -7914,7 +8018,11 @@
       <x:c r="M43" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N43" s="4"/>
+      <x:c r="N43" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/printemps-haussmann</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O43" s="4"/>
       <x:c r="P43" s="4"/>
       <x:c r="Q43" s="4"/>
@@ -7929,9 +8037,21 @@
       <x:c r="A44" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B44" s="4"/>
-      <x:c r="C44" s="4"/>
-      <x:c r="D44" s="4"/>
+      <x:c r="B44" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C44" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Valid until 31 Dec 2027 Elegance is the essence of Sayyar with a 20% off Sayyar is your choice for men’s luxury with 20% off and free delivery using all STC Bank cards.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D44" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from Roasting House, in addition to 10% off all products in branches using all STC Bank cards. Valid until 2 Oct 2026 Earn cash amount on international purchases! Exclusively for selected customers, earn a cash amount on international purchases using Visa payment cards from STC Bank. Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from…</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E44" s="5"/>
       <x:c r="F44" s="5"/>
       <x:c r="G44" s="5"/>
@@ -7947,7 +8067,11 @@
       <x:c r="M44" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N44" s="4"/>
+      <x:c r="N44" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/new_sayyar</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O44" s="4"/>
       <x:c r="P44" s="4"/>
       <x:c r="Q44" s="4"/>
@@ -7962,9 +8086,21 @@
       <x:c r="A45" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B45" s="4"/>
-      <x:c r="C45" s="4"/>
-      <x:c r="D45" s="4"/>
+      <x:c r="B45" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C45" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Valid until 31 Dec 2027 Refresh your space with new plants and enjoy a 15% discount from Nabataty! Enjoy a 15% discount on a variety of plants from the Nabataty website and app us…</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D45" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from Roasting House, in addition to 10% off all products in branches using all STC Bank cards. Valid until 2 Oct 2026 Earn cash amount on international purchases! Exclusively for selected customers, earn a cash amount on international purchases using Visa payment cards from STC Bank. Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from…</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E45" s="5"/>
       <x:c r="F45" s="5"/>
       <x:c r="G45" s="5"/>
@@ -7980,7 +8116,11 @@
       <x:c r="M45" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N45" s="4"/>
+      <x:c r="N45" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/nabataty</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O45" s="4"/>
       <x:c r="P45" s="4"/>
       <x:c r="Q45" s="4"/>
@@ -7995,9 +8135,21 @@
       <x:c r="A46" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B46" s="4"/>
-      <x:c r="C46" s="4"/>
-      <x:c r="D46" s="4"/>
+      <x:c r="B46" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C46" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Valid until 6 Apr 2027 Polish and protect your car with a 20% discount from Dettaglioauto! Enjoy a 20% discount at Dettaglioauto branches around KSA, using any STC Bank card.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D46" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from Roasting House, in addition to 10% off all products in branches using all STC Bank cards. Valid until 2 Oct 2026 Earn cash amount on international purchases! Exclusively for selected customers, earn a cash amount on international purchases using Visa payment cards from STC Bank. Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from…</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E46" s="5"/>
       <x:c r="F46" s="5"/>
       <x:c r="G46" s="5"/>
@@ -8013,7 +8165,11 @@
       <x:c r="M46" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N46" s="4"/>
+      <x:c r="N46" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/dettaglioauto-offer</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O46" s="4"/>
       <x:c r="P46" s="4"/>
       <x:c r="Q46" s="4"/>
@@ -8028,10 +8184,24 @@
       <x:c r="A47" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B47" s="4"/>
-      <x:c r="C47" s="4"/>
-      <x:c r="D47" s="4"/>
-      <x:c r="E47" s="5"/>
+      <x:c r="B47" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Card</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C47" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">جوائز حملة صفّرناها ماتوقف ألف مبروووك للـ 50 فائز، كل فائز ربح قسيمة سفر بقيمة 10,000 ريال 🎉 باقي 50 شخص، خلّك من الأع...</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D47" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">جوائز حملة صفّرناها ماتوقف ألف مبروووك للـ 50 فائز، كل فائز ربح قسيمة سفر بقيمة 10,000 ريال 🎉 باقي 50 شخص، خلّك من الأعلى إنفاقًا دوليًا مع بطاقات الدفع Visa من STC Bank وفالك الفوووز ✈️ الحملة مستمرة الى 3 سبتمبر 2026 https://stcbank.com.sa/…/international-purchases-with-0-fees</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E47" s="5" t="n">
+        <x:v>46245.444085648145</x:v>
+      </x:c>
       <x:c r="F47" s="5"/>
       <x:c r="G47" s="5"/>
       <x:c r="H47" s="7" t="str">
@@ -8049,7 +8219,11 @@
       <x:c r="N47" s="4"/>
       <x:c r="O47" s="4"/>
       <x:c r="P47" s="4"/>
-      <x:c r="Q47" s="4"/>
+      <x:c r="Q47" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://m.facebook.com/stcbank/posts/pfbid0z3FCbNVN2HZG9xUqpxyvHVrGnKCksURgXzJ2hd58fy55RpZ7wptbLuVAkAGrMfesl</x:t>
+        </x:is>
+      </x:c>
       <x:c r="R47" s="4"/>
       <x:c r="S47" s="4"/>
       <x:c r="T47" s="5"/>
@@ -8061,10 +8235,24 @@
       <x:c r="A48" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B48" s="4"/>
-      <x:c r="C48" s="4"/>
-      <x:c r="D48" s="4"/>
-      <x:c r="E48" s="5"/>
+      <x:c r="B48" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Card</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C48" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">جوائز حملة صفّرناها ماتوقف ألف مبروووك للـ 50 فائز، كل فائز ربح قسيمة سفر بقيمة 10,000 ريال 🎉 باقي 50 شخص، خلّك من الأعلى إنفاقًا دوليًا مع بطاقات الدفع Visa من STC Bank وفالك الف…</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D48" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">جوائز حملة صفّرناها ماتوقف ألف مبروووك للـ 50 فائز، كل فائز ربح قسيمة سفر بقيمة 10,000 ريال 🎉 باقي 50 شخص، خلّك من الأعلى إنفاقًا دوليًا مع بطاقات الدفع Visa من STC Bank وفالك الفوووز ✈️ الحملة مستمرة الى 3 سبتمبر 2026 — STC Bank (@stcbank_ksa) Aug 11, 2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E48" s="5" t="n">
+        <x:v>46245.44097222222</x:v>
+      </x:c>
       <x:c r="F48" s="5"/>
       <x:c r="G48" s="5"/>
       <x:c r="H48" s="7" t="str">
@@ -8081,7 +8269,11 @@
       </x:c>
       <x:c r="N48" s="4"/>
       <x:c r="O48" s="4"/>
-      <x:c r="P48" s="4"/>
+      <x:c r="P48" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://x.com/stcbank_ksa/status/2087125864437998021</x:t>
+        </x:is>
+      </x:c>
       <x:c r="Q48" s="4"/>
       <x:c r="R48" s="4"/>
       <x:c r="S48" s="4"/>
@@ -8094,10 +8286,24 @@
       <x:c r="A49" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B49" s="4"/>
-      <x:c r="C49" s="4"/>
-      <x:c r="D49" s="4"/>
-      <x:c r="E49" s="5"/>
+      <x:c r="B49" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C49" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">قهوة الأربعاء بهللة وحدة بس من بيت التحميص 😍#اكسبلور #STCBank #explore</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D49" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">قهوة الأربعاء بهللة وحدة بس من بيت التحميص 😍#اكسبلور #STCBank #explore ♬ original sound - STC Bank</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E49" s="5" t="n">
+        <x:v>46245.859085648146</x:v>
+      </x:c>
       <x:c r="F49" s="5"/>
       <x:c r="G49" s="5"/>
       <x:c r="H49" s="7" t="str">
@@ -8116,7 +8322,11 @@
       <x:c r="O49" s="4"/>
       <x:c r="P49" s="4"/>
       <x:c r="Q49" s="4"/>
-      <x:c r="R49" s="4"/>
+      <x:c r="R49" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.tiktok.com/@stcbank_ksa/video/7672875813536091412</x:t>
+        </x:is>
+      </x:c>
       <x:c r="S49" s="4"/>
       <x:c r="T49" s="5"/>
       <x:c r="U49" s="35" t="str">
@@ -8127,10 +8337,24 @@
       <x:c r="A50" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B50" s="4"/>
-      <x:c r="C50" s="4"/>
-      <x:c r="D50" s="4"/>
-      <x:c r="E50" s="5"/>
+      <x:c r="B50" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C50" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">هللة وش تجيب لك؟ 👀</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D50" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">هللة وش تجيب لك؟ 👀 — STC Bank (@stcbank_ksa) Aug 11, 2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E50" s="5" t="n">
+        <x:v>46245.84652777778</x:v>
+      </x:c>
       <x:c r="F50" s="5"/>
       <x:c r="G50" s="5"/>
       <x:c r="H50" s="7" t="str">
@@ -8147,7 +8371,11 @@
       </x:c>
       <x:c r="N50" s="4"/>
       <x:c r="O50" s="4"/>
-      <x:c r="P50" s="4"/>
+      <x:c r="P50" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://x.com/stcbank_ksa/status/2087272653434339756</x:t>
+        </x:is>
+      </x:c>
       <x:c r="Q50" s="4"/>
       <x:c r="R50" s="4"/>
       <x:c r="S50" s="4"/>
@@ -8910,7 +9138,7 @@
         </x:is>
       </x:c>
       <x:c r="T13" s="5" t="n">
-        <x:v>46240.0</x:v>
+        <x:v>46246.20490914237</x:v>
       </x:c>
       <x:c r="U13" s="35" t="str">
         <x:f t="shared" si="3">IF(C13="","",IF(COUNTA(O13:R13)=0,"No direct social post verified",IF(O13&lt;&gt;"","Instagram","")&amp;IF(AND(O13&lt;&gt;"",OR(P13&lt;&gt;"",Q13&lt;&gt;"",R13&lt;&gt;"")),", ","")&amp;IF(P13&lt;&gt;"","X","")&amp;IF(AND(P13&lt;&gt;"",OR(Q13&lt;&gt;"",R13&lt;&gt;"")),", ","")&amp;IF(Q13&lt;&gt;"","Facebook","")&amp;IF(AND(Q13&lt;&gt;"",R13&lt;&gt;""),", ","")&amp;IF(R13&lt;&gt;"","TikTok","")))</x:f>
@@ -8932,7 +9160,11 @@
           <x:t xml:space="preserve">FX Rate Awareness Campaign</x:t>
         </x:is>
       </x:c>
-      <x:c r="D14" s="4"/>
+      <x:c r="D14" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">‏‎85 likes, 21 comments - ‎‏‏‎usebarq‎‏ في ‏‎July 5, 2026‎‏‏: "⁨ كل دولار يفرق، والفرق يبقى معك ⚡️⁩". ‏</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E14" s="5"/>
       <x:c r="F14" s="5"/>
       <x:c r="G14" s="5"/>
@@ -8973,7 +9205,7 @@
       <x:c r="R14" s="4"/>
       <x:c r="S14" s="4"/>
       <x:c r="T14" s="5" t="n">
-        <x:v>46240.0</x:v>
+        <x:v>46246.20490914237</x:v>
       </x:c>
       <x:c r="U14" s="35" t="str">
         <x:f t="shared" si="3">IF(C14="","",IF(COUNTA(O14:R14)=0,"No direct social post verified",IF(O14&lt;&gt;"","Instagram","")&amp;IF(AND(O14&lt;&gt;"",OR(P14&lt;&gt;"",Q14&lt;&gt;"",R14&lt;&gt;"")),", ","")&amp;IF(P14&lt;&gt;"","X","")&amp;IF(AND(P14&lt;&gt;"",OR(Q14&lt;&gt;"",R14&lt;&gt;"")),", ","")&amp;IF(Q14&lt;&gt;"","Facebook","")&amp;IF(AND(Q14&lt;&gt;"",R14&lt;&gt;""),", ","")&amp;IF(R14&lt;&gt;"","TikTok","")))</x:f>
@@ -8991,16 +9223,16 @@
       </x:c>
       <x:c r="C15" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">اطلب من برقر نورا🍔 واستخدم كود barq والتوصيل بـ 9 ريال بس⚡</x:t>
+          <x:t xml:space="preserve">إجازة وودك ببحر؟ 🌊 احجز في SLS البحر الأحمر واستمتع بخصم 20% باستخدام كود BARQ⚡️</x:t>
         </x:is>
       </x:c>
       <x:c r="D15" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">اطلب من برقر نورا🍔 واستخدم كود barq والتوصيل بـ 9 ريال بس⚡ — barq | برق (@barq) Aug 11, 2026</x:t>
+          <x:t xml:space="preserve">إجازة وودك ببحر؟ 🌊 احجز في SLS البحر الأحمر واستمتع بخصم 20% باستخدام كود BARQ⚡️ — barq | برق (@barq) Aug 11, 2026</x:t>
         </x:is>
       </x:c>
       <x:c r="E15" s="5" t="n">
-        <x:v>46245.73055555556</x:v>
+        <x:v>46245.595138888886</x:v>
       </x:c>
       <x:c r="F15" s="5"/>
       <x:c r="G15" s="5"/>
@@ -9020,7 +9252,7 @@
       <x:c r="O15" s="4"/>
       <x:c r="P15" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://x.com/barq/status/2087230805584011485</x:t>
+          <x:t xml:space="preserve">https://x.com/barq/status/2087181508222046216</x:t>
         </x:is>
       </x:c>
       <x:c r="Q15" s="4"/>
@@ -9042,16 +9274,16 @@
       </x:c>
       <x:c r="C16" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">جوع آخر الليل؟ عرفنا الحل برقر نورا والتوصيل بـ 9 ريال مع كود barq🍔</x:t>
+          <x:t xml:space="preserve">إجازة وودك ببحر؟ 🧐🌊 احجز في SLS البحر الأحمر واستمتع بخصم 20% باستخدام كود BARQ⚡️</x:t>
         </x:is>
       </x:c>
       <x:c r="D16" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">جوع آخر الليل؟ عرفنا الحل برقر نورا والتوصيل بـ 9 ريال مع كود barq🍔</x:t>
+          <x:t xml:space="preserve">إجازة وودك ببحر؟ 🧐🌊 احجز في SLS البحر الأحمر واستمتع بخصم 20% باستخدام كود BARQ⚡️</x:t>
         </x:is>
       </x:c>
       <x:c r="E16" s="5" t="n">
-        <x:v>46245.76534722222</x:v>
+        <x:v>46245.59591435185</x:v>
       </x:c>
       <x:c r="F16" s="5"/>
       <x:c r="G16" s="5"/>
@@ -9072,7 +9304,7 @@
       <x:c r="P16" s="4"/>
       <x:c r="Q16" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://m.facebook.com/usebarq/posts/pfbid028UQ2B7wvC8oC292eJPyDWMYuRBbbyNq7efSrQPqz3KybGHU2WRKRdrnpzayvyZuel</x:t>
+          <x:t xml:space="preserve">https://m.facebook.com/usebarq/posts/pfbid0a1HeUX42KH4Kon9NAT5JgHjENDz3WPR3Z17FVHRgyH4etXTtEDwzwH3b89TxKSDZl</x:t>
         </x:is>
       </x:c>
       <x:c r="R16" s="4"/>
@@ -9093,16 +9325,16 @@
       </x:c>
       <x:c r="C17" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">جوع آخر الليل؟ عرفنا الحل برقر نورا والتوصيل بـ 9 ريال مع كود barq🍔</x:t>
+          <x:t xml:space="preserve">إجازة وودك ببحر؟ 🧐🌊 احجز في SLS البحر الأحمر واستمتع بخصم 20% باستخدام كود BARQ⚡️</x:t>
         </x:is>
       </x:c>
       <x:c r="D17" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">جوع آخر الليل؟ عرفنا الحل برقر نورا والتوصيل بـ 9 ريال مع كود barq🍔</x:t>
+          <x:t xml:space="preserve">إجازة وودك ببحر؟ 🧐🌊 احجز في SLS البحر الأحمر واستمتع بخصم 20% باستخدام كود BARQ⚡️</x:t>
         </x:is>
       </x:c>
       <x:c r="E17" s="5" t="n">
-        <x:v>46245.76528935185</x:v>
+        <x:v>46245.595821759256</x:v>
       </x:c>
       <x:c r="F17" s="5"/>
       <x:c r="G17" s="5"/>
@@ -9121,7 +9353,7 @@
       <x:c r="N17" s="4"/>
       <x:c r="O17" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://www.instagram.com/p/Db6N_tkNgFI</x:t>
+          <x:t xml:space="preserve">https://www.instagram.com/p/Db5yOTdtsRH</x:t>
         </x:is>
       </x:c>
       <x:c r="P17" s="4"/>
@@ -9144,16 +9376,16 @@
       </x:c>
       <x:c r="C18" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">ودك بـرقر نورا؟ 👀🍔 اطلب الحين، واستخدم كود barq وخذ التوصيل بـ 9 ريال⚡</x:t>
+          <x:t xml:space="preserve">اطلب من برقر نورا🍔 واستخدم كود barq والتوصيل بـ 9 ريال بس⚡</x:t>
         </x:is>
       </x:c>
       <x:c r="D18" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">ودك بـرقر نورا؟ 👀🍔 اطلب الحين، واستخدم كود barq وخذ التوصيل بـ 9 ريال⚡ — barq | برق (@barq) Aug 11, 2026</x:t>
+          <x:t xml:space="preserve">اطلب من برقر نورا🍔 واستخدم كود barq والتوصيل بـ 9 ريال بس⚡ — barq | برق (@barq) Aug 11, 2026</x:t>
         </x:is>
       </x:c>
       <x:c r="E18" s="5" t="n">
-        <x:v>46245.8125</x:v>
+        <x:v>46245.73055555556</x:v>
       </x:c>
       <x:c r="F18" s="5"/>
       <x:c r="G18" s="5"/>
@@ -9173,7 +9405,7 @@
       <x:c r="O18" s="4"/>
       <x:c r="P18" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://x.com/barq/status/2087260261455437884</x:t>
+          <x:t xml:space="preserve">https://x.com/barq/status/2087230805584011485</x:t>
         </x:is>
       </x:c>
       <x:c r="Q18" s="4"/>
@@ -9195,16 +9427,16 @@
       </x:c>
       <x:c r="C19" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">‏اطلب من برقر نورا🍔 ‏واستخدم كود barq والتوصيل بـ 9 ريال بس⚡</x:t>
+          <x:t xml:space="preserve">جوع آخر الليل؟ عرفنا الحل برقر نورا والتوصيل بـ 9 ريال مع كود barq🍔</x:t>
         </x:is>
       </x:c>
       <x:c r="D19" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">‏اطلب من برقر نورا🍔 ‏واستخدم كود barq والتوصيل بـ 9 ريال بس⚡</x:t>
+          <x:t xml:space="preserve">جوع آخر الليل؟ عرفنا الحل برقر نورا والتوصيل بـ 9 ريال مع كود barq🍔</x:t>
         </x:is>
       </x:c>
       <x:c r="E19" s="5" t="n">
-        <x:v>46245.73243055555</x:v>
+        <x:v>46245.76534722222</x:v>
       </x:c>
       <x:c r="F19" s="5"/>
       <x:c r="G19" s="5"/>
@@ -9225,7 +9457,7 @@
       <x:c r="P19" s="4"/>
       <x:c r="Q19" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://m.facebook.com/usebarq/posts/pfbid02ESvRFRMukL9ZEP7ojEzxdqxURPJ1qjWqCTBGV3DvaFEggbABdbcKQ3Ywo9ZtKXXql</x:t>
+          <x:t xml:space="preserve">https://m.facebook.com/usebarq/posts/pfbid028UQ2B7wvC8oC292eJPyDWMYuRBbbyNq7efSrQPqz3KybGHU2WRKRdrnpzayvyZuel</x:t>
         </x:is>
       </x:c>
       <x:c r="R19" s="4"/>
@@ -9239,10 +9471,24 @@
       <x:c r="A20" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B20" s="4"/>
-      <x:c r="C20" s="4"/>
-      <x:c r="D20" s="4"/>
-      <x:c r="E20" s="5"/>
+      <x:c r="B20" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C20" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">جوع آخر الليل؟ عرفنا الحل برقر نورا والتوصيل بـ 9 ريال مع كود barq🍔</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D20" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">جوع آخر الليل؟ عرفنا الحل برقر نورا والتوصيل بـ 9 ريال مع كود barq🍔</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E20" s="5" t="n">
+        <x:v>46245.76528935185</x:v>
+      </x:c>
       <x:c r="F20" s="5"/>
       <x:c r="G20" s="5"/>
       <x:c r="H20" s="7" t="str">
@@ -9258,7 +9504,11 @@
         <x:f t="shared" si="4"/>
       </x:c>
       <x:c r="N20" s="4"/>
-      <x:c r="O20" s="4"/>
+      <x:c r="O20" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.instagram.com/p/Db6N_tkNgFI</x:t>
+        </x:is>
+      </x:c>
       <x:c r="P20" s="4"/>
       <x:c r="Q20" s="4"/>
       <x:c r="R20" s="4"/>
@@ -9272,10 +9522,24 @@
       <x:c r="A21" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B21" s="4"/>
-      <x:c r="C21" s="4"/>
-      <x:c r="D21" s="4"/>
-      <x:c r="E21" s="5"/>
+      <x:c r="B21" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C21" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ودك بـرقر نورا؟ 👀🍔 اطلب الحين، واستخدم كود barq وخذ التوصيل بـ 9 ريال⚡</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D21" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ودك بـرقر نورا؟ 👀🍔 اطلب الحين، واستخدم كود barq وخذ التوصيل بـ 9 ريال⚡ — barq | برق (@barq) Aug 11, 2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E21" s="5" t="n">
+        <x:v>46245.8125</x:v>
+      </x:c>
       <x:c r="F21" s="5"/>
       <x:c r="G21" s="5"/>
       <x:c r="H21" s="7" t="str">
@@ -9292,7 +9556,11 @@
       </x:c>
       <x:c r="N21" s="4"/>
       <x:c r="O21" s="4"/>
-      <x:c r="P21" s="4"/>
+      <x:c r="P21" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://x.com/barq/status/2087260261455437884</x:t>
+        </x:is>
+      </x:c>
       <x:c r="Q21" s="4"/>
       <x:c r="R21" s="4"/>
       <x:c r="S21" s="4"/>
@@ -9305,10 +9573,24 @@
       <x:c r="A22" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B22" s="4"/>
-      <x:c r="C22" s="4"/>
-      <x:c r="D22" s="4"/>
-      <x:c r="E22" s="5"/>
+      <x:c r="B22" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C22" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">‏اطلب من برقر نورا🍔 ‏واستخدم كود barq والتوصيل بـ 9 ريال بس⚡</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D22" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">‏اطلب من برقر نورا🍔 ‏واستخدم كود barq والتوصيل بـ 9 ريال بس⚡</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E22" s="5" t="n">
+        <x:v>46245.73243055555</x:v>
+      </x:c>
       <x:c r="F22" s="5"/>
       <x:c r="G22" s="5"/>
       <x:c r="H22" s="7" t="str">
@@ -9326,7 +9608,11 @@
       <x:c r="N22" s="4"/>
       <x:c r="O22" s="4"/>
       <x:c r="P22" s="4"/>
-      <x:c r="Q22" s="4"/>
+      <x:c r="Q22" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://m.facebook.com/usebarq/posts/pfbid02ESvRFRMukL9ZEP7ojEzxdqxURPJ1qjWqCTBGV3DvaFEggbABdbcKQ3Ywo9ZtKXXql</x:t>
+        </x:is>
+      </x:c>
       <x:c r="R22" s="4"/>
       <x:c r="S22" s="4"/>
       <x:c r="T22" s="5"/>
@@ -10437,7 +10723,7 @@
         </x:is>
       </x:c>
       <x:c r="T10" s="5" t="n">
-        <x:v>46240.0</x:v>
+        <x:v>46246.20490914237</x:v>
       </x:c>
       <x:c r="U10" s="35" t="str">
         <x:f t="shared" si="4">IF(C10="","",IF(COUNTA(O10:R10)=0,"No direct social post verified",IF(O10&lt;&gt;"","Instagram","")&amp;IF(AND(O10&lt;&gt;"",OR(P10&lt;&gt;"",Q10&lt;&gt;"",R10&lt;&gt;"")),", ","")&amp;IF(P10&lt;&gt;"","X","")&amp;IF(AND(P10&lt;&gt;"",OR(Q10&lt;&gt;"",R10&lt;&gt;"")),", ","")&amp;IF(Q10&lt;&gt;"","Facebook","")&amp;IF(AND(Q10&lt;&gt;"",R10&lt;&gt;""),", ","")&amp;IF(R10&lt;&gt;"","TikTok","")))</x:f>
@@ -10508,7 +10794,7 @@
         </x:is>
       </x:c>
       <x:c r="T11" s="5" t="n">
-        <x:v>46240.0</x:v>
+        <x:v>46246.20490914237</x:v>
       </x:c>
       <x:c r="U11" s="35" t="str">
         <x:f t="shared" si="4">IF(C11="","",IF(COUNTA(O11:R11)=0,"No direct social post verified",IF(O11&lt;&gt;"","Instagram","")&amp;IF(AND(O11&lt;&gt;"",OR(P11&lt;&gt;"",Q11&lt;&gt;"",R11&lt;&gt;"")),", ","")&amp;IF(P11&lt;&gt;"","X","")&amp;IF(AND(P11&lt;&gt;"",OR(Q11&lt;&gt;"",R11&lt;&gt;"")),", ","")&amp;IF(Q11&lt;&gt;"","Facebook","")&amp;IF(AND(Q11&lt;&gt;"",R11&lt;&gt;""),", ","")&amp;IF(R11&lt;&gt;"","TikTok","")))</x:f>
@@ -12306,14 +12592,18 @@
           <x:t xml:space="preserve">https://www.facebook.com/Tiqmoksa/posts/your-monthly-cashback-is-heretransfer-internationally-sar-1500-or-more-every-mon/1027166950077303/</x:t>
         </x:is>
       </x:c>
-      <x:c r="R12" s="4"/>
+      <x:c r="R12" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.tiktok.com/@tiqmoksa/video/7672683243400957201</x:t>
+        </x:is>
+      </x:c>
       <x:c r="S12" s="4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Current official posts continue to promote Monthly Streak Rewards. The official post does not state a campaign end date.</x:t>
         </x:is>
       </x:c>
       <x:c r="T12" s="5" t="n">
-        <x:v>46240.0</x:v>
+        <x:v>46246.20490914237</x:v>
       </x:c>
       <x:c r="U12" s="35" t="str">
         <x:f t="shared" si="4">IF(C12="","",IF(COUNTA(O12:R12)=0,"No direct social post verified",IF(O12&lt;&gt;"","Instagram","")&amp;IF(AND(O12&lt;&gt;"",OR(P12&lt;&gt;"",Q12&lt;&gt;"",R12&lt;&gt;"")),", ","")&amp;IF(P12&lt;&gt;"","X","")&amp;IF(AND(P12&lt;&gt;"",OR(Q12&lt;&gt;"",R12&lt;&gt;"")),", ","")&amp;IF(Q12&lt;&gt;"","Facebook","")&amp;IF(AND(Q12&lt;&gt;"",R12&lt;&gt;""),", ","")&amp;IF(R12&lt;&gt;"","TikTok","")))</x:f>
@@ -12405,7 +12695,7 @@
         </x:is>
       </x:c>
       <x:c r="T13" s="5" t="n">
-        <x:v>46240.0</x:v>
+        <x:v>46246.20490914237</x:v>
       </x:c>
       <x:c r="U13" s="35" t="str">
         <x:f t="shared" si="4">IF(C13="","",IF(COUNTA(O13:R13)=0,"No direct social post verified",IF(O13&lt;&gt;"","Instagram","")&amp;IF(AND(O13&lt;&gt;"",OR(P13&lt;&gt;"",Q13&lt;&gt;"",R13&lt;&gt;"")),", ","")&amp;IF(P13&lt;&gt;"","X","")&amp;IF(AND(P13&lt;&gt;"",OR(Q13&lt;&gt;"",R13&lt;&gt;"")),", ","")&amp;IF(Q13&lt;&gt;"","Facebook","")&amp;IF(AND(Q13&lt;&gt;"",R13&lt;&gt;""),", ","")&amp;IF(R13&lt;&gt;"","TikTok","")))</x:f>
@@ -12607,16 +12897,16 @@
       </x:c>
       <x:c r="C17" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Win Up to 5X Your Transfer Amount! Transfer money to Nepal via IME for a chance to win 2X, 3X, or even 5X your transfer...</x:t>
+          <x:t xml:space="preserve">Made a Transfer? Claim Your Reward! Visit the International Transfer page, click on Remittance Rewards &amp; claim your international transfer cashback #tiqmo حوّلت؟ لا تنسى مكافأتك!…</x:t>
         </x:is>
       </x:c>
       <x:c r="D17" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Win Up to 5X Your Transfer Amount! Transfer money to Nepal via IME for a chance to win 2X, 3X, or even 5X your transfer amount. No minimum transfer amount. https://tiqmo.go.link/JXFRO</x:t>
+          <x:t xml:space="preserve">Made a Transfer? Claim Your Reward! Visit the International Transfer page, click on Remittance Rewards &amp; claim your international transfer cashback #tiqmo حوّلت؟ لا تنسى مكافأتك! روح لصفحة الحوالات الدولية, واضغط على مكافآت الحوالات واكسب كاش باك حوالتك الدولية #تكمو ♬ original sound - tiqmo</x:t>
         </x:is>
       </x:c>
       <x:c r="E17" s="5" t="n">
-        <x:v>46245.62515046296</x:v>
+        <x:v>46245.341261574074</x:v>
       </x:c>
       <x:c r="F17" s="5"/>
       <x:c r="G17" s="5"/>
@@ -12635,12 +12925,12 @@
       <x:c r="N17" s="4"/>
       <x:c r="O17" s="4"/>
       <x:c r="P17" s="4"/>
-      <x:c r="Q17" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://m.facebook.com/Tiqmoksa/posts/pfbid0Dh8Sn8yM4aaNWTF3JmFa7pDhCFv6C23GC2PVf1f2QiU1Fd9ELZFGitQFTbq3oZ8Tl</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R17" s="4"/>
+      <x:c r="Q17" s="4"/>
+      <x:c r="R17" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.tiktok.com/@tiqmoksa/video/7672683243400957201</x:t>
+        </x:is>
+      </x:c>
       <x:c r="S17" s="4"/>
       <x:c r="T17" s="5"/>
       <x:c r="U17" s="35" t="str">
@@ -12653,21 +12943,21 @@
       </x:c>
       <x:c r="B18" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
+          <x:t xml:space="preserve">Remittance</x:t>
         </x:is>
       </x:c>
       <x:c r="C18" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">هذا وقت السفر! خصم يصل إلى 15% على حجوزات الفنادق والطيران عبر تطبيق المطار باستخدام كود tiqmo</x:t>
+          <x:t xml:space="preserve">Win Up to 5X Your Transfer Amount! Transfer money to Nepal via IME for a chance to win 2X, 3X, or even 5X your transfer...</x:t>
         </x:is>
       </x:c>
       <x:c r="D18" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">هذا وقت السفر! خصم يصل إلى 15% على حجوزات الفنادق والطيران عبر تطبيق المطار باستخدام كود tiqmo — @tiqmo Aug 11, 2026</x:t>
+          <x:t xml:space="preserve">Win Up to 5X Your Transfer Amount! Transfer money to Nepal via IME for a chance to win 2X, 3X, or even 5X your transfer amount. No minimum transfer amount. https://tiqmo.go.link/JXFRO</x:t>
         </x:is>
       </x:c>
       <x:c r="E18" s="5" t="n">
-        <x:v>46245.666666666664</x:v>
+        <x:v>46245.62515046296</x:v>
       </x:c>
       <x:c r="F18" s="5"/>
       <x:c r="G18" s="5"/>
@@ -12685,12 +12975,12 @@
       </x:c>
       <x:c r="N18" s="4"/>
       <x:c r="O18" s="4"/>
-      <x:c r="P18" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://x.com/tiqmo/status/2087207654758469638</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q18" s="4"/>
+      <x:c r="P18" s="4"/>
+      <x:c r="Q18" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://m.facebook.com/Tiqmoksa/posts/pfbid0Dh8Sn8yM4aaNWTF3JmFa7pDhCFv6C23GC2PVf1f2QiU1Fd9ELZFGitQFTbq3oZ8Tl</x:t>
+        </x:is>
+      </x:c>
       <x:c r="R18" s="4"/>
       <x:c r="S18" s="4"/>
       <x:c r="T18" s="5"/>
@@ -12702,10 +12992,24 @@
       <x:c r="A19" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B19" s="4"/>
-      <x:c r="C19" s="4"/>
-      <x:c r="D19" s="4"/>
-      <x:c r="E19" s="5"/>
+      <x:c r="B19" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C19" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">هذا وقت السفر! خصم يصل إلى 15% على حجوزات الفنادق والطيران عبر تطبيق المطار باستخدام كود tiqmo</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D19" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">هذا وقت السفر! خصم يصل إلى 15% على حجوزات الفنادق والطيران عبر تطبيق المطار باستخدام كود tiqmo — @tiqmo Aug 11, 2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E19" s="5" t="n">
+        <x:v>46245.666666666664</x:v>
+      </x:c>
       <x:c r="F19" s="5"/>
       <x:c r="G19" s="5"/>
       <x:c r="H19" s="7" t="str">
@@ -12722,7 +13026,11 @@
       </x:c>
       <x:c r="N19" s="4"/>
       <x:c r="O19" s="4"/>
-      <x:c r="P19" s="4"/>
+      <x:c r="P19" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://x.com/tiqmo/status/2087207654758469638</x:t>
+        </x:is>
+      </x:c>
       <x:c r="Q19" s="4"/>
       <x:c r="R19" s="4"/>
       <x:c r="S19" s="4"/>
@@ -13857,7 +14165,7 @@
         </x:is>
       </x:c>
       <x:c r="T9" s="5" t="n">
-        <x:v>46240.0</x:v>
+        <x:v>46246.20490914237</x:v>
       </x:c>
       <x:c r="U9" s="35" t="str">
         <x:f t="shared" ref="U9:U46" si="4">IF(C9="","",IF(COUNTA(O9:R9)=0,"No direct social post verified",IF(O9&lt;&gt;"","Instagram","")&amp;IF(AND(O9&lt;&gt;"",OR(P9&lt;&gt;"",Q9&lt;&gt;"",R9&lt;&gt;"")),", ","")&amp;IF(P9&lt;&gt;"","X","")&amp;IF(AND(P9&lt;&gt;"",OR(Q9&lt;&gt;"",R9&lt;&gt;"")),", ","")&amp;IF(Q9&lt;&gt;"","Facebook","")&amp;IF(AND(Q9&lt;&gt;"",R9&lt;&gt;""),", ","")&amp;IF(R9&lt;&gt;"","TikTok","")))</x:f>
@@ -13931,7 +14239,7 @@
         </x:is>
       </x:c>
       <x:c r="T10" s="5" t="n">
-        <x:v>46240.0</x:v>
+        <x:v>46246.20490914237</x:v>
       </x:c>
       <x:c r="U10" s="35" t="str">
         <x:f t="shared" si="4">IF(C10="","",IF(COUNTA(O10:R10)=0,"No direct social post verified",IF(O10&lt;&gt;"","Instagram","")&amp;IF(AND(O10&lt;&gt;"",OR(P10&lt;&gt;"",Q10&lt;&gt;"",R10&lt;&gt;"")),", ","")&amp;IF(P10&lt;&gt;"","X","")&amp;IF(AND(P10&lt;&gt;"",OR(Q10&lt;&gt;"",R10&lt;&gt;"")),", ","")&amp;IF(Q10&lt;&gt;"","Facebook","")&amp;IF(AND(Q10&lt;&gt;"",R10&lt;&gt;""),", ","")&amp;IF(R10&lt;&gt;"","TikTok","")))</x:f>
@@ -14005,7 +14313,7 @@
         </x:is>
       </x:c>
       <x:c r="T11" s="5" t="n">
-        <x:v>46240.0</x:v>
+        <x:v>46246.20490914237</x:v>
       </x:c>
       <x:c r="U11" s="35" t="str">
         <x:f t="shared" si="4">IF(C11="","",IF(COUNTA(O11:R11)=0,"No direct social post verified",IF(O11&lt;&gt;"","Instagram","")&amp;IF(AND(O11&lt;&gt;"",OR(P11&lt;&gt;"",Q11&lt;&gt;"",R11&lt;&gt;"")),", ","")&amp;IF(P11&lt;&gt;"","X","")&amp;IF(AND(P11&lt;&gt;"",OR(Q11&lt;&gt;"",R11&lt;&gt;"")),", ","")&amp;IF(Q11&lt;&gt;"","Facebook","")&amp;IF(AND(Q11&lt;&gt;"",R11&lt;&gt;""),", ","")&amp;IF(R11&lt;&gt;"","TikTok","")))</x:f>
@@ -14079,7 +14387,7 @@
         </x:is>
       </x:c>
       <x:c r="T12" s="5" t="n">
-        <x:v>46240.0</x:v>
+        <x:v>46246.20490914237</x:v>
       </x:c>
       <x:c r="U12" s="35" t="str">
         <x:f t="shared" si="4">IF(C12="","",IF(COUNTA(O12:R12)=0,"No direct social post verified",IF(O12&lt;&gt;"","Instagram","")&amp;IF(AND(O12&lt;&gt;"",OR(P12&lt;&gt;"",Q12&lt;&gt;"",R12&lt;&gt;"")),", ","")&amp;IF(P12&lt;&gt;"","X","")&amp;IF(AND(P12&lt;&gt;"",OR(Q12&lt;&gt;"",R12&lt;&gt;"")),", ","")&amp;IF(Q12&lt;&gt;"","Facebook","")&amp;IF(AND(Q12&lt;&gt;"",R12&lt;&gt;""),", ","")&amp;IF(R12&lt;&gt;"","TikTok","")))</x:f>
@@ -14153,7 +14461,7 @@
         </x:is>
       </x:c>
       <x:c r="T13" s="5" t="n">
-        <x:v>46240.0</x:v>
+        <x:v>46246.20490914237</x:v>
       </x:c>
       <x:c r="U13" s="35" t="str">
         <x:f t="shared" si="4">IF(C13="","",IF(COUNTA(O13:R13)=0,"No direct social post verified",IF(O13&lt;&gt;"","Instagram","")&amp;IF(AND(O13&lt;&gt;"",OR(P13&lt;&gt;"",Q13&lt;&gt;"",R13&lt;&gt;"")),", ","")&amp;IF(P13&lt;&gt;"","X","")&amp;IF(AND(P13&lt;&gt;"",OR(Q13&lt;&gt;"",R13&lt;&gt;"")),", ","")&amp;IF(Q13&lt;&gt;"","Facebook","")&amp;IF(AND(Q13&lt;&gt;"",R13&lt;&gt;""),", ","")&amp;IF(R13&lt;&gt;"","TikTok","")))</x:f>
@@ -14227,7 +14535,7 @@
         </x:is>
       </x:c>
       <x:c r="T14" s="5" t="n">
-        <x:v>46240.0</x:v>
+        <x:v>46246.20490914237</x:v>
       </x:c>
       <x:c r="U14" s="35" t="str">
         <x:f t="shared" si="4">IF(C14="","",IF(COUNTA(O14:R14)=0,"No direct social post verified",IF(O14&lt;&gt;"","Instagram","")&amp;IF(AND(O14&lt;&gt;"",OR(P14&lt;&gt;"",Q14&lt;&gt;"",R14&lt;&gt;"")),", ","")&amp;IF(P14&lt;&gt;"","X","")&amp;IF(AND(P14&lt;&gt;"",OR(Q14&lt;&gt;"",R14&lt;&gt;"")),", ","")&amp;IF(Q14&lt;&gt;"","Facebook","")&amp;IF(AND(Q14&lt;&gt;"",R14&lt;&gt;""),", ","")&amp;IF(R14&lt;&gt;"","TikTok","")))</x:f>
@@ -14328,7 +14636,9 @@
           <x:t xml:space="preserve">Transfer a domestic worker's salary through Musaned in urpay and enter a draw to win a travel ticket for the worker to their home country.</x:t>
         </x:is>
       </x:c>
-      <x:c r="E16" s="5"/>
+      <x:c r="E16" s="5" t="n">
+        <x:v>46210.0</x:v>
+      </x:c>
       <x:c r="F16" s="5"/>
       <x:c r="G16" s="5"/>
       <x:c r="H16" s="7" t="str">
@@ -14372,7 +14682,7 @@
         </x:is>
       </x:c>
       <x:c r="T16" s="5" t="n">
-        <x:v>46240.0</x:v>
+        <x:v>46246.20490914237</x:v>
       </x:c>
       <x:c r="U16" s="35" t="str">
         <x:f t="shared" si="4">IF(C16="","",IF(COUNTA(O16:R16)=0,"No direct social post verified",IF(O16&lt;&gt;"","Instagram","")&amp;IF(AND(O16&lt;&gt;"",OR(P16&lt;&gt;"",Q16&lt;&gt;"",R16&lt;&gt;"")),", ","")&amp;IF(P16&lt;&gt;"","X","")&amp;IF(AND(P16&lt;&gt;"",OR(Q16&lt;&gt;"",R16&lt;&gt;"")),", ","")&amp;IF(Q16&lt;&gt;"","Facebook","")&amp;IF(AND(Q16&lt;&gt;"",R16&lt;&gt;""),", ","")&amp;IF(R16&lt;&gt;"","TikTok","")))</x:f>
@@ -14430,10 +14740,14 @@
       </x:c>
       <x:c r="N17" s="124"/>
       <x:c r="O17" s="124"/>
-      <x:c r="P17" s="124"/>
+      <x:c r="P17" s="124" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://x.com/urpay_sa/status/2087192314116731265</x:t>
+        </x:is>
+      </x:c>
       <x:c r="Q17" s="124" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://www.facebook.com/urpay.sa/posts/scratch-win-with-every-international-transfer-via-urpay-and-you-could-win-up-to-/1079237764323076/</x:t>
+          <x:t xml:space="preserve">https://m.facebook.com/urpay.sa/posts/pfbid02g4cfVH8qSs9qiyHLc7vDEsppyS2kcdawe9EoXixtrxnBmQqv7wCCWWy3zMYCScGDl</x:t>
         </x:is>
       </x:c>
       <x:c r="R17" s="124"/>
@@ -14443,7 +14757,7 @@
         </x:is>
       </x:c>
       <x:c r="T17" s="125" t="n">
-        <x:v>46240.0</x:v>
+        <x:v>46246.20490914237</x:v>
       </x:c>
       <x:c r="U17" s="127" t="str">
         <x:f t="shared" si="4">IF(C17="","",IF(COUNTA(O17:R17)=0,"No direct social post verified",IF(O17&lt;&gt;"","Instagram","")&amp;IF(AND(O17&lt;&gt;"",OR(P17&lt;&gt;"",Q17&lt;&gt;"",R17&lt;&gt;"")),", ","")&amp;IF(P17&lt;&gt;"","X","")&amp;IF(AND(P17&lt;&gt;"",OR(Q17&lt;&gt;"",R17&lt;&gt;"")),", ","")&amp;IF(Q17&lt;&gt;"","Facebook","")&amp;IF(AND(Q17&lt;&gt;"",R17&lt;&gt;""),", ","")&amp;IF(R17&lt;&gt;"","TikTok","")))</x:f>
@@ -14454,10 +14768,24 @@
       <x:c r="A18" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B18" s="4"/>
-      <x:c r="C18" s="4"/>
-      <x:c r="D18" s="4"/>
-      <x:c r="E18" s="5"/>
+      <x:c r="B18" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Remittance</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C18" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Why just watch while everyone else is winning? 🤔 With urpay, absolutely everyone is a winner! All you have to do is mak...</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D18" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Why just watch while everyone else is winning? 🤔 With urpay, absolutely everyone is a winner! All you have to do is make an international transfer, and leave the amazing prizes to us 😉💙</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E18" s="5" t="n">
+        <x:v>46245.625</x:v>
+      </x:c>
       <x:c r="F18" s="5"/>
       <x:c r="G18" s="5"/>
       <x:c r="H18" s="7" t="str">
@@ -14475,7 +14803,11 @@
       <x:c r="N18" s="4"/>
       <x:c r="O18" s="4"/>
       <x:c r="P18" s="4"/>
-      <x:c r="Q18" s="4"/>
+      <x:c r="Q18" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://m.facebook.com/urpay.sa/posts/pfbid02g4cfVH8qSs9qiyHLc7vDEsppyS2kcdawe9EoXixtrxnBmQqv7wCCWWy3zMYCScGDl</x:t>
+        </x:is>
+      </x:c>
       <x:c r="R18" s="4"/>
       <x:c r="S18" s="4"/>
       <x:c r="T18" s="5"/>
@@ -14487,10 +14819,24 @@
       <x:c r="A19" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B19" s="4"/>
-      <x:c r="C19" s="4"/>
-      <x:c r="D19" s="4"/>
-      <x:c r="E19" s="5"/>
+      <x:c r="B19" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Remittance</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C19" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ليش واقف تتفرج والكل قاعد يربح؟ 🤔 مع urpay، الكل فايز بلا استثناء كل اللي عليك تحوّلها دولياً وازهل الجوائز اللي بتعجبك 😉💙</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D19" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ليش واقف تتفرج والكل قاعد يربح؟ 🤔 مع urpay، الكل فايز بلا استثناء كل اللي عليك تحوّلها دولياً وازهل الجوائز اللي بتعجبك 😉💙 — urpay المحفظة الرقمية (@urpay_sa) Aug 11, 2026</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E19" s="5" t="n">
+        <x:v>46245.625</x:v>
+      </x:c>
       <x:c r="F19" s="5"/>
       <x:c r="G19" s="5"/>
       <x:c r="H19" s="7" t="str">
@@ -14507,7 +14853,11 @@
       </x:c>
       <x:c r="N19" s="4"/>
       <x:c r="O19" s="4"/>
-      <x:c r="P19" s="4"/>
+      <x:c r="P19" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://x.com/urpay_sa/status/2087192314116731265</x:t>
+        </x:is>
+      </x:c>
       <x:c r="Q19" s="4"/>
       <x:c r="R19" s="4"/>
       <x:c r="S19" s="4"/>

</xml_diff>

<commit_message>
chore: refresh competitor intelligence
</commit_message>
<xml_diff>
--- a/competitor_campaigns_latest.xlsx
+++ b/competitor_campaigns_latest.xlsx
@@ -6100,7 +6100,7 @@
         </x:is>
       </x:c>
       <x:c r="T11" s="5" t="n">
-        <x:v>46246.222289934245</x:v>
+        <x:v>46240.0</x:v>
       </x:c>
       <x:c r="U11" s="35" t="str">
         <x:f t="shared" si="3">IF(C11="","",IF(COUNTA(O11:R11)=0,"No direct social post verified",IF(O11&lt;&gt;"","Instagram","")&amp;IF(AND(O11&lt;&gt;"",OR(P11&lt;&gt;"",Q11&lt;&gt;"",R11&lt;&gt;"")),", ","")&amp;IF(P11&lt;&gt;"","X","")&amp;IF(AND(P11&lt;&gt;"",OR(Q11&lt;&gt;"",R11&lt;&gt;"")),", ","")&amp;IF(Q11&lt;&gt;"","Facebook","")&amp;IF(AND(Q11&lt;&gt;"",R11&lt;&gt;""),", ","")&amp;IF(R11&lt;&gt;"","TikTok","")))</x:f>
@@ -6189,7 +6189,7 @@
         </x:is>
       </x:c>
       <x:c r="T12" s="5" t="n">
-        <x:v>46246.93301310684</x:v>
+        <x:v>46247.278401680414</x:v>
       </x:c>
       <x:c r="U12" s="35" t="str">
         <x:f t="shared" si="3">IF(C12="","",IF(COUNTA(O12:R12)=0,"No direct social post verified",IF(O12&lt;&gt;"","Instagram","")&amp;IF(AND(O12&lt;&gt;"",OR(P12&lt;&gt;"",Q12&lt;&gt;"",R12&lt;&gt;"")),", ","")&amp;IF(P12&lt;&gt;"","X","")&amp;IF(AND(P12&lt;&gt;"",OR(Q12&lt;&gt;"",R12&lt;&gt;"")),", ","")&amp;IF(Q12&lt;&gt;"","Facebook","")&amp;IF(AND(Q12&lt;&gt;"",R12&lt;&gt;""),", ","")&amp;IF(R12&lt;&gt;"","TikTok","")))</x:f>
@@ -6413,7 +6413,7 @@
         </x:is>
       </x:c>
       <x:c r="T15" s="5" t="n">
-        <x:v>46246.93301310684</x:v>
+        <x:v>46247.278401680414</x:v>
       </x:c>
       <x:c r="U15" s="35" t="str">
         <x:f t="shared" si="3">IF(C15="","",IF(COUNTA(O15:R15)=0,"No direct social post verified",IF(O15&lt;&gt;"","Instagram","")&amp;IF(AND(O15&lt;&gt;"",OR(P15&lt;&gt;"",Q15&lt;&gt;"",R15&lt;&gt;"")),", ","")&amp;IF(P15&lt;&gt;"","X","")&amp;IF(AND(P15&lt;&gt;"",OR(Q15&lt;&gt;"",R15&lt;&gt;"")),", ","")&amp;IF(Q15&lt;&gt;"","Facebook","")&amp;IF(AND(Q15&lt;&gt;"",R15&lt;&gt;""),", ","")&amp;IF(R15&lt;&gt;"","TikTok","")))</x:f>
@@ -6487,7 +6487,7 @@
         </x:is>
       </x:c>
       <x:c r="T16" s="5" t="n">
-        <x:v>46246.93301310684</x:v>
+        <x:v>46247.278401680414</x:v>
       </x:c>
       <x:c r="U16" s="35" t="str">
         <x:f t="shared" si="3">IF(C16="","",IF(COUNTA(O16:R16)=0,"No direct social post verified",IF(O16&lt;&gt;"","Instagram","")&amp;IF(AND(O16&lt;&gt;"",OR(P16&lt;&gt;"",Q16&lt;&gt;"",R16&lt;&gt;"")),", ","")&amp;IF(P16&lt;&gt;"","X","")&amp;IF(AND(P16&lt;&gt;"",OR(Q16&lt;&gt;"",R16&lt;&gt;"")),", ","")&amp;IF(Q16&lt;&gt;"","Facebook","")&amp;IF(AND(Q16&lt;&gt;"",R16&lt;&gt;""),", ","")&amp;IF(R16&lt;&gt;"","TikTok","")))</x:f>
@@ -6561,7 +6561,7 @@
         </x:is>
       </x:c>
       <x:c r="T17" s="5" t="n">
-        <x:v>46246.93301310684</x:v>
+        <x:v>46247.278401680414</x:v>
       </x:c>
       <x:c r="U17" s="35" t="str">
         <x:f t="shared" si="3">IF(C17="","",IF(COUNTA(O17:R17)=0,"No direct social post verified",IF(O17&lt;&gt;"","Instagram","")&amp;IF(AND(O17&lt;&gt;"",OR(P17&lt;&gt;"",Q17&lt;&gt;"",R17&lt;&gt;"")),", ","")&amp;IF(P17&lt;&gt;"","X","")&amp;IF(AND(P17&lt;&gt;"",OR(Q17&lt;&gt;"",R17&lt;&gt;"")),", ","")&amp;IF(Q17&lt;&gt;"","Facebook","")&amp;IF(AND(Q17&lt;&gt;"",R17&lt;&gt;""),", ","")&amp;IF(R17&lt;&gt;"","TikTok","")))</x:f>
@@ -6635,7 +6635,7 @@
         </x:is>
       </x:c>
       <x:c r="T18" s="5" t="n">
-        <x:v>46246.93301310684</x:v>
+        <x:v>46247.278401680414</x:v>
       </x:c>
       <x:c r="U18" s="35" t="str">
         <x:f t="shared" si="3">IF(C18="","",IF(COUNTA(O18:R18)=0,"No direct social post verified",IF(O18&lt;&gt;"","Instagram","")&amp;IF(AND(O18&lt;&gt;"",OR(P18&lt;&gt;"",Q18&lt;&gt;"",R18&lt;&gt;"")),", ","")&amp;IF(P18&lt;&gt;"","X","")&amp;IF(AND(P18&lt;&gt;"",OR(Q18&lt;&gt;"",R18&lt;&gt;"")),", ","")&amp;IF(Q18&lt;&gt;"","Facebook","")&amp;IF(AND(Q18&lt;&gt;"",R18&lt;&gt;""),", ","")&amp;IF(R18&lt;&gt;"","TikTok","")))</x:f>
@@ -6709,7 +6709,7 @@
         </x:is>
       </x:c>
       <x:c r="T19" s="5" t="n">
-        <x:v>46246.93301310684</x:v>
+        <x:v>46247.278401680414</x:v>
       </x:c>
       <x:c r="U19" s="35" t="str">
         <x:f t="shared" si="3">IF(C19="","",IF(COUNTA(O19:R19)=0,"No direct social post verified",IF(O19&lt;&gt;"","Instagram","")&amp;IF(AND(O19&lt;&gt;"",OR(P19&lt;&gt;"",Q19&lt;&gt;"",R19&lt;&gt;"")),", ","")&amp;IF(P19&lt;&gt;"","X","")&amp;IF(AND(P19&lt;&gt;"",OR(Q19&lt;&gt;"",R19&lt;&gt;"")),", ","")&amp;IF(Q19&lt;&gt;"","Facebook","")&amp;IF(AND(Q19&lt;&gt;"",R19&lt;&gt;""),", ","")&amp;IF(R19&lt;&gt;"","TikTok","")))</x:f>
@@ -6783,7 +6783,7 @@
         </x:is>
       </x:c>
       <x:c r="T20" s="5" t="n">
-        <x:v>46246.93301310684</x:v>
+        <x:v>46247.278401680414</x:v>
       </x:c>
       <x:c r="U20" s="35" t="str">
         <x:f t="shared" si="3">IF(C20="","",IF(COUNTA(O20:R20)=0,"No direct social post verified",IF(O20&lt;&gt;"","Instagram","")&amp;IF(AND(O20&lt;&gt;"",OR(P20&lt;&gt;"",Q20&lt;&gt;"",R20&lt;&gt;"")),", ","")&amp;IF(P20&lt;&gt;"","X","")&amp;IF(AND(P20&lt;&gt;"",OR(Q20&lt;&gt;"",R20&lt;&gt;"")),", ","")&amp;IF(Q20&lt;&gt;"","Facebook","")&amp;IF(AND(Q20&lt;&gt;"",R20&lt;&gt;""),", ","")&amp;IF(R20&lt;&gt;"","TikTok","")))</x:f>
@@ -6857,7 +6857,7 @@
         </x:is>
       </x:c>
       <x:c r="T21" s="5" t="n">
-        <x:v>46246.93301310684</x:v>
+        <x:v>46247.278401680414</x:v>
       </x:c>
       <x:c r="U21" s="35" t="str">
         <x:f t="shared" si="3">IF(C21="","",IF(COUNTA(O21:R21)=0,"No direct social post verified",IF(O21&lt;&gt;"","Instagram","")&amp;IF(AND(O21&lt;&gt;"",OR(P21&lt;&gt;"",Q21&lt;&gt;"",R21&lt;&gt;"")),", ","")&amp;IF(P21&lt;&gt;"","X","")&amp;IF(AND(P21&lt;&gt;"",OR(Q21&lt;&gt;"",R21&lt;&gt;"")),", ","")&amp;IF(Q21&lt;&gt;"","Facebook","")&amp;IF(AND(Q21&lt;&gt;"",R21&lt;&gt;""),", ","")&amp;IF(R21&lt;&gt;"","TikTok","")))</x:f>
@@ -8051,7 +8051,7 @@
       </x:c>
       <x:c r="N44" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/%D9%82%D9%87%D9%88%D8%AA%D9%83-%D8%A8%D9%87%D9%84%D9%84%D8%A9-%D9%85%D9%86-%D8%A8%D9%8A%D8%AA-%D8%A7%D9%84%D8%AA%D8%AD%D9%85%D9%8A%D8%B5-</x:t>
+          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/roastinghouse3</x:t>
         </x:is>
       </x:c>
       <x:c r="O44" s="4"/>
@@ -8068,21 +8068,9 @@
       <x:c r="A45" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B45" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C45" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Your coffee with 1 Halala!</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D45" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from Roasting House, in addition to 10% off all products in branches using all STC Bank cards. Valid until 2 Oct 2026 Earn cash amount on international purchases! Exclusively for selected customers, earn a cash amount on international purchases using Visa payment cards from STC Bank. Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from…</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B45" s="4"/>
+      <x:c r="C45" s="4"/>
+      <x:c r="D45" s="4"/>
       <x:c r="E45" s="5"/>
       <x:c r="F45" s="5"/>
       <x:c r="G45" s="5"/>
@@ -8098,11 +8086,7 @@
       <x:c r="M45" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N45" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/roastinghouse2</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N45" s="4"/>
       <x:c r="O45" s="4"/>
       <x:c r="P45" s="4"/>
       <x:c r="Q45" s="4"/>
@@ -8117,21 +8101,9 @@
       <x:c r="A46" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B46" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C46" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Your coffee with 1 Halala!</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D46" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from Roasting House, in addition to 10% off all products in branches using all STC Bank cards. Valid until 2 Oct 2026 Earn cash amount on international purchases! Exclusively for selected customers, earn a cash amount on international purchases using Visa payment cards from STC Bank. Valid until 13 Aug 2026 Your coffee with 1 Halala! Enjoy your cold or hot coffee day, with 1 Halala only from…</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B46" s="4"/>
+      <x:c r="C46" s="4"/>
+      <x:c r="D46" s="4"/>
       <x:c r="E46" s="5"/>
       <x:c r="F46" s="5"/>
       <x:c r="G46" s="5"/>
@@ -8147,11 +8119,7 @@
       <x:c r="M46" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N46" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/roastinghouse3</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N46" s="4"/>
       <x:c r="O46" s="4"/>
       <x:c r="P46" s="4"/>
       <x:c r="Q46" s="4"/>
@@ -8756,7 +8724,7 @@
         </x:is>
       </x:c>
       <x:c r="T9" s="5" t="n">
-        <x:v>46247.22243816139</x:v>
+        <x:v>46240.0</x:v>
       </x:c>
       <x:c r="U9" s="35" t="str">
         <x:f t="shared" ref="U9:U42" si="3">IF(C9="","",IF(COUNTA(O9:R9)=0,"No direct social post verified",IF(O9&lt;&gt;"","Instagram","")&amp;IF(AND(O9&lt;&gt;"",OR(P9&lt;&gt;"",Q9&lt;&gt;"",R9&lt;&gt;"")),", ","")&amp;IF(P9&lt;&gt;"","X","")&amp;IF(AND(P9&lt;&gt;"",OR(Q9&lt;&gt;"",R9&lt;&gt;"")),", ","")&amp;IF(Q9&lt;&gt;"","Facebook","")&amp;IF(AND(Q9&lt;&gt;"",R9&lt;&gt;""),", ","")&amp;IF(R9&lt;&gt;"","TikTok","")))</x:f>
@@ -8827,7 +8795,7 @@
         </x:is>
       </x:c>
       <x:c r="T10" s="5" t="n">
-        <x:v>46247.22243816139</x:v>
+        <x:v>46240.0</x:v>
       </x:c>
       <x:c r="U10" s="35" t="str">
         <x:f t="shared" si="3">IF(C10="","",IF(COUNTA(O10:R10)=0,"No direct social post verified",IF(O10&lt;&gt;"","Instagram","")&amp;IF(AND(O10&lt;&gt;"",OR(P10&lt;&gt;"",Q10&lt;&gt;"",R10&lt;&gt;"")),", ","")&amp;IF(P10&lt;&gt;"","X","")&amp;IF(AND(P10&lt;&gt;"",OR(Q10&lt;&gt;"",R10&lt;&gt;"")),", ","")&amp;IF(Q10&lt;&gt;"","Facebook","")&amp;IF(AND(Q10&lt;&gt;"",R10&lt;&gt;""),", ","")&amp;IF(R10&lt;&gt;"","TikTok","")))</x:f>
@@ -8898,7 +8866,7 @@
         </x:is>
       </x:c>
       <x:c r="T11" s="5" t="n">
-        <x:v>46246.93301310684</x:v>
+        <x:v>46240.0</x:v>
       </x:c>
       <x:c r="U11" s="35" t="str">
         <x:f t="shared" si="3">IF(C11="","",IF(COUNTA(O11:R11)=0,"No direct social post verified",IF(O11&lt;&gt;"","Instagram","")&amp;IF(AND(O11&lt;&gt;"",OR(P11&lt;&gt;"",Q11&lt;&gt;"",R11&lt;&gt;"")),", ","")&amp;IF(P11&lt;&gt;"","X","")&amp;IF(AND(P11&lt;&gt;"",OR(Q11&lt;&gt;"",R11&lt;&gt;"")),", ","")&amp;IF(Q11&lt;&gt;"","Facebook","")&amp;IF(AND(Q11&lt;&gt;"",R11&lt;&gt;""),", ","")&amp;IF(R11&lt;&gt;"","TikTok","")))</x:f>
@@ -8973,7 +8941,7 @@
         </x:is>
       </x:c>
       <x:c r="T12" s="5" t="n">
-        <x:v>46247.22243816139</x:v>
+        <x:v>46240.0</x:v>
       </x:c>
       <x:c r="U12" s="35" t="str">
         <x:f t="shared" si="3">IF(C12="","",IF(COUNTA(O12:R12)=0,"No direct social post verified",IF(O12&lt;&gt;"","Instagram","")&amp;IF(AND(O12&lt;&gt;"",OR(P12&lt;&gt;"",Q12&lt;&gt;"",R12&lt;&gt;"")),", ","")&amp;IF(P12&lt;&gt;"","X","")&amp;IF(AND(P12&lt;&gt;"",OR(Q12&lt;&gt;"",R12&lt;&gt;"")),", ","")&amp;IF(Q12&lt;&gt;"","Facebook","")&amp;IF(AND(Q12&lt;&gt;"",R12&lt;&gt;""),", ","")&amp;IF(R12&lt;&gt;"","TikTok","")))</x:f>
@@ -9048,7 +9016,7 @@
         </x:is>
       </x:c>
       <x:c r="T13" s="5" t="n">
-        <x:v>46247.22243816139</x:v>
+        <x:v>46240.0</x:v>
       </x:c>
       <x:c r="U13" s="35" t="str">
         <x:f t="shared" si="3">IF(C13="","",IF(COUNTA(O13:R13)=0,"No direct social post verified",IF(O13&lt;&gt;"","Instagram","")&amp;IF(AND(O13&lt;&gt;"",OR(P13&lt;&gt;"",Q13&lt;&gt;"",R13&lt;&gt;"")),", ","")&amp;IF(P13&lt;&gt;"","X","")&amp;IF(AND(P13&lt;&gt;"",OR(Q13&lt;&gt;"",R13&lt;&gt;"")),", ","")&amp;IF(Q13&lt;&gt;"","Facebook","")&amp;IF(AND(Q13&lt;&gt;"",R13&lt;&gt;""),", ","")&amp;IF(R13&lt;&gt;"","TikTok","")))</x:f>
@@ -9070,11 +9038,7 @@
           <x:t xml:space="preserve">FX Rate Awareness Campaign</x:t>
         </x:is>
       </x:c>
-      <x:c r="D14" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">‏‎85 likes, 21 comments - ‎‏‏‎usebarq‎‏ في ‏‎July 5, 2026‎‏‏: "⁨ كل دولار يفرق، والفرق يبقى معك ⚡️⁩". ‏</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="D14" s="4"/>
       <x:c r="E14" s="5"/>
       <x:c r="F14" s="5"/>
       <x:c r="G14" s="5"/>
@@ -9115,7 +9079,7 @@
       <x:c r="R14" s="4"/>
       <x:c r="S14" s="4"/>
       <x:c r="T14" s="5" t="n">
-        <x:v>46247.22243816139</x:v>
+        <x:v>46240.0</x:v>
       </x:c>
       <x:c r="U14" s="35" t="str">
         <x:f t="shared" si="3">IF(C14="","",IF(COUNTA(O14:R14)=0,"No direct social post verified",IF(O14&lt;&gt;"","Instagram","")&amp;IF(AND(O14&lt;&gt;"",OR(P14&lt;&gt;"",Q14&lt;&gt;"",R14&lt;&gt;"")),", ","")&amp;IF(P14&lt;&gt;"","X","")&amp;IF(AND(P14&lt;&gt;"",OR(Q14&lt;&gt;"",R14&lt;&gt;"")),", ","")&amp;IF(Q14&lt;&gt;"","Facebook","")&amp;IF(AND(Q14&lt;&gt;"",R14&lt;&gt;""),", ","")&amp;IF(R14&lt;&gt;"","TikTok","")))</x:f>
@@ -10473,7 +10437,7 @@
       </x:c>
       <x:c r="O10" s="63" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://www.instagram.com/p/Db2_eJcjpKO</x:t>
+          <x:t xml:space="preserve">https://www.instagram.com/reel/DZuhOEDFRNn/</x:t>
         </x:is>
       </x:c>
       <x:c r="P10" s="4" t="inlineStr">
@@ -10483,7 +10447,7 @@
       </x:c>
       <x:c r="Q10" s="63" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://m.facebook.com/mobilypay/posts/pfbid023qrERXR1VTkTXRaFcXAMT9XPQCUVgiRwbZWEgbxoQZz37XEitqK5bfLKFdWWoVaEl</x:t>
+          <x:t xml:space="preserve">https://www.facebook.com/mobilypay/videos/transfer-now/829680072943900/</x:t>
         </x:is>
       </x:c>
       <x:c r="R10" s="4"/>
@@ -10564,7 +10528,7 @@
         </x:is>
       </x:c>
       <x:c r="T11" s="5" t="n">
-        <x:v>46247.22243816139</x:v>
+        <x:v>46240.0</x:v>
       </x:c>
       <x:c r="U11" s="35" t="str">
         <x:f t="shared" si="4">IF(C11="","",IF(COUNTA(O11:R11)=0,"No direct social post verified",IF(O11&lt;&gt;"","Instagram","")&amp;IF(AND(O11&lt;&gt;"",OR(P11&lt;&gt;"",Q11&lt;&gt;"",R11&lt;&gt;"")),", ","")&amp;IF(P11&lt;&gt;"","X","")&amp;IF(AND(P11&lt;&gt;"",OR(Q11&lt;&gt;"",R11&lt;&gt;"")),", ","")&amp;IF(Q11&lt;&gt;"","Facebook","")&amp;IF(AND(Q11&lt;&gt;"",R11&lt;&gt;""),", ","")&amp;IF(R11&lt;&gt;"","TikTok","")))</x:f>
@@ -10702,7 +10666,11 @@
           <x:t xml:space="preserve">https://mobilypay.sa/offer-details.html?id=offer-53</x:t>
         </x:is>
       </x:c>
-      <x:c r="O13" s="4"/>
+      <x:c r="O13" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.instagram.com/p/DbyWZy7gV0O</x:t>
+        </x:is>
+      </x:c>
       <x:c r="P13" s="63" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://x.com/MobilyPay/status/2080699530656510080</x:t>
@@ -12112,7 +12080,7 @@
         </x:is>
       </x:c>
       <x:c r="T9" s="5" t="n">
-        <x:v>46246.222289934245</x:v>
+        <x:v>46240.0</x:v>
       </x:c>
       <x:c r="U9" s="35" t="str">
         <x:f t="shared" ref="U9:U42" si="4">IF(C9="","",IF(COUNTA(O9:R9)=0,"No direct social post verified",IF(O9&lt;&gt;"","Instagram","")&amp;IF(AND(O9&lt;&gt;"",OR(P9&lt;&gt;"",Q9&lt;&gt;"",R9&lt;&gt;"")),", ","")&amp;IF(P9&lt;&gt;"","X","")&amp;IF(AND(P9&lt;&gt;"",OR(Q9&lt;&gt;"",R9&lt;&gt;"")),", ","")&amp;IF(Q9&lt;&gt;"","Facebook","")&amp;IF(AND(Q9&lt;&gt;"",R9&lt;&gt;""),", ","")&amp;IF(R9&lt;&gt;"","TikTok","")))</x:f>
@@ -12355,7 +12323,7 @@
         </x:is>
       </x:c>
       <x:c r="T12" s="5" t="n">
-        <x:v>46247.22243816139</x:v>
+        <x:v>46240.0</x:v>
       </x:c>
       <x:c r="U12" s="35" t="str">
         <x:f t="shared" si="4">IF(C12="","",IF(COUNTA(O12:R12)=0,"No direct social post verified",IF(O12&lt;&gt;"","Instagram","")&amp;IF(AND(O12&lt;&gt;"",OR(P12&lt;&gt;"",Q12&lt;&gt;"",R12&lt;&gt;"")),", ","")&amp;IF(P12&lt;&gt;"","X","")&amp;IF(AND(P12&lt;&gt;"",OR(Q12&lt;&gt;"",R12&lt;&gt;"")),", ","")&amp;IF(Q12&lt;&gt;"","Facebook","")&amp;IF(AND(Q12&lt;&gt;"",R12&lt;&gt;""),", ","")&amp;IF(R12&lt;&gt;"","TikTok","")))</x:f>
@@ -12423,17 +12391,17 @@
       </x:c>
       <x:c r="O13" s="63" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://www.instagram.com/p/Db00V21gbnU</x:t>
+          <x:t xml:space="preserve">https://www.instagram.com/p/DbQxYrrjfrH/</x:t>
         </x:is>
       </x:c>
       <x:c r="P13" s="63" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://x.com/tiqmo/status/2086482776635895956</x:t>
+          <x:t xml:space="preserve">https://x.com/tiqmo/status/2082496811798085847</x:t>
         </x:is>
       </x:c>
       <x:c r="Q13" s="63" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://m.facebook.com/Tiqmoksa/posts/pfbid023MnKcCoq4PEqGKN5zDB9GCBJb963RNiQjMn3x1cCRajnppZHB6SgLUv8SyLpny48l</x:t>
+          <x:t xml:space="preserve">https://www.facebook.com/Tiqmoksa/posts/sar-250000-cashbacksimple-every-riyal-you-spend-a-chance-to-win-sar-250000-every/1001313055996026/</x:t>
         </x:is>
       </x:c>
       <x:c r="R13" s="63" t="inlineStr">
@@ -13857,7 +13825,7 @@
         </x:is>
       </x:c>
       <x:c r="T10" s="5" t="n">
-        <x:v>46246.93301310684</x:v>
+        <x:v>46247.278401680414</x:v>
       </x:c>
       <x:c r="U10" s="35" t="str">
         <x:f t="shared" si="4">IF(C10="","",IF(COUNTA(O10:R10)=0,"No direct social post verified",IF(O10&lt;&gt;"","Instagram","")&amp;IF(AND(O10&lt;&gt;"",OR(P10&lt;&gt;"",Q10&lt;&gt;"",R10&lt;&gt;"")),", ","")&amp;IF(P10&lt;&gt;"","X","")&amp;IF(AND(P10&lt;&gt;"",OR(Q10&lt;&gt;"",R10&lt;&gt;"")),", ","")&amp;IF(Q10&lt;&gt;"","Facebook","")&amp;IF(AND(Q10&lt;&gt;"",R10&lt;&gt;""),", ","")&amp;IF(R10&lt;&gt;"","TikTok","")))</x:f>
@@ -13931,7 +13899,7 @@
         </x:is>
       </x:c>
       <x:c r="T11" s="5" t="n">
-        <x:v>46246.93301310684</x:v>
+        <x:v>46247.278401680414</x:v>
       </x:c>
       <x:c r="U11" s="35" t="str">
         <x:f t="shared" si="4">IF(C11="","",IF(COUNTA(O11:R11)=0,"No direct social post verified",IF(O11&lt;&gt;"","Instagram","")&amp;IF(AND(O11&lt;&gt;"",OR(P11&lt;&gt;"",Q11&lt;&gt;"",R11&lt;&gt;"")),", ","")&amp;IF(P11&lt;&gt;"","X","")&amp;IF(AND(P11&lt;&gt;"",OR(Q11&lt;&gt;"",R11&lt;&gt;"")),", ","")&amp;IF(Q11&lt;&gt;"","Facebook","")&amp;IF(AND(Q11&lt;&gt;"",R11&lt;&gt;""),", ","")&amp;IF(R11&lt;&gt;"","TikTok","")))</x:f>
@@ -14005,7 +13973,7 @@
         </x:is>
       </x:c>
       <x:c r="T12" s="5" t="n">
-        <x:v>46246.93301310684</x:v>
+        <x:v>46247.278401680414</x:v>
       </x:c>
       <x:c r="U12" s="35" t="str">
         <x:f t="shared" si="4">IF(C12="","",IF(COUNTA(O12:R12)=0,"No direct social post verified",IF(O12&lt;&gt;"","Instagram","")&amp;IF(AND(O12&lt;&gt;"",OR(P12&lt;&gt;"",Q12&lt;&gt;"",R12&lt;&gt;"")),", ","")&amp;IF(P12&lt;&gt;"","X","")&amp;IF(AND(P12&lt;&gt;"",OR(Q12&lt;&gt;"",R12&lt;&gt;"")),", ","")&amp;IF(Q12&lt;&gt;"","Facebook","")&amp;IF(AND(Q12&lt;&gt;"",R12&lt;&gt;""),", ","")&amp;IF(R12&lt;&gt;"","TikTok","")))</x:f>
@@ -14079,7 +14047,7 @@
         </x:is>
       </x:c>
       <x:c r="T13" s="5" t="n">
-        <x:v>46246.20490914237</x:v>
+        <x:v>46247.278401680414</x:v>
       </x:c>
       <x:c r="U13" s="35" t="str">
         <x:f t="shared" si="4">IF(C13="","",IF(COUNTA(O13:R13)=0,"No direct social post verified",IF(O13&lt;&gt;"","Instagram","")&amp;IF(AND(O13&lt;&gt;"",OR(P13&lt;&gt;"",Q13&lt;&gt;"",R13&lt;&gt;"")),", ","")&amp;IF(P13&lt;&gt;"","X","")&amp;IF(AND(P13&lt;&gt;"",OR(Q13&lt;&gt;"",R13&lt;&gt;"")),", ","")&amp;IF(Q13&lt;&gt;"","Facebook","")&amp;IF(AND(Q13&lt;&gt;"",R13&lt;&gt;""),", ","")&amp;IF(R13&lt;&gt;"","TikTok","")))</x:f>
@@ -14153,7 +14121,7 @@
         </x:is>
       </x:c>
       <x:c r="T14" s="5" t="n">
-        <x:v>46246.20490914237</x:v>
+        <x:v>46247.278401680414</x:v>
       </x:c>
       <x:c r="U14" s="35" t="str">
         <x:f t="shared" si="4">IF(C14="","",IF(COUNTA(O14:R14)=0,"No direct social post verified",IF(O14&lt;&gt;"","Instagram","")&amp;IF(AND(O14&lt;&gt;"",OR(P14&lt;&gt;"",Q14&lt;&gt;"",R14&lt;&gt;"")),", ","")&amp;IF(P14&lt;&gt;"","X","")&amp;IF(AND(P14&lt;&gt;"",OR(Q14&lt;&gt;"",R14&lt;&gt;"")),", ","")&amp;IF(Q14&lt;&gt;"","Facebook","")&amp;IF(AND(Q14&lt;&gt;"",R14&lt;&gt;""),", ","")&amp;IF(R14&lt;&gt;"","TikTok","")))</x:f>
@@ -14254,9 +14222,7 @@
           <x:t xml:space="preserve">Transfer a domestic worker's salary through Musaned in urpay and enter a draw to win a travel ticket for the worker to their home country.</x:t>
         </x:is>
       </x:c>
-      <x:c r="E16" s="5" t="n">
-        <x:v>46210.0</x:v>
-      </x:c>
+      <x:c r="E16" s="5"/>
       <x:c r="F16" s="5"/>
       <x:c r="G16" s="5"/>
       <x:c r="H16" s="7" t="str">
@@ -14300,7 +14266,7 @@
         </x:is>
       </x:c>
       <x:c r="T16" s="5" t="n">
-        <x:v>46247.22243816139</x:v>
+        <x:v>46240.0</x:v>
       </x:c>
       <x:c r="U16" s="35" t="str">
         <x:f t="shared" si="4">IF(C16="","",IF(COUNTA(O16:R16)=0,"No direct social post verified",IF(O16&lt;&gt;"","Instagram","")&amp;IF(AND(O16&lt;&gt;"",OR(P16&lt;&gt;"",Q16&lt;&gt;"",R16&lt;&gt;"")),", ","")&amp;IF(P16&lt;&gt;"","X","")&amp;IF(AND(P16&lt;&gt;"",OR(Q16&lt;&gt;"",R16&lt;&gt;"")),", ","")&amp;IF(Q16&lt;&gt;"","Facebook","")&amp;IF(AND(Q16&lt;&gt;"",R16&lt;&gt;""),", ","")&amp;IF(R16&lt;&gt;"","TikTok","")))</x:f>
@@ -14365,7 +14331,7 @@
       </x:c>
       <x:c r="Q17" s="124" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://m.facebook.com/urpay.sa/posts/pfbid02g4cfVH8qSs9qiyHLc7vDEsppyS2kcdawe9EoXixtrxnBmQqv7wCCWWy3zMYCScGDl</x:t>
+          <x:t xml:space="preserve">https://www.facebook.com/urpay.sa/posts/scratch-win-with-every-international-transfer-via-urpay-and-you-could-win-up-to-/1079237764323076/</x:t>
         </x:is>
       </x:c>
       <x:c r="R17" s="124"/>
@@ -14375,7 +14341,7 @@
         </x:is>
       </x:c>
       <x:c r="T17" s="125" t="n">
-        <x:v>46247.22243816139</x:v>
+        <x:v>46240.0</x:v>
       </x:c>
       <x:c r="U17" s="127" t="str">
         <x:f t="shared" si="4">IF(C17="","",IF(COUNTA(O17:R17)=0,"No direct social post verified",IF(O17&lt;&gt;"","Instagram","")&amp;IF(AND(O17&lt;&gt;"",OR(P17&lt;&gt;"",Q17&lt;&gt;"",R17&lt;&gt;"")),", ","")&amp;IF(P17&lt;&gt;"","X","")&amp;IF(AND(P17&lt;&gt;"",OR(Q17&lt;&gt;"",R17&lt;&gt;"")),", ","")&amp;IF(Q17&lt;&gt;"","Facebook","")&amp;IF(AND(Q17&lt;&gt;"",R17&lt;&gt;""),", ","")&amp;IF(R17&lt;&gt;"","TikTok","")))</x:f>
@@ -15711,7 +15677,7 @@
         </x:is>
       </x:c>
       <x:c r="T9" s="5" t="n">
-        <x:v>46246.93301310684</x:v>
+        <x:v>46240.0</x:v>
       </x:c>
       <x:c r="U9" s="35" t="str">
         <x:f t="shared" ref="U9:U42" si="4">IF(C9="","",IF(COUNTA(O9:R9)=0,"No direct social post verified",IF(O9&lt;&gt;"","Instagram","")&amp;IF(AND(O9&lt;&gt;"",OR(P9&lt;&gt;"",Q9&lt;&gt;"",R9&lt;&gt;"")),", ","")&amp;IF(P9&lt;&gt;"","X","")&amp;IF(AND(P9&lt;&gt;"",OR(Q9&lt;&gt;"",R9&lt;&gt;"")),", ","")&amp;IF(Q9&lt;&gt;"","Facebook","")&amp;IF(AND(Q9&lt;&gt;"",R9&lt;&gt;""),", ","")&amp;IF(R9&lt;&gt;"","TikTok","")))</x:f>
@@ -15786,7 +15752,7 @@
         </x:is>
       </x:c>
       <x:c r="T10" s="5" t="n">
-        <x:v>46246.93301310684</x:v>
+        <x:v>46240.0</x:v>
       </x:c>
       <x:c r="U10" s="35" t="str">
         <x:f t="shared" si="4">IF(C10="","",IF(COUNTA(O10:R10)=0,"No direct social post verified",IF(O10&lt;&gt;"","Instagram","")&amp;IF(AND(O10&lt;&gt;"",OR(P10&lt;&gt;"",Q10&lt;&gt;"",R10&lt;&gt;"")),", ","")&amp;IF(P10&lt;&gt;"","X","")&amp;IF(AND(P10&lt;&gt;"",OR(Q10&lt;&gt;"",R10&lt;&gt;"")),", ","")&amp;IF(Q10&lt;&gt;"","Facebook","")&amp;IF(AND(Q10&lt;&gt;"",R10&lt;&gt;""),", ","")&amp;IF(R10&lt;&gt;"","TikTok","")))</x:f>
@@ -15865,7 +15831,7 @@
         </x:is>
       </x:c>
       <x:c r="T11" s="5" t="n">
-        <x:v>46246.93301310684</x:v>
+        <x:v>46240.0</x:v>
       </x:c>
       <x:c r="U11" s="35" t="str">
         <x:f t="shared" si="4">IF(C11="","",IF(COUNTA(O11:R11)=0,"No direct social post verified",IF(O11&lt;&gt;"","Instagram","")&amp;IF(AND(O11&lt;&gt;"",OR(P11&lt;&gt;"",Q11&lt;&gt;"",R11&lt;&gt;"")),", ","")&amp;IF(P11&lt;&gt;"","X","")&amp;IF(AND(P11&lt;&gt;"",OR(Q11&lt;&gt;"",R11&lt;&gt;"")),", ","")&amp;IF(Q11&lt;&gt;"","Facebook","")&amp;IF(AND(Q11&lt;&gt;"",R11&lt;&gt;""),", ","")&amp;IF(R11&lt;&gt;"","TikTok","")))</x:f>
@@ -15938,7 +15904,7 @@
         </x:is>
       </x:c>
       <x:c r="T12" s="5" t="n">
-        <x:v>46246.222289934245</x:v>
+        <x:v>46240.0</x:v>
       </x:c>
       <x:c r="U12" s="35" t="str">
         <x:f t="shared" si="4">IF(C12="","",IF(COUNTA(O12:R12)=0,"No direct social post verified",IF(O12&lt;&gt;"","Instagram","")&amp;IF(AND(O12&lt;&gt;"",OR(P12&lt;&gt;"",Q12&lt;&gt;"",R12&lt;&gt;"")),", ","")&amp;IF(P12&lt;&gt;"","X","")&amp;IF(AND(P12&lt;&gt;"",OR(Q12&lt;&gt;"",R12&lt;&gt;"")),", ","")&amp;IF(Q12&lt;&gt;"","Facebook","")&amp;IF(AND(Q12&lt;&gt;"",R12&lt;&gt;""),", ","")&amp;IF(R12&lt;&gt;"","TikTok","")))</x:f>
@@ -16019,7 +15985,7 @@
         </x:is>
       </x:c>
       <x:c r="T13" s="5" t="n">
-        <x:v>46246.222289934245</x:v>
+        <x:v>46240.0</x:v>
       </x:c>
       <x:c r="U13" s="35" t="str">
         <x:f t="shared" si="4">IF(C13="","",IF(COUNTA(O13:R13)=0,"No direct social post verified",IF(O13&lt;&gt;"","Instagram","")&amp;IF(AND(O13&lt;&gt;"",OR(P13&lt;&gt;"",Q13&lt;&gt;"",R13&lt;&gt;"")),", ","")&amp;IF(P13&lt;&gt;"","X","")&amp;IF(AND(P13&lt;&gt;"",OR(Q13&lt;&gt;"",R13&lt;&gt;"")),", ","")&amp;IF(Q13&lt;&gt;"","Facebook","")&amp;IF(AND(Q13&lt;&gt;"",R13&lt;&gt;""),", ","")&amp;IF(R13&lt;&gt;"","TikTok","")))</x:f>
@@ -16209,7 +16175,7 @@
       </x:c>
       <x:c r="N17" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Winter---at-Urth-Caffe-offer-Dece25</x:t>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Urth-Cafe-dec25</x:t>
         </x:is>
       </x:c>
       <x:c r="O17" s="4"/>
@@ -16233,7 +16199,7 @@
       </x:c>
       <x:c r="C18" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء رائعة واحصل على خصم 15% في أيرث كافيه</x:t>
+          <x:t xml:space="preserve">استمتع بأجواء رائعة واستمتع بخصم 20% في بيف بار</x:t>
         </x:is>
       </x:c>
       <x:c r="D18" s="4" t="inlineStr">
@@ -16258,7 +16224,7 @@
       </x:c>
       <x:c r="N18" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Urth-Cafe-dec25</x:t>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Beefbar-dec25</x:t>
         </x:is>
       </x:c>
       <x:c r="O18" s="4"/>
@@ -16282,7 +16248,7 @@
       </x:c>
       <x:c r="C19" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء رائعة واستمتع بخصم 20% في بيف بار</x:t>
+          <x:t xml:space="preserve">استمتع بأجواء رائعة واستمتع بخصم 20% في روباتا</x:t>
         </x:is>
       </x:c>
       <x:c r="D19" s="4" t="inlineStr">
@@ -16307,7 +16273,7 @@
       </x:c>
       <x:c r="N19" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Beefbar-dec25</x:t>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Robata-dec25</x:t>
         </x:is>
       </x:c>
       <x:c r="O19" s="4"/>
@@ -16331,7 +16297,7 @@
       </x:c>
       <x:c r="C20" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء رائعة واستمتع بخصم 20% في روباتا</x:t>
+          <x:t xml:space="preserve">استمتع بأجواء رائعة واستمتع بخصم 20% في كريزي بيتزا</x:t>
         </x:is>
       </x:c>
       <x:c r="D20" s="4" t="inlineStr">
@@ -16356,7 +16322,7 @@
       </x:c>
       <x:c r="N20" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Robata-dec25</x:t>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Crazy-Pizza-dec25</x:t>
         </x:is>
       </x:c>
       <x:c r="O20" s="4"/>
@@ -16380,7 +16346,7 @@
       </x:c>
       <x:c r="C21" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء رائعة واستمتع بخصم 20% في كريزي بيتزا</x:t>
+          <x:t xml:space="preserve">استمتع بأجواء رائعة واستمتع بخصم 20% في كويا</x:t>
         </x:is>
       </x:c>
       <x:c r="D21" s="4" t="inlineStr">
@@ -16405,7 +16371,7 @@
       </x:c>
       <x:c r="N21" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Crazy-Pizza-dec25</x:t>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Coya-dec25</x:t>
         </x:is>
       </x:c>
       <x:c r="O21" s="4"/>
@@ -16429,7 +16395,7 @@
       </x:c>
       <x:c r="C22" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء رائعة واستمتع بخصم 20% في كويا</x:t>
+          <x:t xml:space="preserve">استمتع بأجواء واستمتع بخصم 20% رائعة في سان كارلو شيكيتي</x:t>
         </x:is>
       </x:c>
       <x:c r="D22" s="4" t="inlineStr">
@@ -16454,7 +16420,7 @@
       </x:c>
       <x:c r="N22" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Coya-dec25</x:t>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/San-Carlo-Cicchetti-dec25</x:t>
         </x:is>
       </x:c>
       <x:c r="O22" s="4"/>
@@ -16478,7 +16444,7 @@
       </x:c>
       <x:c r="C23" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء واستمتع بخصم 20% رائعة في سان كارلو شيكيتي</x:t>
+          <x:t xml:space="preserve">استمتع بأجواء واستمتع بخصم 20% رائعة في سينيور ساسي</x:t>
         </x:is>
       </x:c>
       <x:c r="D23" s="4" t="inlineStr">
@@ -16503,7 +16469,7 @@
       </x:c>
       <x:c r="N23" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/San-Carlo-Cicchetti-dec25</x:t>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Signor-Sassi-dec25</x:t>
         </x:is>
       </x:c>
       <x:c r="O23" s="4"/>
@@ -16527,7 +16493,7 @@
       </x:c>
       <x:c r="C24" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء واستمتع بخصم 20% رائعة في سينيور ساسي</x:t>
+          <x:t xml:space="preserve">استمتع بأجواء واستمتع بخصم 20% رائعة في كايزو</x:t>
         </x:is>
       </x:c>
       <x:c r="D24" s="4" t="inlineStr">
@@ -16552,7 +16518,7 @@
       </x:c>
       <x:c r="N24" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Signor-Sassi-dec25</x:t>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Kayzo-dec25</x:t>
         </x:is>
       </x:c>
       <x:c r="O24" s="4"/>
@@ -16576,7 +16542,7 @@
       </x:c>
       <x:c r="C25" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء واستمتع بخصم 20% رائعة في كايزو</x:t>
+          <x:t xml:space="preserve">استمتع بأجواء واستمتع بخصم 20% رائعة في ميازو</x:t>
         </x:is>
       </x:c>
       <x:c r="D25" s="4" t="inlineStr">
@@ -16601,7 +16567,7 @@
       </x:c>
       <x:c r="N25" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Kayzo-dec25</x:t>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/MYAZU-dec25</x:t>
         </x:is>
       </x:c>
       <x:c r="O25" s="4"/>
@@ -16625,7 +16591,7 @@
       </x:c>
       <x:c r="C26" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء واستمتع بخصم 20% رائعة في ميازو</x:t>
+          <x:t xml:space="preserve">استمتع بخصم 15% لدى المهيدب ريزدنس</x:t>
         </x:is>
       </x:c>
       <x:c r="D26" s="4" t="inlineStr">
@@ -16650,7 +16616,7 @@
       </x:c>
       <x:c r="N26" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/MYAZU-dec25</x:t>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Al-Muhaidb-Offer---Feb-2026</x:t>
         </x:is>
       </x:c>
       <x:c r="O26" s="4"/>
@@ -16674,7 +16640,7 @@
       </x:c>
       <x:c r="C27" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">استمتع بخصم 15% لدى المهيدب ريزدنس</x:t>
+          <x:t xml:space="preserve">استمتع بخصم 15% لدى فنادق إيواء</x:t>
         </x:is>
       </x:c>
       <x:c r="D27" s="4" t="inlineStr">
@@ -16699,7 +16665,7 @@
       </x:c>
       <x:c r="N27" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Al-Muhaidb-Offer---Feb-2026</x:t>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/EWAA-Hotels-Offer---Feb-2026</x:t>
         </x:is>
       </x:c>
       <x:c r="O27" s="4"/>
@@ -16723,7 +16689,7 @@
       </x:c>
       <x:c r="C28" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">استمتع بخصم 15% لدى فنادق إيواء</x:t>
+          <x:t xml:space="preserve">استمتع بخصم 15% لدى فنادق جراند بلازا</x:t>
         </x:is>
       </x:c>
       <x:c r="D28" s="4" t="inlineStr">
@@ -16748,7 +16714,7 @@
       </x:c>
       <x:c r="N28" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/EWAA-Hotels-Offer---Feb-2026</x:t>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Grand-Plaza-Hotels---Feb-2026</x:t>
         </x:is>
       </x:c>
       <x:c r="O28" s="4"/>
@@ -16772,7 +16738,7 @@
       </x:c>
       <x:c r="C29" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">استمتع بخصم 15% لدى فنادق جراند بلازا</x:t>
+          <x:t xml:space="preserve">استمتع بخصم 30% لدى ستايلي</x:t>
         </x:is>
       </x:c>
       <x:c r="D29" s="4" t="inlineStr">
@@ -16797,7 +16763,7 @@
       </x:c>
       <x:c r="N29" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Grand-Plaza-Hotels---Feb-2026</x:t>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Stily-Offer---Feb-2026</x:t>
         </x:is>
       </x:c>
       <x:c r="O29" s="4"/>
@@ -16821,7 +16787,7 @@
       </x:c>
       <x:c r="C30" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">استمتع بخصم 30% لدى ستايلي</x:t>
+          <x:t xml:space="preserve">خصم 20% لدى سيار</x:t>
         </x:is>
       </x:c>
       <x:c r="D30" s="4" t="inlineStr">
@@ -16846,7 +16812,7 @@
       </x:c>
       <x:c r="N30" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Stily-Offer---Feb-2026</x:t>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Sayyar---April2026</x:t>
         </x:is>
       </x:c>
       <x:c r="O30" s="4"/>
@@ -16870,7 +16836,7 @@
       </x:c>
       <x:c r="C31" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">خصم 20% لدى سيار</x:t>
+          <x:t xml:space="preserve">عرض نون</x:t>
         </x:is>
       </x:c>
       <x:c r="D31" s="4" t="inlineStr">
@@ -16895,7 +16861,7 @@
       </x:c>
       <x:c r="N31" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Sayyar---April2026</x:t>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Noon-Aug-Offer</x:t>
         </x:is>
       </x:c>
       <x:c r="O31" s="4"/>
@@ -16912,21 +16878,9 @@
       <x:c r="A32" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B32" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C32" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">عرض نون</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D32" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء رائعة واحصل على خصم 15% في أيرث كافيه حتى نوفمبر 20, 2026 استمتع بأجواء واستمتع بخصم 20% رائعة في كايزو حتى نوفمبر 20, 2026 استمتع بأجواء رائعة بخصم 20% في سان كارلو شيكيتي حتى نوفمبر 20, 2026 استمتع بأجواء رائعة بخصم 20% في بيف بار حتى نوفمبر 20, 2026 خصم 20% لدى سيار حتى ديسمبر 31, 2026 استمتع بأجواء رائعة واستمتع بخصم 20% في كريزي بيتزا حتى نوفمبر 20, 2026 استمتع بأجواء رائعة واستمتع بخصم 20% في روباتا حتى نوفمبر 20, 2026 استمتع بأجواء واستمتع بخصم 20% رائعة في ميازو حتى نوفمبر…</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B32" s="4"/>
+      <x:c r="C32" s="4"/>
+      <x:c r="D32" s="4"/>
       <x:c r="E32" s="5"/>
       <x:c r="F32" s="5"/>
       <x:c r="G32" s="5"/>
@@ -16942,11 +16896,7 @@
       <x:c r="M32" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N32" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Noon-Aug-Offer</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N32" s="4"/>
       <x:c r="O32" s="4"/>
       <x:c r="P32" s="4"/>
       <x:c r="Q32" s="4"/>

</xml_diff>

<commit_message>
chore: refresh competitor intelligence (all)
</commit_message>
<xml_diff>
--- a/competitor_campaigns_latest.xlsx
+++ b/competitor_campaigns_latest.xlsx
@@ -8325,7 +8325,9 @@
         </x:is>
       </x:c>
       <x:c r="E9" s="5"/>
-      <x:c r="F9" s="5"/>
+      <x:c r="F9" s="5" t="n">
+        <x:v>46166.0</x:v>
+      </x:c>
       <x:c r="G9" s="5"/>
       <x:c r="H9" s="7" t="str">
         <x:f t="shared" ref="H9:H42" si="1">IF(OR(C9="",G9=""),"",G9-TODAY())</x:f>
@@ -8353,7 +8355,11 @@
         <x:f>IF(C9="","",IF(N9&lt;&gt;"",N9,IF(O9&lt;&gt;"",O9,IF(P9&lt;&gt;"",P9,IF(Q9&lt;&gt;"",Q9,IF(R9&lt;&gt;"",R9,""))))))</x:f>
         <x:v>https://www.instagram.com/reel/DYxvJOWiZY5/</x:v>
       </x:c>
-      <x:c r="N9" s="4"/>
+      <x:c r="N9" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/ar/offers/%d8%ad%d9%85%d9%84%d8%a9-%d8%a7%d9%84%d8%b5%d9%8a%d9%81/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O9" s="63" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://www.instagram.com/reel/DYxvJOWiZY5/</x:t>
@@ -8742,12 +8748,28 @@
       <x:c r="A15" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B15" s="4"/>
-      <x:c r="C15" s="4"/>
-      <x:c r="D15" s="4"/>
+      <x:c r="B15" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C15" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Beefbar offer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D15" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Terms and Conditions By using this offer, you agree to the following terms and conditions.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E15" s="5"/>
-      <x:c r="F15" s="5"/>
-      <x:c r="G15" s="5"/>
+      <x:c r="F15" s="5" t="n">
+        <x:v>46054.0</x:v>
+      </x:c>
+      <x:c r="G15" s="5" t="n">
+        <x:v>46234.0</x:v>
+      </x:c>
       <x:c r="H15" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -8760,13 +8782,19 @@
       <x:c r="M15" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N15" s="4"/>
+      <x:c r="N15" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/offers/beefbar/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O15" s="4"/>
       <x:c r="P15" s="4"/>
       <x:c r="Q15" s="4"/>
       <x:c r="R15" s="4"/>
       <x:c r="S15" s="4"/>
-      <x:c r="T15" s="5"/>
+      <x:c r="T15" s="5" t="n">
+        <x:v>46260.08078116647</x:v>
+      </x:c>
       <x:c r="U15" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -8775,9 +8803,21 @@
       <x:c r="A16" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B16" s="4"/>
-      <x:c r="C16" s="4"/>
-      <x:c r="D16" s="4"/>
+      <x:c r="B16" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C16" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Boulangerie Moderne offer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D16" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Terms and Conditions Offer • 10% Discount</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E16" s="5"/>
       <x:c r="F16" s="5"/>
       <x:c r="G16" s="5"/>
@@ -8793,13 +8833,19 @@
       <x:c r="M16" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N16" s="4"/>
+      <x:c r="N16" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/offers/boulangerie-moderne/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O16" s="4"/>
       <x:c r="P16" s="4"/>
       <x:c r="Q16" s="4"/>
       <x:c r="R16" s="4"/>
       <x:c r="S16" s="4"/>
-      <x:c r="T16" s="5"/>
+      <x:c r="T16" s="5" t="n">
+        <x:v>46260.08078116647</x:v>
+      </x:c>
       <x:c r="U16" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -8808,9 +8854,21 @@
       <x:c r="A17" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B17" s="4"/>
-      <x:c r="C17" s="4"/>
-      <x:c r="D17" s="4"/>
+      <x:c r="B17" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C17" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Brunch and Cake offer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D17" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Terms and Conditions Offer • 10% Discount</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E17" s="5"/>
       <x:c r="F17" s="5"/>
       <x:c r="G17" s="5"/>
@@ -8826,13 +8884,19 @@
       <x:c r="M17" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N17" s="4"/>
+      <x:c r="N17" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/offers/brunch-and-cake/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O17" s="4"/>
       <x:c r="P17" s="4"/>
       <x:c r="Q17" s="4"/>
       <x:c r="R17" s="4"/>
       <x:c r="S17" s="4"/>
-      <x:c r="T17" s="5"/>
+      <x:c r="T17" s="5" t="n">
+        <x:v>46260.08078116647</x:v>
+      </x:c>
       <x:c r="U17" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -8841,12 +8905,28 @@
       <x:c r="A18" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B18" s="4"/>
-      <x:c r="C18" s="4"/>
-      <x:c r="D18" s="4"/>
+      <x:c r="B18" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C18" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Carrefour × barq Offer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D18" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">By using this offer, you acknowledge and agree to the following terms and conditions. To be eligible for this offer, customers must:</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E18" s="5"/>
-      <x:c r="F18" s="5"/>
-      <x:c r="G18" s="5"/>
+      <x:c r="F18" s="5" t="n">
+        <x:v>46063.0</x:v>
+      </x:c>
+      <x:c r="G18" s="5" t="n">
+        <x:v>46074.0</x:v>
+      </x:c>
       <x:c r="H18" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -8859,13 +8939,19 @@
       <x:c r="M18" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N18" s="4"/>
+      <x:c r="N18" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/offers/carrefour-x-barq/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O18" s="4"/>
       <x:c r="P18" s="4"/>
       <x:c r="Q18" s="4"/>
       <x:c r="R18" s="4"/>
       <x:c r="S18" s="4"/>
-      <x:c r="T18" s="5"/>
+      <x:c r="T18" s="5" t="n">
+        <x:v>46260.08078116647</x:v>
+      </x:c>
       <x:c r="U18" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -8874,9 +8960,21 @@
       <x:c r="A19" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B19" s="4"/>
-      <x:c r="C19" s="4"/>
-      <x:c r="D19" s="4"/>
+      <x:c r="B19" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C19" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Crazy Pizza offer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D19" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Terms and Conditions Offer • Enjoy a 20% discount at Crazy Pizza Tahlia, Oud Square, north yard and Khobar when paying with barq Visa cards.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E19" s="5"/>
       <x:c r="F19" s="5"/>
       <x:c r="G19" s="5"/>
@@ -8892,13 +8990,19 @@
       <x:c r="M19" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N19" s="4"/>
+      <x:c r="N19" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/offers/crazy-pizza/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O19" s="4"/>
       <x:c r="P19" s="4"/>
       <x:c r="Q19" s="4"/>
       <x:c r="R19" s="4"/>
       <x:c r="S19" s="4"/>
-      <x:c r="T19" s="5"/>
+      <x:c r="T19" s="5" t="n">
+        <x:v>46260.08078116647</x:v>
+      </x:c>
       <x:c r="U19" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -8907,9 +9011,21 @@
       <x:c r="A20" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B20" s="4"/>
-      <x:c r="C20" s="4"/>
-      <x:c r="D20" s="4"/>
+      <x:c r="B20" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C20" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Crimson Lounge offer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D20" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Terms and Conditions • By using this offer, you agree to the following terms and conditions.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E20" s="5"/>
       <x:c r="F20" s="5"/>
       <x:c r="G20" s="5"/>
@@ -8925,13 +9041,19 @@
       <x:c r="M20" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N20" s="4"/>
+      <x:c r="N20" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/offers/crimson-lounge/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O20" s="4"/>
       <x:c r="P20" s="4"/>
       <x:c r="Q20" s="4"/>
       <x:c r="R20" s="4"/>
       <x:c r="S20" s="4"/>
-      <x:c r="T20" s="5"/>
+      <x:c r="T20" s="5" t="n">
+        <x:v>46260.08078116647</x:v>
+      </x:c>
       <x:c r="U20" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -8940,12 +9062,28 @@
       <x:c r="A21" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B21" s="4"/>
-      <x:c r="C21" s="4"/>
-      <x:c r="D21" s="4"/>
+      <x:c r="B21" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C21" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">FARFETCH × barq عرض</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D21" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">تقدم فيزا بالشراكة مع FARFTECH عرضًا لحاملي بطاقة برق فيزا، وذلك وفق الشروط والأحكام الموضحة أدناه. بالاستفادة من العرض، يقر العميل بموافقته الكاملة على هذه الشروط. للاستفادة من العرض، يجب استيفاء الشروط التالية:</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E21" s="5"/>
-      <x:c r="F21" s="5"/>
-      <x:c r="G21" s="5"/>
+      <x:c r="F21" s="5" t="n">
+        <x:v>46128.0</x:v>
+      </x:c>
+      <x:c r="G21" s="5" t="n">
+        <x:v>46295.0</x:v>
+      </x:c>
       <x:c r="H21" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -8958,13 +9096,19 @@
       <x:c r="M21" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N21" s="4"/>
+      <x:c r="N21" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/ar/offers/farfetch-offer/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O21" s="4"/>
       <x:c r="P21" s="4"/>
       <x:c r="Q21" s="4"/>
       <x:c r="R21" s="4"/>
       <x:c r="S21" s="4"/>
-      <x:c r="T21" s="5"/>
+      <x:c r="T21" s="5" t="n">
+        <x:v>46259.875649202964</x:v>
+      </x:c>
       <x:c r="U21" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -8973,9 +9117,21 @@
       <x:c r="A22" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B22" s="4"/>
-      <x:c r="C22" s="4"/>
-      <x:c r="D22" s="4"/>
+      <x:c r="B22" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C22" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">JO Spa offer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D22" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Terms and Conditions • By using this offer, you agree to the following terms and conditions.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E22" s="5"/>
       <x:c r="F22" s="5"/>
       <x:c r="G22" s="5"/>
@@ -8991,13 +9147,19 @@
       <x:c r="M22" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N22" s="4"/>
+      <x:c r="N22" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/offers/jo-spa-offer/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O22" s="4"/>
       <x:c r="P22" s="4"/>
       <x:c r="Q22" s="4"/>
       <x:c r="R22" s="4"/>
       <x:c r="S22" s="4"/>
-      <x:c r="T22" s="5"/>
+      <x:c r="T22" s="5" t="n">
+        <x:v>46260.08078116647</x:v>
+      </x:c>
       <x:c r="U22" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -9006,9 +9168,21 @@
       <x:c r="A23" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B23" s="4"/>
-      <x:c r="C23" s="4"/>
-      <x:c r="D23" s="4"/>
+      <x:c r="B23" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C23" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Lilt Furniture offer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D23" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Terms and Conditions Offer • 15% Discount for barq cardholders</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E23" s="5"/>
       <x:c r="F23" s="5"/>
       <x:c r="G23" s="5"/>
@@ -9024,13 +9198,19 @@
       <x:c r="M23" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N23" s="4"/>
+      <x:c r="N23" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/offers/lilt-furniture/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O23" s="4"/>
       <x:c r="P23" s="4"/>
       <x:c r="Q23" s="4"/>
       <x:c r="R23" s="4"/>
       <x:c r="S23" s="4"/>
-      <x:c r="T23" s="5"/>
+      <x:c r="T23" s="5" t="n">
+        <x:v>46260.08078116647</x:v>
+      </x:c>
       <x:c r="U23" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -9039,12 +9219,28 @@
       <x:c r="A24" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B24" s="4"/>
-      <x:c r="C24" s="4"/>
-      <x:c r="D24" s="4"/>
+      <x:c r="B24" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C24" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Lucca Steakhouse offer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D24" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Terms and Conditions • By using this offer, you agree to the following terms and conditions.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E24" s="5"/>
-      <x:c r="F24" s="5"/>
-      <x:c r="G24" s="5"/>
+      <x:c r="F24" s="5" t="n">
+        <x:v>46054.0</x:v>
+      </x:c>
+      <x:c r="G24" s="5" t="n">
+        <x:v>46234.0</x:v>
+      </x:c>
       <x:c r="H24" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -9057,13 +9253,19 @@
       <x:c r="M24" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N24" s="4"/>
+      <x:c r="N24" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/offers/lucca-steakhouse/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O24" s="4"/>
       <x:c r="P24" s="4"/>
       <x:c r="Q24" s="4"/>
       <x:c r="R24" s="4"/>
       <x:c r="S24" s="4"/>
-      <x:c r="T24" s="5"/>
+      <x:c r="T24" s="5" t="n">
+        <x:v>46260.08078116647</x:v>
+      </x:c>
       <x:c r="U24" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -9072,12 +9274,28 @@
       <x:c r="A25" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B25" s="4"/>
-      <x:c r="C25" s="4"/>
-      <x:c r="D25" s="4"/>
+      <x:c r="B25" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C25" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Mazrood offer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D25" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Terms and Conditions Offer • 10% discount</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E25" s="5"/>
-      <x:c r="F25" s="5"/>
-      <x:c r="G25" s="5"/>
+      <x:c r="F25" s="5" t="n">
+        <x:v>46054.0</x:v>
+      </x:c>
+      <x:c r="G25" s="5" t="n">
+        <x:v>46234.0</x:v>
+      </x:c>
       <x:c r="H25" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -9090,13 +9308,19 @@
       <x:c r="M25" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N25" s="4"/>
+      <x:c r="N25" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/ar/offers/mazrood/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O25" s="4"/>
       <x:c r="P25" s="4"/>
       <x:c r="Q25" s="4"/>
       <x:c r="R25" s="4"/>
       <x:c r="S25" s="4"/>
-      <x:c r="T25" s="5"/>
+      <x:c r="T25" s="5" t="n">
+        <x:v>46260.08078116647</x:v>
+      </x:c>
       <x:c r="U25" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -9105,9 +9329,21 @@
       <x:c r="A26" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B26" s="4"/>
-      <x:c r="C26" s="4"/>
-      <x:c r="D26" s="4"/>
+      <x:c r="B26" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C26" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Miro Furniture offer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D26" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Terms and Conditions Offer • 15% Discount for barq cardholders</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E26" s="5"/>
       <x:c r="F26" s="5"/>
       <x:c r="G26" s="5"/>
@@ -9123,13 +9359,19 @@
       <x:c r="M26" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N26" s="4"/>
+      <x:c r="N26" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/offers/miro-furniture-offer/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O26" s="4"/>
       <x:c r="P26" s="4"/>
       <x:c r="Q26" s="4"/>
       <x:c r="R26" s="4"/>
       <x:c r="S26" s="4"/>
-      <x:c r="T26" s="5"/>
+      <x:c r="T26" s="5" t="n">
+        <x:v>46260.08078116647</x:v>
+      </x:c>
       <x:c r="U26" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -9138,12 +9380,28 @@
       <x:c r="A27" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B27" s="4"/>
-      <x:c r="C27" s="4"/>
-      <x:c r="D27" s="4"/>
+      <x:c r="B27" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C27" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Mrsool × barq Offer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D27" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">By using this offer, the customer acknowledges and agrees to the following terms and conditions. To be eligible for this offer, customers must meet the following criteria:</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E27" s="5"/>
-      <x:c r="F27" s="5"/>
-      <x:c r="G27" s="5"/>
+      <x:c r="F27" s="5" t="n">
+        <x:v>46063.0</x:v>
+      </x:c>
+      <x:c r="G27" s="5" t="n">
+        <x:v>46075.0</x:v>
+      </x:c>
       <x:c r="H27" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -9156,13 +9414,19 @@
       <x:c r="M27" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N27" s="4"/>
+      <x:c r="N27" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/offers/mrsool-x-barq-offer/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O27" s="4"/>
       <x:c r="P27" s="4"/>
       <x:c r="Q27" s="4"/>
       <x:c r="R27" s="4"/>
       <x:c r="S27" s="4"/>
-      <x:c r="T27" s="5"/>
+      <x:c r="T27" s="5" t="n">
+        <x:v>46260.08078116647</x:v>
+      </x:c>
       <x:c r="U27" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -9171,9 +9435,21 @@
       <x:c r="A28" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B28" s="4"/>
-      <x:c r="C28" s="4"/>
-      <x:c r="D28" s="4"/>
+      <x:c r="B28" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C28" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Nabataty offer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D28" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Terms and Conditions Offer • 15% Discount</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E28" s="5"/>
       <x:c r="F28" s="5"/>
       <x:c r="G28" s="5"/>
@@ -9189,13 +9465,19 @@
       <x:c r="M28" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N28" s="4"/>
+      <x:c r="N28" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/offers/nabataty-offer/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O28" s="4"/>
       <x:c r="P28" s="4"/>
       <x:c r="Q28" s="4"/>
       <x:c r="R28" s="4"/>
       <x:c r="S28" s="4"/>
-      <x:c r="T28" s="5"/>
+      <x:c r="T28" s="5" t="n">
+        <x:v>46260.08078116647</x:v>
+      </x:c>
       <x:c r="U28" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -9204,9 +9486,21 @@
       <x:c r="A29" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B29" s="4"/>
-      <x:c r="C29" s="4"/>
-      <x:c r="D29" s="4"/>
+      <x:c r="B29" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C29" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Namu offer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D29" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Terms and Conditions Offer • 15% Discount</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E29" s="5"/>
       <x:c r="F29" s="5"/>
       <x:c r="G29" s="5"/>
@@ -9222,13 +9516,19 @@
       <x:c r="M29" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N29" s="4"/>
+      <x:c r="N29" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/offers/namu-offer/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O29" s="4"/>
       <x:c r="P29" s="4"/>
       <x:c r="Q29" s="4"/>
       <x:c r="R29" s="4"/>
       <x:c r="S29" s="4"/>
-      <x:c r="T29" s="5"/>
+      <x:c r="T29" s="5" t="n">
+        <x:v>46260.08078116647</x:v>
+      </x:c>
       <x:c r="U29" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -9237,9 +9537,21 @@
       <x:c r="A30" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B30" s="4"/>
-      <x:c r="C30" s="4"/>
-      <x:c r="D30" s="4"/>
+      <x:c r="B30" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C30" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ORO OXO Café offer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D30" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Terms and Conditions Offer • 20% discount</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E30" s="5"/>
       <x:c r="F30" s="5"/>
       <x:c r="G30" s="5"/>
@@ -9255,13 +9567,19 @@
       <x:c r="M30" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N30" s="4"/>
+      <x:c r="N30" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/offers/oro-oxo-cafe-offer/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O30" s="4"/>
       <x:c r="P30" s="4"/>
       <x:c r="Q30" s="4"/>
       <x:c r="R30" s="4"/>
       <x:c r="S30" s="4"/>
-      <x:c r="T30" s="5"/>
+      <x:c r="T30" s="5" t="n">
+        <x:v>46260.08078116647</x:v>
+      </x:c>
       <x:c r="U30" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -9270,9 +9588,21 @@
       <x:c r="A31" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B31" s="4"/>
-      <x:c r="C31" s="4"/>
-      <x:c r="D31" s="4"/>
+      <x:c r="B31" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C31" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Rose Maison offer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D31" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Terms and Conditions Offer • 10% Discount</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E31" s="5"/>
       <x:c r="F31" s="5"/>
       <x:c r="G31" s="5"/>
@@ -9288,13 +9618,19 @@
       <x:c r="M31" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N31" s="4"/>
+      <x:c r="N31" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/offers/rose-maison-offer/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O31" s="4"/>
       <x:c r="P31" s="4"/>
       <x:c r="Q31" s="4"/>
       <x:c r="R31" s="4"/>
       <x:c r="S31" s="4"/>
-      <x:c r="T31" s="5"/>
+      <x:c r="T31" s="5" t="n">
+        <x:v>46260.08078116647</x:v>
+      </x:c>
       <x:c r="U31" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -9303,12 +9639,28 @@
       <x:c r="A32" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B32" s="4"/>
-      <x:c r="C32" s="4"/>
-      <x:c r="D32" s="4"/>
+      <x:c r="B32" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C32" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Urth Caffe offer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D32" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Terms and Conditions • By using this offer, you agree to the following terms and conditions.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E32" s="5"/>
-      <x:c r="F32" s="5"/>
-      <x:c r="G32" s="5"/>
+      <x:c r="F32" s="5" t="n">
+        <x:v>46054.0</x:v>
+      </x:c>
+      <x:c r="G32" s="5" t="n">
+        <x:v>46234.0</x:v>
+      </x:c>
       <x:c r="H32" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -9321,13 +9673,19 @@
       <x:c r="M32" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N32" s="4"/>
+      <x:c r="N32" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/offers/urth-caffe-offer/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O32" s="4"/>
       <x:c r="P32" s="4"/>
       <x:c r="Q32" s="4"/>
       <x:c r="R32" s="4"/>
       <x:c r="S32" s="4"/>
-      <x:c r="T32" s="5"/>
+      <x:c r="T32" s="5" t="n">
+        <x:v>46260.08078116647</x:v>
+      </x:c>
       <x:c r="U32" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -9336,12 +9694,28 @@
       <x:c r="A33" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B33" s="4"/>
-      <x:c r="C33" s="4"/>
-      <x:c r="D33" s="4"/>
+      <x:c r="B33" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C33" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">VogaCloset × برق</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D33" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">تقدم فيزا بالشراكة مع VogaCloset عرضًا لحاملي بطاقة برق فيزا، وذلك وفق الشروط والأحكام الموضحة أدناه. بالاستفادة من العرض، يقر العميل بموافقته الكاملة على هذه الشروط. للاستفادة من العرض، يجب استيفاء الشروط التالية:</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E33" s="5"/>
-      <x:c r="F33" s="5"/>
-      <x:c r="G33" s="5"/>
+      <x:c r="F33" s="5" t="n">
+        <x:v>46128.0</x:v>
+      </x:c>
+      <x:c r="G33" s="5" t="n">
+        <x:v>46295.0</x:v>
+      </x:c>
       <x:c r="H33" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -9354,13 +9728,19 @@
       <x:c r="M33" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N33" s="4"/>
+      <x:c r="N33" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/ar/offers/vogacloset-offer/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O33" s="4"/>
       <x:c r="P33" s="4"/>
       <x:c r="Q33" s="4"/>
       <x:c r="R33" s="4"/>
       <x:c r="S33" s="4"/>
-      <x:c r="T33" s="5"/>
+      <x:c r="T33" s="5" t="n">
+        <x:v>46259.875649202964</x:v>
+      </x:c>
       <x:c r="U33" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -9369,9 +9749,21 @@
       <x:c r="A34" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B34" s="4"/>
-      <x:c r="C34" s="4"/>
-      <x:c r="D34" s="4"/>
+      <x:c r="B34" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C34" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Wafi Gourmet offer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D34" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Terms and Conditions Offer • 15% Discount</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E34" s="5"/>
       <x:c r="F34" s="5"/>
       <x:c r="G34" s="5"/>
@@ -9387,13 +9779,19 @@
       <x:c r="M34" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N34" s="4"/>
+      <x:c r="N34" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/offers/wafi-gourmet/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O34" s="4"/>
       <x:c r="P34" s="4"/>
       <x:c r="Q34" s="4"/>
       <x:c r="R34" s="4"/>
       <x:c r="S34" s="4"/>
-      <x:c r="T34" s="5"/>
+      <x:c r="T34" s="5" t="n">
+        <x:v>46260.08078116647</x:v>
+      </x:c>
       <x:c r="U34" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -9402,12 +9800,28 @@
       <x:c r="A35" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B35" s="4"/>
-      <x:c r="C35" s="4"/>
-      <x:c r="D35" s="4"/>
+      <x:c r="B35" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C35" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">عرض برق × Gunaydin</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D35" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">تقدّم Gunaydin لعملاء محفظة برق خصمًا حصريًا وفق الشروط والأحكام الموضّحة أدناه. باستخدام هذا العرض، يقرّ العميل بموافقته الكاملة على هذه الشروط والأحكام. للاستفادة من العرض، يجب استيفاء الشروط التالية:</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E35" s="5"/>
-      <x:c r="F35" s="5"/>
-      <x:c r="G35" s="5"/>
+      <x:c r="F35" s="5" t="n">
+        <x:v>46204.0</x:v>
+      </x:c>
+      <x:c r="G35" s="5" t="n">
+        <x:v>46723.0</x:v>
+      </x:c>
       <x:c r="H35" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -9420,13 +9834,19 @@
       <x:c r="M35" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N35" s="4"/>
+      <x:c r="N35" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/ar/offers/%d8%b9%d8%b1%d8%b6-%d8%a8%d8%b1%d9%82-x-gunaydin/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O35" s="4"/>
       <x:c r="P35" s="4"/>
       <x:c r="Q35" s="4"/>
       <x:c r="R35" s="4"/>
       <x:c r="S35" s="4"/>
-      <x:c r="T35" s="5"/>
+      <x:c r="T35" s="5" t="n">
+        <x:v>46259.875649202964</x:v>
+      </x:c>
       <x:c r="U35" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -9435,12 +9855,28 @@
       <x:c r="A36" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B36" s="4"/>
-      <x:c r="C36" s="4"/>
-      <x:c r="D36" s="4"/>
+      <x:c r="B36" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C36" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">عرض برق × Meat Moot</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D36" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">تقدّم Meat Moot لعملاء محفظة برق خصمًا حصريًا وفق الشروط والأحكام الموضّحة أدناه. باستخدام هذا العرض، يقرّ العميل بموافقته الكاملة على هذه الشروط والأحكام. للاستفادة من العرض، يجب استيفاء الشروط التالية:</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E36" s="5"/>
-      <x:c r="F36" s="5"/>
-      <x:c r="G36" s="5"/>
+      <x:c r="F36" s="5" t="n">
+        <x:v>46204.0</x:v>
+      </x:c>
+      <x:c r="G36" s="5" t="n">
+        <x:v>46126.0</x:v>
+      </x:c>
       <x:c r="H36" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -9453,13 +9889,19 @@
       <x:c r="M36" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N36" s="4"/>
+      <x:c r="N36" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/ar/offers/%d8%b9%d8%b1%d8%b6-%d8%a8%d8%b1%d9%82-x-meat-moot/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O36" s="4"/>
       <x:c r="P36" s="4"/>
       <x:c r="Q36" s="4"/>
       <x:c r="R36" s="4"/>
       <x:c r="S36" s="4"/>
-      <x:c r="T36" s="5"/>
+      <x:c r="T36" s="5" t="n">
+        <x:v>46259.875649202964</x:v>
+      </x:c>
       <x:c r="U36" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -9468,12 +9910,28 @@
       <x:c r="A37" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B37" s="4"/>
-      <x:c r="C37" s="4"/>
-      <x:c r="D37" s="4"/>
+      <x:c r="B37" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C37" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">عرض برق × Taleed by Michael Mina Bab Samhan (Diriyah)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D37" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">تقدّم Taleed by Michael Mina Bab Samhan (Diriyah) لعملاء محفظة برق خصمًا حصريًا وفق الشروط والأحكام الموضّحة أدناه. باستخدام هذا العرض، يقرّ العميل بموافقته الكاملة على هذه الشروط والأحكام. للاستفادة من العرض، يجب استيفاء الشروط التالية:</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E37" s="5"/>
-      <x:c r="F37" s="5"/>
-      <x:c r="G37" s="5"/>
+      <x:c r="F37" s="5" t="n">
+        <x:v>46204.0</x:v>
+      </x:c>
+      <x:c r="G37" s="5" t="n">
+        <x:v>46454.0</x:v>
+      </x:c>
       <x:c r="H37" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -9486,13 +9944,19 @@
       <x:c r="M37" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N37" s="4"/>
+      <x:c r="N37" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/ar/offers/%d8%b9%d8%b1%d8%b6-%d8%a8%d8%b1%d9%82-x-taleed-by-michael-mina-bab-samhan-diriyah/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O37" s="4"/>
       <x:c r="P37" s="4"/>
       <x:c r="Q37" s="4"/>
       <x:c r="R37" s="4"/>
       <x:c r="S37" s="4"/>
-      <x:c r="T37" s="5"/>
+      <x:c r="T37" s="5" t="n">
+        <x:v>46259.875649202964</x:v>
+      </x:c>
       <x:c r="U37" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -9501,12 +9965,28 @@
       <x:c r="A38" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B38" s="4"/>
-      <x:c r="C38" s="4"/>
-      <x:c r="D38" s="4"/>
+      <x:c r="B38" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C38" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">عرض برق × محمصة الرياض</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D38" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">تقدم محفظة برق بالشراكة مع محمصة الرياض عرضًا، وذلك وفق الشروط والأحكام الموضحة أدناه. بالاستفادة من العرض، يقر العميل بموافقته الكاملة على هذه الشروط. للاستفادة من العرض، يجب استيفاء الشروط التالية:</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E38" s="5"/>
-      <x:c r="F38" s="5"/>
-      <x:c r="G38" s="5"/>
+      <x:c r="F38" s="5" t="n">
+        <x:v>46180.0</x:v>
+      </x:c>
+      <x:c r="G38" s="5" t="n">
+        <x:v>46363.0</x:v>
+      </x:c>
       <x:c r="H38" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -9519,13 +9999,19 @@
       <x:c r="M38" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N38" s="4"/>
+      <x:c r="N38" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/ar/offers/%d8%b9%d8%b1%d8%b6-%d8%a8%d8%b1%d9%82-x-%d9%85%d8%ad%d9%85%d8%b5%d8%a9-%d8%a7%d9%84%d8%b1%d9%8a%d8%a7%d8%b6/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O38" s="4"/>
       <x:c r="P38" s="4"/>
       <x:c r="Q38" s="4"/>
       <x:c r="R38" s="4"/>
       <x:c r="S38" s="4"/>
-      <x:c r="T38" s="5"/>
+      <x:c r="T38" s="5" t="n">
+        <x:v>46259.875649202964</x:v>
+      </x:c>
       <x:c r="U38" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -9534,12 +10020,28 @@
       <x:c r="A39" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B39" s="4"/>
-      <x:c r="C39" s="4"/>
-      <x:c r="D39" s="4"/>
+      <x:c r="B39" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C39" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">عرض جو سبا</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D39" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">الاتفاقية • باستخدام هذا العرض، فإنك توافق على الشروط والأحكام التالية. • من 1 فبراير 2026 حتى 31 يوليو 2026</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E39" s="5"/>
-      <x:c r="F39" s="5"/>
-      <x:c r="G39" s="5"/>
+      <x:c r="F39" s="5" t="n">
+        <x:v>46054.0</x:v>
+      </x:c>
+      <x:c r="G39" s="5" t="n">
+        <x:v>46234.0</x:v>
+      </x:c>
       <x:c r="H39" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -9552,13 +10054,19 @@
       <x:c r="M39" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N39" s="4"/>
+      <x:c r="N39" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/ar/offers/jo-spa/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O39" s="4"/>
       <x:c r="P39" s="4"/>
       <x:c r="Q39" s="4"/>
       <x:c r="R39" s="4"/>
       <x:c r="S39" s="4"/>
-      <x:c r="T39" s="5"/>
+      <x:c r="T39" s="5" t="n">
+        <x:v>46259.875649202964</x:v>
+      </x:c>
       <x:c r="U39" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -9567,12 +10075,28 @@
       <x:c r="A40" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B40" s="4"/>
-      <x:c r="C40" s="4"/>
-      <x:c r="D40" s="4"/>
+      <x:c r="B40" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C40" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">عرض درايف 7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D40" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">باستخدام هذا العرض، فإنك توافق على الشروط والأحكام التالية، ويُعد استخدام العرض موافقة صريحة من العميل بعد اطلاعه على هذه الشروط والمنشورة عبر القنوات الرسمية لتطبيق برق. للاستفادة من العرض، يجب استيفاء الشروط التالية:</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E40" s="5"/>
-      <x:c r="F40" s="5"/>
-      <x:c r="G40" s="5"/>
+      <x:c r="F40" s="5" t="n">
+        <x:v>46054.0</x:v>
+      </x:c>
+      <x:c r="G40" s="5" t="n">
+        <x:v>46269.0</x:v>
+      </x:c>
       <x:c r="H40" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -9585,13 +10109,19 @@
       <x:c r="M40" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N40" s="4"/>
+      <x:c r="N40" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/ar/offers/drive7/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O40" s="4"/>
       <x:c r="P40" s="4"/>
       <x:c r="Q40" s="4"/>
       <x:c r="R40" s="4"/>
       <x:c r="S40" s="4"/>
-      <x:c r="T40" s="5"/>
+      <x:c r="T40" s="5" t="n">
+        <x:v>46259.875649202964</x:v>
+      </x:c>
       <x:c r="U40" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -9600,12 +10130,28 @@
       <x:c r="A41" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B41" s="4"/>
-      <x:c r="C41" s="4"/>
-      <x:c r="D41" s="4"/>
+      <x:c r="B41" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C41" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">عرض شي ان × برق</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D41" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">تقدم فيزا بالشراكة مع شي ان عرضًا لحاملي بطاقة برق فيزا، وذلك وفق الشروط والأحكام الموضحة أدناه. بالاستفادة من العرض، يقر العميل بموافقته الكاملة على هذه الشروط. للاستفادة من العرض، يجب استيفاء الشروط التالية:</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E41" s="5"/>
-      <x:c r="F41" s="5"/>
-      <x:c r="G41" s="5"/>
+      <x:c r="F41" s="5" t="n">
+        <x:v>46128.0</x:v>
+      </x:c>
+      <x:c r="G41" s="5" t="n">
+        <x:v>46295.0</x:v>
+      </x:c>
       <x:c r="H41" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -9618,13 +10164,19 @@
       <x:c r="M41" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N41" s="4"/>
+      <x:c r="N41" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/ar/offers/shein-offer/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O41" s="4"/>
       <x:c r="P41" s="4"/>
       <x:c r="Q41" s="4"/>
       <x:c r="R41" s="4"/>
       <x:c r="S41" s="4"/>
-      <x:c r="T41" s="5"/>
+      <x:c r="T41" s="5" t="n">
+        <x:v>46259.875649202964</x:v>
+      </x:c>
       <x:c r="U41" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -9633,12 +10185,28 @@
       <x:c r="A42" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B42" s="4"/>
-      <x:c r="C42" s="4"/>
-      <x:c r="D42" s="4"/>
+      <x:c r="B42" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C42" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">فايف سكندز صالون</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D42" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">خصم 20% على كل الخدمات من 01/02/2026 إلى 31/12/2026</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E42" s="5"/>
-      <x:c r="F42" s="5"/>
-      <x:c r="G42" s="5"/>
+      <x:c r="F42" s="5" t="n">
+        <x:v>46054.0</x:v>
+      </x:c>
+      <x:c r="G42" s="5" t="n">
+        <x:v>46387.0</x:v>
+      </x:c>
       <x:c r="H42" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -9651,13 +10219,19 @@
       <x:c r="M42" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N42" s="4"/>
+      <x:c r="N42" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://barq.com/ar/offers/5-second-salon/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O42" s="4"/>
       <x:c r="P42" s="4"/>
       <x:c r="Q42" s="4"/>
       <x:c r="R42" s="4"/>
       <x:c r="S42" s="4"/>
-      <x:c r="T42" s="5"/>
+      <x:c r="T42" s="5" t="n">
+        <x:v>46259.958868124806</x:v>
+      </x:c>
       <x:c r="U42" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -10084,7 +10658,7 @@
       </x:c>
       <x:c r="N10" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-56.html</x:t>
+          <x:t xml:space="preserve">https://mobilypay.sa/en/offers/offer-56.html</x:t>
         </x:is>
       </x:c>
       <x:c r="O10" s="63" t="inlineStr">
@@ -10446,12 +11020,12 @@
       </x:c>
       <x:c r="C15" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">10 ريال سعودي كاش باك</x:t>
+          <x:t xml:space="preserve">10 SAR CASHBACK</x:t>
         </x:is>
       </x:c>
       <x:c r="D15" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">العرض ساري من تاريخ 5 يناير حتى 30 أغسطس 2026. شارك الكود الخاص بك مع أصدقائك واحصل على 5 ريال كاش باك وسيحصل صديقك على 5 ريال كاش باك.</x:t>
+          <x:t xml:space="preserve">The offer is valid from 5 Jan until 30 Aug 2026. Share your promo code with your friends to get SAR 5 Cashback, and them get SAR 5 Cashback.</x:t>
         </x:is>
       </x:c>
       <x:c r="E15" s="5"/>
@@ -10484,7 +11058,7 @@
       <x:c r="R15" s="4"/>
       <x:c r="S15" s="4"/>
       <x:c r="T15" s="5" t="n">
-        <x:v>46260.11321182853</x:v>
+        <x:v>46260.20266816726</x:v>
       </x:c>
       <x:c r="U15" s="35" t="str">
         <x:f t="shared" si="4"/>
@@ -10501,17 +11075,17 @@
       </x:c>
       <x:c r="C16" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">أوشن سبا</x:t>
+          <x:t xml:space="preserve">AL MABAT HOTEL</x:t>
         </x:is>
       </x:c>
       <x:c r="D16" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">يسري العرض من 20 مايو 2025 حتى 30 نوفمبر 2026. خصم 20% على جميع الخدمات بدون حد ادنى.</x:t>
+          <x:t xml:space="preserve">Offer is valid from 10 July 2025 to 30 Nov 2026. 15% discount with no limit on your full hotel experience — buffet service excluded.</x:t>
         </x:is>
       </x:c>
       <x:c r="E16" s="5"/>
       <x:c r="F16" s="5" t="n">
-        <x:v>45797.0</x:v>
+        <x:v>45848.0</x:v>
       </x:c>
       <x:c r="G16" s="5" t="n">
         <x:v>46356.0</x:v>
@@ -10530,7 +11104,7 @@
       </x:c>
       <x:c r="N16" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-10.html</x:t>
+          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-13.html</x:t>
         </x:is>
       </x:c>
       <x:c r="O16" s="4"/>
@@ -10539,7 +11113,7 @@
       <x:c r="R16" s="4"/>
       <x:c r="S16" s="4"/>
       <x:c r="T16" s="5" t="n">
-        <x:v>46260.11321182853</x:v>
+        <x:v>46260.20266816726</x:v>
       </x:c>
       <x:c r="U16" s="35" t="str">
         <x:f t="shared" si="4"/>
@@ -10551,22 +11125,22 @@
       </x:c>
       <x:c r="B17" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
+          <x:t xml:space="preserve">Other</x:t>
         </x:is>
       </x:c>
       <x:c r="C17" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">أيهيرب</x:t>
+          <x:t xml:space="preserve">EARN MILES WITH ALL MOBILY PAY SERVICES</x:t>
         </x:is>
       </x:c>
       <x:c r="D17" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">يسري العرض من 1 أبريل حتى 30 سبتمبر 2026. احصل على خصم %25 على أول طلب لك من أيهيرب، أو خصم %10 إذا كنت عميلاً حالياً.</x:t>
+          <x:t xml:space="preserve">Offer is valid from 1 Feb 2025 until 30 Sep 2026. Offer includes only the services specified in the Miles Earning Schedule when using Mobily Pay App</x:t>
         </x:is>
       </x:c>
       <x:c r="E17" s="5"/>
       <x:c r="F17" s="5" t="n">
-        <x:v>46113.0</x:v>
+        <x:v>45689.0</x:v>
       </x:c>
       <x:c r="G17" s="5" t="n">
         <x:v>46295.0</x:v>
@@ -10585,7 +11159,7 @@
       </x:c>
       <x:c r="N17" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-50.html</x:t>
+          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-7.html</x:t>
         </x:is>
       </x:c>
       <x:c r="O17" s="4"/>
@@ -10594,7 +11168,7 @@
       <x:c r="R17" s="4"/>
       <x:c r="S17" s="4"/>
       <x:c r="T17" s="5" t="n">
-        <x:v>46260.11321182853</x:v>
+        <x:v>46260.20266816726</x:v>
       </x:c>
       <x:c r="U17" s="35" t="str">
         <x:f t="shared" si="4"/>
@@ -10606,25 +11180,25 @@
       </x:c>
       <x:c r="B18" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Other</x:t>
+          <x:t xml:space="preserve">Merchant</x:t>
         </x:is>
       </x:c>
       <x:c r="C18" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">اكسب أميال مع جميع خدمات Mobily Pay</x:t>
+          <x:t xml:space="preserve">FANOS LIGHTING</x:t>
         </x:is>
       </x:c>
       <x:c r="D18" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">العرض ساري من 1 فبراير 2025 حتى 30 سبتمبر 2026. العرض يشمل الخدمات المحددة في جدول اكتساب الأميال باستخدام تطبيق Mobily Pay</x:t>
+          <x:t xml:space="preserve">Offer is valid from 22 Oct 2025 until 20 Oct 2026. 12% discount without limit on all products except establishment products.</x:t>
         </x:is>
       </x:c>
       <x:c r="E18" s="5"/>
       <x:c r="F18" s="5" t="n">
-        <x:v>45689.0</x:v>
+        <x:v>45952.0</x:v>
       </x:c>
       <x:c r="G18" s="5" t="n">
-        <x:v>46295.0</x:v>
+        <x:v>46315.0</x:v>
       </x:c>
       <x:c r="H18" s="7" t="str">
         <x:f t="shared" si="1"/>
@@ -10640,7 +11214,7 @@
       </x:c>
       <x:c r="N18" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-7.html</x:t>
+          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-19.html</x:t>
         </x:is>
       </x:c>
       <x:c r="O18" s="4"/>
@@ -10649,7 +11223,7 @@
       <x:c r="R18" s="4"/>
       <x:c r="S18" s="4"/>
       <x:c r="T18" s="5" t="n">
-        <x:v>46260.11321182853</x:v>
+        <x:v>46260.20266816726</x:v>
       </x:c>
       <x:c r="U18" s="35" t="str">
         <x:f t="shared" si="4"/>
@@ -10666,20 +11240,20 @@
       </x:c>
       <x:c r="C19" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">الحمد للحقائب</x:t>
+          <x:t xml:space="preserve">SWEATER</x:t>
         </x:is>
       </x:c>
       <x:c r="D19" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">يسري العرض من 18 يونيو 2025 حتى 30 نوفمبر 2026. خصم 10% على جميع المنتجات للفاتورة التي تبلغ قيمتها 100 ريال أو أكثر</x:t>
+          <x:t xml:space="preserve">Offer valid from 26 Oct 2025 until 30 Dec 2026 40% discount on single wash only from 9:00 AM to 2 PM when using promo code MobilyPay40</x:t>
         </x:is>
       </x:c>
       <x:c r="E19" s="5"/>
       <x:c r="F19" s="5" t="n">
-        <x:v>45826.0</x:v>
+        <x:v>45956.0</x:v>
       </x:c>
       <x:c r="G19" s="5" t="n">
-        <x:v>46356.0</x:v>
+        <x:v>46386.0</x:v>
       </x:c>
       <x:c r="H19" s="7" t="str">
         <x:f t="shared" si="1"/>
@@ -10695,7 +11269,7 @@
       </x:c>
       <x:c r="N19" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-12.html</x:t>
+          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-20.html</x:t>
         </x:is>
       </x:c>
       <x:c r="O19" s="4"/>
@@ -10704,7 +11278,7 @@
       <x:c r="R19" s="4"/>
       <x:c r="S19" s="4"/>
       <x:c r="T19" s="5" t="n">
-        <x:v>46260.11321182853</x:v>
+        <x:v>46260.20266816726</x:v>
       </x:c>
       <x:c r="U19" s="35" t="str">
         <x:f t="shared" si="4"/>
@@ -10716,25 +11290,25 @@
       </x:c>
       <x:c r="B20" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
+          <x:t xml:space="preserve">Other</x:t>
         </x:is>
       </x:c>
       <x:c r="C20" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">باقيت في مجال التغذية الصحية</x:t>
+          <x:t xml:space="preserve">Trips For hotel and flight reservations</x:t>
         </x:is>
       </x:c>
       <x:c r="D20" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">يسري العرض من 19 أبريل حتى 31 ديسمبر 2026 . خصم %35 على جميع الباقات الشهرية.</x:t>
+          <x:t xml:space="preserve">Offer is valid from 16 Aug until 31 Aug 2026. 5% discount on hotels and 5% cashback on domestic and international airlines with no maximum discount or cashback.</x:t>
         </x:is>
       </x:c>
       <x:c r="E20" s="5"/>
       <x:c r="F20" s="5" t="n">
-        <x:v>46131.0</x:v>
+        <x:v>46250.0</x:v>
       </x:c>
       <x:c r="G20" s="5" t="n">
-        <x:v>46387.0</x:v>
+        <x:v>46265.0</x:v>
       </x:c>
       <x:c r="H20" s="7" t="str">
         <x:f t="shared" si="1"/>
@@ -10750,7 +11324,7 @@
       </x:c>
       <x:c r="N20" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-41.html</x:t>
+          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-57.html</x:t>
         </x:is>
       </x:c>
       <x:c r="O20" s="4"/>
@@ -10759,7 +11333,7 @@
       <x:c r="R20" s="4"/>
       <x:c r="S20" s="4"/>
       <x:c r="T20" s="5" t="n">
-        <x:v>46260.11321182853</x:v>
+        <x:v>46260.20266816726</x:v>
       </x:c>
       <x:c r="U20" s="35" t="str">
         <x:f t="shared" si="4"/>
@@ -10776,20 +11350,20 @@
       </x:c>
       <x:c r="C21" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">بيلاتس استديو</x:t>
+          <x:t xml:space="preserve">Vogacloset</x:t>
         </x:is>
       </x:c>
       <x:c r="D21" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">يسري العرض من 6 أبريل حتى 31 ديسمبر 2026. اشترك في 10 حصص بيلاتس واحصل على حصتين يوقا مجاناً.</x:t>
+          <x:t xml:space="preserve">Offer valid from 19 April to 30 September 2026. Offer is valid on all purchases when using a Mobily Pay card (Platinum &amp; Signature) with promo code "VISA10".</x:t>
         </x:is>
       </x:c>
       <x:c r="E21" s="5"/>
       <x:c r="F21" s="5" t="n">
-        <x:v>46118.0</x:v>
+        <x:v>46131.0</x:v>
       </x:c>
       <x:c r="G21" s="5" t="n">
-        <x:v>46387.0</x:v>
+        <x:v>46295.0</x:v>
       </x:c>
       <x:c r="H21" s="7" t="str">
         <x:f t="shared" si="1"/>
@@ -10805,7 +11379,7 @@
       </x:c>
       <x:c r="N21" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-36.html</x:t>
+          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-49.html</x:t>
         </x:is>
       </x:c>
       <x:c r="O21" s="4"/>
@@ -10814,7 +11388,7 @@
       <x:c r="R21" s="4"/>
       <x:c r="S21" s="4"/>
       <x:c r="T21" s="5" t="n">
-        <x:v>46260.11321182853</x:v>
+        <x:v>46260.20266816726</x:v>
       </x:c>
       <x:c r="U21" s="35" t="str">
         <x:f t="shared" si="4"/>
@@ -10831,17 +11405,17 @@
       </x:c>
       <x:c r="C22" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">تاكوهت</x:t>
+          <x:t xml:space="preserve">أوشن سبا</x:t>
         </x:is>
       </x:c>
       <x:c r="D22" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">يسري العرض من 19 أبريل حتى 30 نوفمبر 2026. خصم 20% على جميع الطلبات بدون حد أدنى من خلال التطبيق المخصص لاستلام الطلبات.</x:t>
+          <x:t xml:space="preserve">يسري العرض من 20 مايو 2025 حتى 30 نوفمبر 2026. خصم 20% على جميع الخدمات بدون حد ادنى.</x:t>
         </x:is>
       </x:c>
       <x:c r="E22" s="5"/>
       <x:c r="F22" s="5" t="n">
-        <x:v>46131.0</x:v>
+        <x:v>45797.0</x:v>
       </x:c>
       <x:c r="G22" s="5" t="n">
         <x:v>46356.0</x:v>
@@ -10860,7 +11434,7 @@
       </x:c>
       <x:c r="N22" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-44.html</x:t>
+          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-10.html</x:t>
         </x:is>
       </x:c>
       <x:c r="O22" s="4"/>
@@ -10886,20 +11460,20 @@
       </x:c>
       <x:c r="C23" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">جيم تك</x:t>
+          <x:t xml:space="preserve">أيهيرب</x:t>
         </x:is>
       </x:c>
       <x:c r="D23" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">يسري العرض من 19 أبريل حتى 31 ديسمبر 2026. خصم 50% على جميع الباقات.</x:t>
+          <x:t xml:space="preserve">يسري العرض من 1 أبريل حتى 30 سبتمبر 2026. احصل على خصم %25 على أول طلب لك من أيهيرب، أو خصم %10 إذا كنت عميلاً حالياً.</x:t>
         </x:is>
       </x:c>
       <x:c r="E23" s="5"/>
       <x:c r="F23" s="5" t="n">
-        <x:v>46131.0</x:v>
+        <x:v>46113.0</x:v>
       </x:c>
       <x:c r="G23" s="5" t="n">
-        <x:v>46387.0</x:v>
+        <x:v>46295.0</x:v>
       </x:c>
       <x:c r="H23" s="7" t="str">
         <x:f t="shared" si="1"/>
@@ -10915,7 +11489,7 @@
       </x:c>
       <x:c r="N23" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-45.html</x:t>
+          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-50.html</x:t>
         </x:is>
       </x:c>
       <x:c r="O23" s="4"/>
@@ -10936,24 +11510,26 @@
       </x:c>
       <x:c r="B24" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Other</x:t>
+          <x:t xml:space="preserve">Merchant</x:t>
         </x:is>
       </x:c>
       <x:c r="C24" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">حوالتك الدولية إلى باكستان مجانية</x:t>
+          <x:t xml:space="preserve">الحمد للحقائب</x:t>
         </x:is>
       </x:c>
       <x:c r="D24" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">هذا العرض ساري من 8 نوفمبر 2023. التحويل الدولي إلى حساب بنكي أو محافظ رقمية في باكستان بدون رسوم.</x:t>
+          <x:t xml:space="preserve">يسري العرض من 18 يونيو 2025 حتى 30 نوفمبر 2026. خصم 10% على جميع المنتجات للفاتورة التي تبلغ قيمتها 100 ريال أو أكثر</x:t>
         </x:is>
       </x:c>
       <x:c r="E24" s="5"/>
       <x:c r="F24" s="5" t="n">
-        <x:v>45238.0</x:v>
-      </x:c>
-      <x:c r="G24" s="5"/>
+        <x:v>45826.0</x:v>
+      </x:c>
+      <x:c r="G24" s="5" t="n">
+        <x:v>46356.0</x:v>
+      </x:c>
       <x:c r="H24" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -10968,7 +11544,7 @@
       </x:c>
       <x:c r="N24" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-2.html</x:t>
+          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-12.html</x:t>
         </x:is>
       </x:c>
       <x:c r="O24" s="4"/>
@@ -10994,12 +11570,12 @@
       </x:c>
       <x:c r="C25" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">روماوَي</x:t>
+          <x:t xml:space="preserve">باقيت في مجال التغذية الصحية</x:t>
         </x:is>
       </x:c>
       <x:c r="D25" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">يسري العرض من 19 أبريل حتى 30 نوفمبر 2026 خصم 20% على جميع الطلبات بدون حد أدنى من خلال التطبيق المخصص لاستلام الطلبات.</x:t>
+          <x:t xml:space="preserve">يسري العرض من 19 أبريل حتى 31 ديسمبر 2026 . خصم %35 على جميع الباقات الشهرية.</x:t>
         </x:is>
       </x:c>
       <x:c r="E25" s="5"/>
@@ -11007,7 +11583,7 @@
         <x:v>46131.0</x:v>
       </x:c>
       <x:c r="G25" s="5" t="n">
-        <x:v>46356.0</x:v>
+        <x:v>46387.0</x:v>
       </x:c>
       <x:c r="H25" s="7" t="str">
         <x:f t="shared" si="1"/>
@@ -11023,7 +11599,7 @@
       </x:c>
       <x:c r="N25" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-42.html</x:t>
+          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-41.html</x:t>
         </x:is>
       </x:c>
       <x:c r="O25" s="4"/>
@@ -11049,20 +11625,20 @@
       </x:c>
       <x:c r="C26" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">سويتر</x:t>
+          <x:t xml:space="preserve">بيلاتس استديو</x:t>
         </x:is>
       </x:c>
       <x:c r="D26" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">يسري العرض من 26 أكتوبر 2025 حتى 30 ديسمير 2026 خصم 40٪ على الغسلة الفردية فقط من الساعة 9:00 صباحاً حتى الساعة 2 ظهراً عند استخدام الرمز الترويجي MobilyPay40</x:t>
+          <x:t xml:space="preserve">يسري العرض من 6 أبريل حتى 31 ديسمبر 2026. اشترك في 10 حصص بيلاتس واحصل على حصتين يوقا مجاناً.</x:t>
         </x:is>
       </x:c>
       <x:c r="E26" s="5"/>
       <x:c r="F26" s="5" t="n">
-        <x:v>45956.0</x:v>
+        <x:v>46118.0</x:v>
       </x:c>
       <x:c r="G26" s="5" t="n">
-        <x:v>46386.0</x:v>
+        <x:v>46387.0</x:v>
       </x:c>
       <x:c r="H26" s="7" t="str">
         <x:f t="shared" si="1"/>
@@ -11078,7 +11654,7 @@
       </x:c>
       <x:c r="N26" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-20.html</x:t>
+          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-36.html</x:t>
         </x:is>
       </x:c>
       <x:c r="O26" s="4"/>
@@ -11099,25 +11675,25 @@
       </x:c>
       <x:c r="B27" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Other</x:t>
+          <x:t xml:space="preserve">Merchant</x:t>
         </x:is>
       </x:c>
       <x:c r="C27" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">عرض تربز لحجوزات الفنادق ورحلات الطيران</x:t>
+          <x:t xml:space="preserve">تاكوهت</x:t>
         </x:is>
       </x:c>
       <x:c r="D27" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">يسري العرض من 16 أغسطس حتى 31 أغسطس 2026 خصم 5% على حجوزات الفنادق وكاش باك 5% على رحلات الطيران الداخلية والدولية بدون حد أقصى للخصم أو الكاش باك.</x:t>
+          <x:t xml:space="preserve">يسري العرض من 19 أبريل حتى 30 نوفمبر 2026. خصم 20% على جميع الطلبات بدون حد أدنى من خلال التطبيق المخصص لاستلام الطلبات.</x:t>
         </x:is>
       </x:c>
       <x:c r="E27" s="5"/>
       <x:c r="F27" s="5" t="n">
-        <x:v>46250.0</x:v>
+        <x:v>46131.0</x:v>
       </x:c>
       <x:c r="G27" s="5" t="n">
-        <x:v>46265.0</x:v>
+        <x:v>46356.0</x:v>
       </x:c>
       <x:c r="H27" s="7" t="str">
         <x:f t="shared" si="1"/>
@@ -11133,7 +11709,7 @@
       </x:c>
       <x:c r="N27" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-57.html</x:t>
+          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-44.html</x:t>
         </x:is>
       </x:c>
       <x:c r="O27" s="4"/>
@@ -11154,25 +11730,25 @@
       </x:c>
       <x:c r="B28" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Card</x:t>
+          <x:t xml:space="preserve">Merchant</x:t>
         </x:is>
       </x:c>
       <x:c r="C28" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">عروض الصيف مع بطاقاتنا</x:t>
+          <x:t xml:space="preserve">جيم تك</x:t>
         </x:is>
       </x:c>
       <x:c r="D28" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">يسري العرض من 19 يوليو حتى 26 سبتمبر 2026. 0% رسوم على العمليات الدولية بدون حد أدنى أو أعلى لمبلغ العملية باستخدام بطاقاتنا من فيزا.</x:t>
+          <x:t xml:space="preserve">يسري العرض من 19 أبريل حتى 31 ديسمبر 2026. خصم 50% على جميع الباقات.</x:t>
         </x:is>
       </x:c>
       <x:c r="E28" s="5"/>
       <x:c r="F28" s="5" t="n">
-        <x:v>46222.0</x:v>
+        <x:v>46131.0</x:v>
       </x:c>
       <x:c r="G28" s="5" t="n">
-        <x:v>46291.0</x:v>
+        <x:v>46387.0</x:v>
       </x:c>
       <x:c r="H28" s="7" t="str">
         <x:f t="shared" si="1"/>
@@ -11188,7 +11764,7 @@
       </x:c>
       <x:c r="N28" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-53.html</x:t>
+          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-45.html</x:t>
         </x:is>
       </x:c>
       <x:c r="O28" s="4"/>
@@ -11209,26 +11785,24 @@
       </x:c>
       <x:c r="B29" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
+          <x:t xml:space="preserve">Other</x:t>
         </x:is>
       </x:c>
       <x:c r="C29" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">فانوس للإنارة</x:t>
+          <x:t xml:space="preserve">حوالتك الدولية إلى باكستان مجانية</x:t>
         </x:is>
       </x:c>
       <x:c r="D29" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">يسري العرض من 22 أكتوبر 2025 حتى 20 أكتوبر 2026. خصم %12 بدون حد على جميع المنتجات باستثناء منتجات التأسيس.</x:t>
+          <x:t xml:space="preserve">هذا العرض ساري من 8 نوفمبر 2023. التحويل الدولي إلى حساب بنكي أو محافظ رقمية في باكستان بدون رسوم.</x:t>
         </x:is>
       </x:c>
       <x:c r="E29" s="5"/>
       <x:c r="F29" s="5" t="n">
-        <x:v>45952.0</x:v>
-      </x:c>
-      <x:c r="G29" s="5" t="n">
-        <x:v>46315.0</x:v>
-      </x:c>
+        <x:v>45238.0</x:v>
+      </x:c>
+      <x:c r="G29" s="5"/>
       <x:c r="H29" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -11243,7 +11817,7 @@
       </x:c>
       <x:c r="N29" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-19.html</x:t>
+          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-2.html</x:t>
         </x:is>
       </x:c>
       <x:c r="O29" s="4"/>
@@ -11269,17 +11843,17 @@
       </x:c>
       <x:c r="C30" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">فندق المبات</x:t>
+          <x:t xml:space="preserve">روماوَي</x:t>
         </x:is>
       </x:c>
       <x:c r="D30" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">يسري العرض من 10يوليو 2025 حتى 30 نوفمبر 2026. خصم %15 بدون حد على تجربتك الكاملة للفندق باستثناء خدمة البوفيه.</x:t>
+          <x:t xml:space="preserve">يسري العرض من 19 أبريل حتى 30 نوفمبر 2026 خصم 20% على جميع الطلبات بدون حد أدنى من خلال التطبيق المخصص لاستلام الطلبات.</x:t>
         </x:is>
       </x:c>
       <x:c r="E30" s="5"/>
       <x:c r="F30" s="5" t="n">
-        <x:v>45848.0</x:v>
+        <x:v>46131.0</x:v>
       </x:c>
       <x:c r="G30" s="5" t="n">
         <x:v>46356.0</x:v>
@@ -11298,7 +11872,7 @@
       </x:c>
       <x:c r="N30" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-13.html</x:t>
+          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-42.html</x:t>
         </x:is>
       </x:c>
       <x:c r="O30" s="4"/>
@@ -11319,25 +11893,25 @@
       </x:c>
       <x:c r="B31" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
+          <x:t xml:space="preserve">Card</x:t>
         </x:is>
       </x:c>
       <x:c r="C31" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">فوغا كلوسيت</x:t>
+          <x:t xml:space="preserve">عروض الصيف مع بطاقاتنا</x:t>
         </x:is>
       </x:c>
       <x:c r="D31" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">يسري العرض من 19 أبريل حتى 30 سبتمبر 2026. ادفع باستخدام البطاقات التالية لـ Mobily Pay (البلاتينية و سجنيتشر) مع الرمز الترويجي "VISA10" للحصول على الخصم.</x:t>
+          <x:t xml:space="preserve">يسري العرض من 19 يوليو حتى 26 سبتمبر 2026. 0% رسوم على العمليات الدولية بدون حد أدنى أو أعلى لمبلغ العملية باستخدام بطاقاتنا من فيزا.</x:t>
         </x:is>
       </x:c>
       <x:c r="E31" s="5"/>
       <x:c r="F31" s="5" t="n">
-        <x:v>46131.0</x:v>
+        <x:v>46222.0</x:v>
       </x:c>
       <x:c r="G31" s="5" t="n">
-        <x:v>46295.0</x:v>
+        <x:v>46291.0</x:v>
       </x:c>
       <x:c r="H31" s="7" t="str">
         <x:f t="shared" si="1"/>
@@ -11353,7 +11927,7 @@
       </x:c>
       <x:c r="N31" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-49.html</x:t>
+          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-53.html</x:t>
         </x:is>
       </x:c>
       <x:c r="O31" s="4"/>
@@ -12517,7 +13091,7 @@
       </x:c>
       <x:c r="D13" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">0% fees on eligible international POS purchases and international ATM withdrawals outside Saudi Arabia.</x:t>
+          <x:t xml:space="preserve">Zero International Card Transaction Fees The offer is valid from May 1, 2026, at 12:00 AM until December 31, 2026, at 11:59 PM, KSA time. International transaction fees are reduced to 0% (instead of 2.25%) for international Point of Sale (POS) transactions. Zero fees apply to international ATM cash withdrawals. The offer is valid while traveling outside the Kingdom of Saudi Arabia and does not apply to international online stores, websites, or mobile applications. tiqmo’s Standard Terms and Conditions, available on the App, shall apply. tiqmo reserves the right to amend the terms and conditions or suspend or cancel this promotion at any time. The revised terms and conditions shall become effective immediately upon publication on the App or the tiqmo website.</x:t>
         </x:is>
       </x:c>
       <x:c r="E13" s="5"/>
@@ -12556,7 +13130,7 @@
       </x:c>
       <x:c r="N13" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://www.tiqmo.com/ar/offers</x:t>
+          <x:t xml:space="preserve">https://tiqmo.com/en/offers</x:t>
         </x:is>
       </x:c>
       <x:c r="O13" s="63" t="inlineStr">
@@ -12566,12 +13140,12 @@
       </x:c>
       <x:c r="P13" s="63" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://x.com/tiqmo/status/2082496811798085847</x:t>
+          <x:t xml:space="preserve">https://x.com/tiqmo/status/2081409451844870239</x:t>
         </x:is>
       </x:c>
       <x:c r="Q13" s="63" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">https://www.facebook.com/Tiqmoksa/posts/sar-250000-cashbacksimple-every-riyal-you-spend-a-chance-to-win-sar-250000-every/1001313055996026/</x:t>
+          <x:t xml:space="preserve">https://www.facebook.com/Tiqmoksa/videos/1605667747644721/</x:t>
         </x:is>
       </x:c>
       <x:c r="R13" s="63" t="inlineStr">
@@ -12597,12 +13171,26 @@
         <x:f t="shared" si="0">IF(C14="","",ROW()-8)</x:f>
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B14" s="4"/>
-      <x:c r="C14" s="4"/>
-      <x:c r="D14" s="4"/>
+      <x:c r="B14" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Card</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C14" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SAR 250,000 Spend &amp; Win Campaign</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D14" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Card spending generated chances to win SAR 250,000, with enhanced chances on international purchases.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E14" s="5"/>
       <x:c r="F14" s="5"/>
-      <x:c r="G14" s="5"/>
+      <x:c r="G14" s="5" t="n">
+        <x:v>46234.0</x:v>
+      </x:c>
       <x:c r="H14" s="7" t="n">
         <x:f t="shared" si="1">IF(OR(C14="",G14=""),"",G14-TODAY())</x:f>
         <x:v>-6</x:v>
@@ -12611,20 +13199,50 @@
         <x:f t="shared" si="2">IF(C14="","",IF(G14="","End Date Not Stated",IF(G14&lt;TODAY(),"Expired",IF(G14&lt;=TODAY()+7,"Expiring ≤7 Days",IF(G14&lt;=TODAY()+30,"Expiring 8–30 Days","Active")))))</x:f>
         <x:v>Expired</x:v>
       </x:c>
-      <x:c r="J14" s="4"/>
-      <x:c r="K14" s="4"/>
-      <x:c r="L14" s="4"/>
+      <x:c r="J14" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Card purchases</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K14" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Each SAR spent generated multiple chances; international purchases generated up to eight chances per SAR</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L14" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">tiqmo card customers</x:t>
+        </x:is>
+      </x:c>
       <x:c r="M14" s="9" t="str">
         <x:f t="shared" si="3">IF(C14="","",IF(N14&lt;&gt;"",N14,IF(O14&lt;&gt;"",O14,IF(P14&lt;&gt;"",P14,IF(Q14&lt;&gt;"",Q14,IF(R14&lt;&gt;"",R14,""))))))</x:f>
         <x:v>https://www.tiqmo.com/ar/offers</x:v>
       </x:c>
-      <x:c r="N14" s="4"/>
+      <x:c r="N14" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.tiqmo.com/ar/offers</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O14" s="4"/>
-      <x:c r="P14" s="4"/>
-      <x:c r="Q14" s="4"/>
+      <x:c r="P14" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://x.com/tiqmo/status/2082496811798085847</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q14" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.facebook.com/Tiqmoksa/posts/sar-250000-cashbacksimple-every-riyal-you-spend-a-chance-to-win-sar-250000-every/1001313055996026/</x:t>
+        </x:is>
+      </x:c>
       <x:c r="R14" s="4"/>
-      <x:c r="S14" s="4"/>
-      <x:c r="T14" s="5"/>
+      <x:c r="S14" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">An official X post dated 29 July stated that two days remained, so the campaign end date is recorded as 31 July 2026. The campaign is retained as recent expired context.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="T14" s="5" t="n">
+        <x:v>46240.0</x:v>
+      </x:c>
       <x:c r="U14" s="35" t="str">
         <x:f t="shared" si="4">IF(C14="","",IF(COUNTA(O14:R14)=0,"No direct social post verified",IF(O14&lt;&gt;"","Instagram","")&amp;IF(AND(O14&lt;&gt;"",OR(P14&lt;&gt;"",Q14&lt;&gt;"",R14&lt;&gt;"")),", ","")&amp;IF(P14&lt;&gt;"","X","")&amp;IF(AND(P14&lt;&gt;"",OR(Q14&lt;&gt;"",R14&lt;&gt;"")),", ","")&amp;IF(Q14&lt;&gt;"","Facebook","")&amp;IF(AND(Q14&lt;&gt;"",R14&lt;&gt;""),", ","")&amp;IF(R14&lt;&gt;"","TikTok","")))</x:f>
         <x:v>X, Facebook</x:v>
@@ -12634,12 +13252,28 @@
       <x:c r="A15" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B15" s="4"/>
-      <x:c r="C15" s="4"/>
-      <x:c r="D15" s="4"/>
+      <x:c r="B15" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Card</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C15" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Every riyal you spend is a chance to win 250,000 SAR</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D15" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Every riyal you spend is a chance to win 250,000 SAR The offer is valid from June 1, 2026, at 12:00 AM until June 30, 2026, at 11:59 PM, KSA time. Instant Cashback applies to total eligible purchases made with tiqmo Platinum Card, where the user will be entitled to increasing cashback on the value of transactions only upon successful payment online or at points of sale (POS). The cashback percentage is as per the following tiers: Tier 1: 0.1% for transactions between SAR 0 and SAR 1,500. Tier 2: 0.2% for transactions between SAR 1,501 and SAR 3,000. Tier 3: 0.3% for transactions between SAR 3,001 and SAR 5,000. Tier 4: 0.4% for transactions of SAR 5,001 and above. Eligibility to enter the draw for cashback prizes is as follows: Local Card Transactions: For every Riyal spent in Tier 1, the customer will receive 1 chance. For every Riyal spent in Tier 2, the customer will receive 2 chances. For every Riyal spent in Tier 3, the customer will receive 3 chances. For every Riyal spent in Tier 4, the customer will receive 4 chances. International Card Transactions &amp; E-commerce: For every Riyal spent in Tier 1, the customer will receive 2 chances. For every Riyal spent in Tier 2, the customer will receive 4 chances. For every Riyal spent in Tier 3, the customer will receive 6 chances. For every Riyal spent in Tier 4, the customer will receive 8 chances. Monthly Cashback Prize Allocation: SAR 250,000 → 1 winner = SAR 250,000 SAR 100,000 → 2 winners = SAR 200,000 SAR 50,000 → 3 winners = SAR 150,000 SAR 20,000 → 4 winners = SAR 80,000 SAR 10,000 → 10 winners = SAR 100,000 SAR 5,000 →</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E15" s="5"/>
-      <x:c r="F15" s="5"/>
-      <x:c r="G15" s="5"/>
+      <x:c r="F15" s="5" t="n">
+        <x:v>46174.0</x:v>
+      </x:c>
+      <x:c r="G15" s="5" t="n">
+        <x:v>46203.0</x:v>
+      </x:c>
       <x:c r="H15" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -12652,7 +13286,11 @@
       <x:c r="M15" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N15" s="4"/>
+      <x:c r="N15" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://tiqmo.com/en/offers</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O15" s="4"/>
       <x:c r="P15" s="4"/>
       <x:c r="Q15" s="4"/>
@@ -12667,9 +13305,21 @@
       <x:c r="A16" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B16" s="4"/>
-      <x:c r="C16" s="4"/>
-      <x:c r="D16" s="4"/>
+      <x:c r="B16" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Engagement</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C16" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Play and Earn</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D16" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Play and Earn Terms and Conditions for the Game: The game is free to play for all tiqmo users (no conditions or limitations). The game center’s daily rounds are based on winners' points, which are calculated daily from 12:00:00 AM to 11:59:59 PM. Rewards will be deposited into the winners' wallets during the following day. Attempts are unlimited. After playing, the following information will be showcased: Points Current rank The game consists of 25 levels, with a maximum score of 11,378 points. Players are ranked based on points earned during the game. The rewards per rank are: 1st place = SAR 100 2nd place = SAR 75 3rd place = SAR 50 4th to 50th place = SAR 30 51st to 100th place = SAR 20 101st to 500th place = SAR 10 In case of a tie in points, priority for a higher rank will be given to the first user reaching the highest score. tiqmo’s Standard Terms and Conditions, available on the App, shall apply.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E16" s="5"/>
       <x:c r="F16" s="5"/>
       <x:c r="G16" s="5"/>
@@ -12685,7 +13335,11 @@
       <x:c r="M16" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N16" s="4"/>
+      <x:c r="N16" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://tiqmo.com/en/offers</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O16" s="4"/>
       <x:c r="P16" s="4"/>
       <x:c r="Q16" s="4"/>
@@ -12700,9 +13354,21 @@
       <x:c r="A17" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B17" s="4"/>
-      <x:c r="C17" s="4"/>
-      <x:c r="D17" s="4"/>
+      <x:c r="B17" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Remittance</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C17" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Your Monthly Streak</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D17" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Your Monthly Streak The campaign is valid from June 1st, 2026 until June 30st, 2026, KSA time. The rewards are applicable to successful international transfers with a value of SAR 1,500 or more, where: All successful international transfers with an amount of SAR 1,500 or more are subject to a 5 SAR fee based on the transfer destination. Transfers below SAR 1,500 will be subject to fees based on the transfer destination. Each user is eligible to receive one cashback reward per month upon completing their first successful international transfer of SAR 1,500 or more in that month, according to the monthly reward structure below. The monthly cashback rewards are granted sequentially and are limited to a maximum of 12 months, provided the eligibility criteria are met in each qualifying month. Monthly Cashback Rewards: 1st month: SAR 5 2nd month: SAR 10 3rd month: SAR 5 4th month: SAR 10 5th month: SAR 5 6th month: SAR 10 7th month: SAR 5 8th month: SAR 10 9th month: SAR 5 10th month: SAR 10 11th month: SAR 5 12th month: SAR 10 To upgrade to the next monthly cashback reward, customers must complete at least one successful international transfer of SAR 1,500 or more before 11:59:59 PM on the last day of each qualifying month. The 12-month cashback eligibility period starts from the month in which the customer completes their first qualifying international transfer of SAR 1,500 or more. Customers who qualify in any month between January 2026 and December 2026 may continue to earn one cashback reward per month for up to 12 consecutive months, provided the monthly criteria are met. I</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E17" s="5"/>
       <x:c r="F17" s="5"/>
       <x:c r="G17" s="5"/>
@@ -12718,7 +13384,11 @@
       <x:c r="M17" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N17" s="4"/>
+      <x:c r="N17" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://tiqmo.com/en/offers</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O17" s="4"/>
       <x:c r="P17" s="4"/>
       <x:c r="Q17" s="4"/>
@@ -15871,8 +16541,12 @@
         </x:is>
       </x:c>
       <x:c r="E10" s="5"/>
-      <x:c r="F10" s="5"/>
-      <x:c r="G10" s="5"/>
+      <x:c r="F10" s="5" t="n">
+        <x:v>46197.0</x:v>
+      </x:c>
+      <x:c r="G10" s="5" t="n">
+        <x:v>46265.0</x:v>
+      </x:c>
       <x:c r="H10" s="7" t="str">
         <x:f t="shared" si="1">IF(OR(C10="",G10=""),"",G10-TODAY())</x:f>
       </x:c>
@@ -15899,7 +16573,11 @@
         <x:f t="shared" si="3">IF(C10="","",IF(N10&lt;&gt;"",N10,IF(O10&lt;&gt;"",O10,IF(P10&lt;&gt;"",P10,IF(Q10&lt;&gt;"",Q10,IF(R10&lt;&gt;"",R10,""))))))</x:f>
         <x:v>https://www.facebook.com/AlinmaPaySA/posts/%EF%B8%8F-fees-gonetravel-anywhere-and-use-your-alinmapay-cashback-cards-without-worryin/1619335260194305/</x:v>
       </x:c>
-      <x:c r="N10" s="4"/>
+      <x:c r="N10" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/OIF-JUN2026</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O10" s="4"/>
       <x:c r="P10" s="4"/>
       <x:c r="Q10" s="63" t="inlineStr">
@@ -15942,8 +16620,12 @@
         </x:is>
       </x:c>
       <x:c r="E11" s="5"/>
-      <x:c r="F11" s="5"/>
-      <x:c r="G11" s="5"/>
+      <x:c r="F11" s="5" t="n">
+        <x:v>46242.0</x:v>
+      </x:c>
+      <x:c r="G11" s="5" t="n">
+        <x:v>46387.0</x:v>
+      </x:c>
       <x:c r="H11" s="7" t="str">
         <x:f t="shared" si="1">IF(OR(C11="",G11=""),"",G11-TODAY())</x:f>
       </x:c>
@@ -15970,7 +16652,11 @@
         <x:f t="shared" si="3">IF(C11="","",IF(N11&lt;&gt;"",N11,IF(O11&lt;&gt;"",O11,IF(P11&lt;&gt;"",P11,IF(Q11&lt;&gt;"",Q11,IF(R11&lt;&gt;"",R11,""))))))</x:f>
         <x:v>https://www.instagram.com/alinmapay/p/CC_U-JDB6yh/</x:v>
       </x:c>
-      <x:c r="N11" s="4"/>
+      <x:c r="N11" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/India-Transfer-Fee-Offer-Aug26</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O11" s="63" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://www.instagram.com/alinmapay/p/CC_U-JDB6yh/</x:t>
@@ -15987,11 +16673,7 @@
         </x:is>
       </x:c>
       <x:c r="R11" s="4"/>
-      <x:c r="S11" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Campaign end date is not stated in the official post. Social verification: Official Instagram and X posts explicitly promote international transfers for a SAR 5 fee. The Instagram creative is a corridor-specific execution within the same offer.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="S11" s="4"/>
       <x:c r="T11" s="5" t="n">
         <x:v>46240.0</x:v>
       </x:c>
@@ -16097,7 +16779,9 @@
         <x:v>46239.0</x:v>
       </x:c>
       <x:c r="F13" s="5"/>
-      <x:c r="G13" s="5"/>
+      <x:c r="G13" s="5" t="n">
+        <x:v>46384.0</x:v>
+      </x:c>
       <x:c r="H13" s="7" t="str">
         <x:f t="shared" si="1">IF(OR(C13="",G13=""),"",G13-TODAY())</x:f>
       </x:c>
@@ -16124,7 +16808,11 @@
         <x:f t="shared" si="3">IF(C13="","",IF(N13&lt;&gt;"",N13,IF(O13&lt;&gt;"",O13,IF(P13&lt;&gt;"",P13,IF(Q13&lt;&gt;"",Q13,IF(R13&lt;&gt;"",R13,""))))))</x:f>
         <x:v>https://www.instagram.com/alinmapay/p/DbqaY05mm9E/</x:v>
       </x:c>
-      <x:c r="N13" s="4"/>
+      <x:c r="N13" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Musaned-Cashback</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O13" s="4" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">https://www.instagram.com/alinmapay/p/DbqaY05mm9E/</x:t>
@@ -16137,11 +16825,7 @@
       </x:c>
       <x:c r="Q13" s="4"/>
       <x:c r="R13" s="4"/>
-      <x:c r="S13" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Official Instagram and X posts announce three winners, each receiving 100% cashback up to SAR 1,000. The campaign end date is not stated.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="S13" s="4"/>
       <x:c r="T13" s="5" t="n">
         <x:v>46240.0</x:v>
       </x:c>
@@ -16154,12 +16838,28 @@
       <x:c r="A14" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B14" s="4"/>
-      <x:c r="C14" s="4"/>
-      <x:c r="D14" s="4"/>
+      <x:c r="B14" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C14" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بأجواء رائعة بخصم 20% في اجو</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D14" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بأجواء رائعة بخصم 20% في اجو الشروط والأحكام: • استمتع بأجواء رائعة في اجو واستمتع بخصم 20% عند الدفع باستخدام بطاقات الكاش باك من الإنماء باي. • يسري العرض من 7 ديسمبر 2025 و حتى 20 نوفمبر 2026. • خصم 20% عند الدفع باستخدام بطاقات الكاش باك للإنماء باي خلال الفترة المشار إليها على جميع الطلبات من قائمة الطعام الانتقائية ولا يسري على قائمة الطعام المجهز مسبقاً ( Set Menu) • يسري العرض من الاحد الى الخميس من الساعة 1 م الى الساعة 6 م. • العرض لا يشمل تطبيقات التوصيل. • الخصم يشمل الفروع داخل السعودية في الرياض • لا يطبق العرض مع اي عروض اخرى ولا يمكن الجمع بين اكثر من عرض في نفس الوقت. • لا يسري العرض مع ايام المناسبات والاعياد والاجازات الرسمية مثال (اليوم الوطني – يوم التأسيس – ويوم </x:t>
+        </x:is>
+      </x:c>
       <x:c r="E14" s="5"/>
-      <x:c r="F14" s="5"/>
-      <x:c r="G14" s="5"/>
+      <x:c r="F14" s="5" t="n">
+        <x:v>45998.0</x:v>
+      </x:c>
+      <x:c r="G14" s="5" t="n">
+        <x:v>46346.0</x:v>
+      </x:c>
       <x:c r="H14" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16172,13 +16872,19 @@
       <x:c r="M14" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N14" s="4"/>
+      <x:c r="N14" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Agio-dec25</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O14" s="4"/>
       <x:c r="P14" s="4"/>
       <x:c r="Q14" s="4"/>
       <x:c r="R14" s="4"/>
       <x:c r="S14" s="4"/>
-      <x:c r="T14" s="5"/>
+      <x:c r="T14" s="5" t="n">
+        <x:v>46259.741513515</x:v>
+      </x:c>
       <x:c r="U14" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16187,12 +16893,26 @@
       <x:c r="A15" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B15" s="4"/>
-      <x:c r="C15" s="4"/>
-      <x:c r="D15" s="4"/>
+      <x:c r="B15" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C15" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بأجواء رائعة بخصم 20% في بيف بار</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D15" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بأجواء رائعة بخصم 20% في بيف بار الشروط والأحكام : • استمتع بأجواء رائعة في بيف بار واستمتع بخصم 20% عند الدفع باستخدام بطاقات الكاش باك للإنماء باي • يسري العرض حتى 20-11-2026. • خصم 20% عند الدفع باستخدام بطاقات الكاش باك للإنماء باي خلال الفترة المشار إليها على جميع الطلبات من قائمة الطعام الانتقائية ولا يسري على قائمة الطعام المجهز مسبقاً ( Set Menu) • يسري العرض من الاحد الى الخميس من الساعة 1 م الى الساعة 6 م. • العرض لا يشمل تطبيقات التوصيل. • الخصم يشمل الفروع داخل السعودية في الرياض • لا يطبق العرض مع اي عروض اخرى ولا يمكن الجمع بين اكثر من عرض في نفس الوقت. • لا يسري العرض مع ايام المناسبات والاعياد والاجازات الرسمية مثال (اليوم الوطني – يوم التأسيس – ويوم 31/12 ويوم 01/01 م</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E15" s="5"/>
       <x:c r="F15" s="5"/>
-      <x:c r="G15" s="5"/>
+      <x:c r="G15" s="5" t="n">
+        <x:v>46346.0</x:v>
+      </x:c>
       <x:c r="H15" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16205,13 +16925,19 @@
       <x:c r="M15" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N15" s="4"/>
+      <x:c r="N15" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Winter---Beefbar-offer-Dece25</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O15" s="4"/>
       <x:c r="P15" s="4"/>
       <x:c r="Q15" s="4"/>
       <x:c r="R15" s="4"/>
       <x:c r="S15" s="4"/>
-      <x:c r="T15" s="5"/>
+      <x:c r="T15" s="5" t="n">
+        <x:v>46259.741513515</x:v>
+      </x:c>
       <x:c r="U15" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16220,12 +16946,26 @@
       <x:c r="A16" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B16" s="4"/>
-      <x:c r="C16" s="4"/>
-      <x:c r="D16" s="4"/>
+      <x:c r="B16" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C16" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بأجواء رائعة بخصم 20% في سان كارلو شيكيتي</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D16" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بأجواء رائعة في سان كارلو شيكيتي واستمتع بخصم 20% عند الدفع باستخدام بطاقات الكاش باك للإنماء باي يسري العرض حتى 20-11-2026.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E16" s="5"/>
       <x:c r="F16" s="5"/>
-      <x:c r="G16" s="5"/>
+      <x:c r="G16" s="5" t="n">
+        <x:v>46346.0</x:v>
+      </x:c>
       <x:c r="H16" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16238,13 +16978,19 @@
       <x:c r="M16" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N16" s="4"/>
+      <x:c r="N16" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Winter-San-Carlo-Cicchetti-offer-Dece25</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O16" s="4"/>
       <x:c r="P16" s="4"/>
       <x:c r="Q16" s="4"/>
       <x:c r="R16" s="4"/>
       <x:c r="S16" s="4"/>
-      <x:c r="T16" s="5"/>
+      <x:c r="T16" s="5" t="n">
+        <x:v>46259.741513515</x:v>
+      </x:c>
       <x:c r="U16" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16253,12 +16999,28 @@
       <x:c r="A17" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B17" s="4"/>
-      <x:c r="C17" s="4"/>
-      <x:c r="D17" s="4"/>
+      <x:c r="B17" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C17" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بأجواء رائعة واحصل على خصم 15% في أيرث كافيه</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D17" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بأجواء رائعة واحصل على خصم 15% في أيرث كافيه الشروط والأحكام : • استمتع بأجواء رائعة في أيرث كافيه وحصل على خصم 15% عند الدفع باستخدام ب طاقات الكاش باك للإنماء باي • يسري العرض حتى 20-11-2026. • خصم 15% عند الدفع باستخدام بطاقات الكاش باي للإنماء خلال الفترة المشار إليها على جميع الطلبات من قائمة الطعام الانتقائية ولا يسري على قائمة الطعام المجهز مسبقاً ( Set Menu) • يسري العرض من الاحد الى الخميس من الساعة 7 ص الى الساعة 6 م. • العرض لا يشمل تطبيقات التوصيل. • الخصم يشمل الفروع داخل السعودية في الرياض و جدة و الخبر . • لا يطبق العرض مع اي عروض اخرى ولا يمكن الجمع بين اكثر من عرض في نفس الوقت. • لا يسري العرض مع ايام المناسبات والاعياد والاجازات الرسمية مثال (اليوم الوطني – يوم التأس</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E17" s="5"/>
-      <x:c r="F17" s="5"/>
-      <x:c r="G17" s="5"/>
+      <x:c r="F17" s="5" t="n">
+        <x:v>45998.0</x:v>
+      </x:c>
+      <x:c r="G17" s="5" t="n">
+        <x:v>46346.0</x:v>
+      </x:c>
       <x:c r="H17" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16271,13 +17033,19 @@
       <x:c r="M17" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N17" s="4"/>
+      <x:c r="N17" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Urth-Cafe-dec25</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O17" s="4"/>
       <x:c r="P17" s="4"/>
       <x:c r="Q17" s="4"/>
       <x:c r="R17" s="4"/>
       <x:c r="S17" s="4"/>
-      <x:c r="T17" s="5"/>
+      <x:c r="T17" s="5" t="n">
+        <x:v>46259.741513515</x:v>
+      </x:c>
       <x:c r="U17" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16286,12 +17054,28 @@
       <x:c r="A18" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B18" s="4"/>
-      <x:c r="C18" s="4"/>
-      <x:c r="D18" s="4"/>
+      <x:c r="B18" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C18" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بأجواء رائعة واستمتع بخصم 20% في بيف بار</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D18" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بأجواء رائعة واستمتع بخصم 20% في بيف بار الشروط والأحكام: • استمتع بأجواء رائعة في بيف بار واستمتع بخصم 20% عند الدفع باستخدام بطاقات الكاش باك من الإنماء باي • يسري العرض من 7 ديسمبر 2025 و حتى 20 نوفمبر 2026. • خصم 20% عند الدفع باستخدام بطاقات الكاش باك للإنماء باي خلال الفترة المشار إليها على جميع الطلبات من قائمة الطعام الانتقائية ولا يسري على قائمة الطعام المجهز مسبقاً ( Set Menu) • يسري العرض من الاحد الى الخميس من الساعة 1 م الى الساعة 6 م. • العرض لا يشمل تطبيقات التوصيل. • الخصم يشمل الفروع داخل السعودية في الرياض • لا يطبق العرض مع اي عروض اخرى ولا يمكن الجمع بين اكثر من عرض في نفس الوقت. • لا يسري العرض مع ايام المناسبات والاعياد والاجازات الرسمية مثال (اليوم الوطني – يوم </x:t>
+        </x:is>
+      </x:c>
       <x:c r="E18" s="5"/>
-      <x:c r="F18" s="5"/>
-      <x:c r="G18" s="5"/>
+      <x:c r="F18" s="5" t="n">
+        <x:v>45998.0</x:v>
+      </x:c>
+      <x:c r="G18" s="5" t="n">
+        <x:v>46346.0</x:v>
+      </x:c>
       <x:c r="H18" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16304,13 +17088,19 @@
       <x:c r="M18" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N18" s="4"/>
+      <x:c r="N18" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Beefbar-dec25</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O18" s="4"/>
       <x:c r="P18" s="4"/>
       <x:c r="Q18" s="4"/>
       <x:c r="R18" s="4"/>
       <x:c r="S18" s="4"/>
-      <x:c r="T18" s="5"/>
+      <x:c r="T18" s="5" t="n">
+        <x:v>46259.82478451854</x:v>
+      </x:c>
       <x:c r="U18" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16319,12 +17109,28 @@
       <x:c r="A19" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B19" s="4"/>
-      <x:c r="C19" s="4"/>
-      <x:c r="D19" s="4"/>
+      <x:c r="B19" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C19" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بأجواء رائعة واستمتع بخصم 20% في روباتا</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D19" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بأجواء رائعة واستمتع بخصم 20% في روباتا الشروط والأحكام: • استمتع بأجواء رائعة في روباتا واستمتع بخصم 20% عند الدفع باستخدام بطاقات الكاش باك من الإنماء باي. • يسري العرض من 7 ديسمبر 2025 و حتى 20 نوفمبر 2026. • خصم 20% عند الدفع باستخدام بطاقات الكاش باك للإنماء باي خلال الفترة المشار إليها على جميع الطلبات من قائمة الطعام الانتقائية ولا يسري على قائمة الطعام المجهز مسبقاً ( Set Menu) • يسري العرض من الاحد الى الخميس من الساعة 1 م الى الساعة 6 م. • العرض لا يشمل تطبيقات التوصيل. • الخصم يشمل الفروع داخل السعودية في الرياض • لا يطبق العرض مع اي عروض اخرى ولا يمكن الجمع بين اكثر من عرض في نفس الوقت. • لا يسري العرض مع ايام المناسبات والاعياد والاجازات الرسمية مثال (اليوم الوطني – يوم ا</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E19" s="5"/>
-      <x:c r="F19" s="5"/>
-      <x:c r="G19" s="5"/>
+      <x:c r="F19" s="5" t="n">
+        <x:v>45998.0</x:v>
+      </x:c>
+      <x:c r="G19" s="5" t="n">
+        <x:v>46346.0</x:v>
+      </x:c>
       <x:c r="H19" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16337,13 +17143,19 @@
       <x:c r="M19" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N19" s="4"/>
+      <x:c r="N19" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Robata-dec25</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O19" s="4"/>
       <x:c r="P19" s="4"/>
       <x:c r="Q19" s="4"/>
       <x:c r="R19" s="4"/>
       <x:c r="S19" s="4"/>
-      <x:c r="T19" s="5"/>
+      <x:c r="T19" s="5" t="n">
+        <x:v>46259.741513515</x:v>
+      </x:c>
       <x:c r="U19" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16352,12 +17164,28 @@
       <x:c r="A20" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B20" s="4"/>
-      <x:c r="C20" s="4"/>
-      <x:c r="D20" s="4"/>
+      <x:c r="B20" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C20" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بأجواء رائعة واستمتع بخصم 20% في كريزي بيتزا</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D20" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بأجواء رائعة واستمتع بخصم 20% في كريزي بيتزا الشروط والأحكام: • استمتع بأجواء رائعة في كريزي بيتزا واستمتع بخصم 20% عند الدفع باستخدام بطاقات الكاش باك من الإنماء باي • يسري العرض من 7 ديسمبر 2025 و حتى 20 نوفمبر 2026. • خصم 20% عند الدفع باستخدام بطاقات الكاش باك للإنماء باي خلال الفترة المشار إليها على جميع الطلبات من قائمة الطعام الانتقائية ولا يسري على قائمة الطعام المجهز مسبقاً ( Set Menu) • يسري العرض من الاحد الى الخميس من الساعة 1 م الى الساعة 6 م. • العرض لا يشمل تطبيقات التوصيل. • الخصم يشمل الفروع داخل السعودية: • الرياض فرع شارع التحلية طوال أيام الأسبوع وطوال اليوم • الرياض فرع عود سكوير من الأحد الى الخميس من 1 م حتى 6 م • الرياض فرع نورث يارد من الأحد الى الخميس من 1 م </x:t>
+        </x:is>
+      </x:c>
       <x:c r="E20" s="5"/>
-      <x:c r="F20" s="5"/>
-      <x:c r="G20" s="5"/>
+      <x:c r="F20" s="5" t="n">
+        <x:v>45998.0</x:v>
+      </x:c>
+      <x:c r="G20" s="5" t="n">
+        <x:v>46346.0</x:v>
+      </x:c>
       <x:c r="H20" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16370,13 +17198,19 @@
       <x:c r="M20" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N20" s="4"/>
+      <x:c r="N20" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Crazy-Pizza-dec25</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O20" s="4"/>
       <x:c r="P20" s="4"/>
       <x:c r="Q20" s="4"/>
       <x:c r="R20" s="4"/>
       <x:c r="S20" s="4"/>
-      <x:c r="T20" s="5"/>
+      <x:c r="T20" s="5" t="n">
+        <x:v>46259.741513515</x:v>
+      </x:c>
       <x:c r="U20" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16385,12 +17219,28 @@
       <x:c r="A21" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B21" s="4"/>
-      <x:c r="C21" s="4"/>
-      <x:c r="D21" s="4"/>
+      <x:c r="B21" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C21" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بأجواء رائعة واستمتع بخصم 20% في كويا</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D21" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بأجواء رائعة واستمتع بخصم 20% في كويا الشروط والأحكام: • استمتع بأجواء رائعة في كويا واستمتع بخصم 20% عند الدفع باستخدام بطاقات الكاش باك من الإنماء باي • يسري العرض من 7 ديسمبر 2025 و حتى 20 نوفمبر 2026. • خصم 20% عند الدفع باستخدام بطاقات الكاش باك للإنماء باي خلال الفترة المشار إليها على جميع الطلبات من قائمة الطعام الانتقائية ولا يسري على قائمة الطعام المجهز مسبقاً ( Set Menu) • يسري العرض من الاحد الى الخميس من الساعة 1 م الى الساعة 6 م. • العرض لا يشمل تطبيقات التوصيل. • الخصم يشمل الفروع داخل السعودية في الرياض • لا يطبق العرض مع اي عروض اخرى ولا يمكن الجمع بين اكثر من عرض في نفس الوقت. • لا يسري العرض مع ايام المناسبات والاعياد والاجازات الرسمية مثال (اليوم الوطني – يوم التأسي</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E21" s="5"/>
-      <x:c r="F21" s="5"/>
-      <x:c r="G21" s="5"/>
+      <x:c r="F21" s="5" t="n">
+        <x:v>45998.0</x:v>
+      </x:c>
+      <x:c r="G21" s="5" t="n">
+        <x:v>46346.0</x:v>
+      </x:c>
       <x:c r="H21" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16403,13 +17253,19 @@
       <x:c r="M21" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N21" s="4"/>
+      <x:c r="N21" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Coya-dec25</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O21" s="4"/>
       <x:c r="P21" s="4"/>
       <x:c r="Q21" s="4"/>
       <x:c r="R21" s="4"/>
       <x:c r="S21" s="4"/>
-      <x:c r="T21" s="5"/>
+      <x:c r="T21" s="5" t="n">
+        <x:v>46259.741513515</x:v>
+      </x:c>
       <x:c r="U21" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16418,12 +17274,28 @@
       <x:c r="A22" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B22" s="4"/>
-      <x:c r="C22" s="4"/>
-      <x:c r="D22" s="4"/>
+      <x:c r="B22" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C22" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بأجواء واستمتع بخصم 20% رائعة في سان كارلو شيكيتي</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D22" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بأجواء واستمتع بخصم 20% رائعة في سان كارلو شيكيتي الشروط والأحكام: • استمتع بأجواء رائعة في سان كارلو شيكيتي واستمتع بخصم 20% عند الدفع باستخدام بطاقات الكاش باك من الإنماء باي • يسري العرض من 7 ديسمبر 2025 و حتى 20 نوفمبر 2026. • خصم 20% عند الدفع باستخدام بطاقات الكاش باك للإنماء باي خلال الفترة المشار إليها على جميع الطلبات من قائمة الطعام الانتقائية ولا يسري على قائمة الطعام المجهز مسبقاً ( Set Menu) • يسري العرض من الاحد الى الخميس من الساعة 1 م الى الساعة 6 م. • العرض لا يشمل تطبيقات التوصيل. • • الخصم يشمل الفروع داخل السعودية في الرياض وجده والخبر • لا يطبق العرض مع اي عروض اخرى ولا يمكن الجمع بين اكثر من عرض في نفس الوقت. • لا يسري العرض مع ايام المناسبات والاعياد والاجازات ا</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E22" s="5"/>
-      <x:c r="F22" s="5"/>
-      <x:c r="G22" s="5"/>
+      <x:c r="F22" s="5" t="n">
+        <x:v>45998.0</x:v>
+      </x:c>
+      <x:c r="G22" s="5" t="n">
+        <x:v>46346.0</x:v>
+      </x:c>
       <x:c r="H22" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16436,13 +17308,19 @@
       <x:c r="M22" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N22" s="4"/>
+      <x:c r="N22" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/San-Carlo-Cicchetti-dec25</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O22" s="4"/>
       <x:c r="P22" s="4"/>
       <x:c r="Q22" s="4"/>
       <x:c r="R22" s="4"/>
       <x:c r="S22" s="4"/>
-      <x:c r="T22" s="5"/>
+      <x:c r="T22" s="5" t="n">
+        <x:v>46259.741513515</x:v>
+      </x:c>
       <x:c r="U22" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16451,12 +17329,28 @@
       <x:c r="A23" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B23" s="4"/>
-      <x:c r="C23" s="4"/>
-      <x:c r="D23" s="4"/>
+      <x:c r="B23" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C23" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بأجواء واستمتع بخصم 20% رائعة في سينيور ساسي</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D23" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بأجواء واستمتع بخصم 20% رائعة في سينيور ساسي الشروط والأحكام: • استمتع بأجواء رائعة في سينيور ساسي واستمتع بخصم 20% عند الدفع باستخدام بطاقات الكاش باك من الإنماء باي • يسري العرض من 7 ديسمبر 2025 و حتى 20 نوفمبر 2026. • خصم 20% عند الدفع باستخدام بطاقات الكاش باك للإنماء باي خلال الفترة المشار إليها على جميع الطلبات من قائمة الطعام الانتقائية ولا يسري على قائمة الطعام المجهز مسبقاً ( (Set Menu • يسري العرض من الاحد الى الخميس من الساعة 1 م الى الساعة 6 م. • العرض لا يشمل تطبيقات التوصيل. • الخصم يشمل الفروع داخل السعودية في الرياض • لا يطبق العرض مع اي عروض اخرى ولا يمكن الجمع بين اكثر من عرض في نفس الوقت. • لا يسري العرض مع ايام المناسبات والاعياد والاجازات الرسمية مثال (اليوم الوطن</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E23" s="5"/>
-      <x:c r="F23" s="5"/>
-      <x:c r="G23" s="5"/>
+      <x:c r="F23" s="5" t="n">
+        <x:v>45998.0</x:v>
+      </x:c>
+      <x:c r="G23" s="5" t="n">
+        <x:v>46346.0</x:v>
+      </x:c>
       <x:c r="H23" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16469,13 +17363,19 @@
       <x:c r="M23" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N23" s="4"/>
+      <x:c r="N23" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Signor-Sassi-dec25</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O23" s="4"/>
       <x:c r="P23" s="4"/>
       <x:c r="Q23" s="4"/>
       <x:c r="R23" s="4"/>
       <x:c r="S23" s="4"/>
-      <x:c r="T23" s="5"/>
+      <x:c r="T23" s="5" t="n">
+        <x:v>46259.741513515</x:v>
+      </x:c>
       <x:c r="U23" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16484,12 +17384,28 @@
       <x:c r="A24" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B24" s="4"/>
-      <x:c r="C24" s="4"/>
-      <x:c r="D24" s="4"/>
+      <x:c r="B24" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C24" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بأجواء واستمتع بخصم 20% رائعة في كايزو</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D24" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بأجواء واستمتع بخصم 20% رائعة في كايزو الشروط والأحكام: • استمتع بأجواء رائعة في كايزو واستمتع بخصم 20% عند الدفع باستخدام بطاقات الكاش باك من الإنماء باي • يسري العرض من 7 ديسمبر 2025 و حتى 20 نوفمبر 2026. • خصم 20% عند الدفع باستخدام بطاقات الكاش باك للإنماء باي خلال الفترة المشار إليها على جميع الطلبات من قائمة الطعام الانتقائية ولا يسري على قائمة الطعام المجهز مسبقاً ( Set Menu) • يسري العرض من الاحد الى الخميس من الساعة 1 م الى الساعة 6 م. • العرض لا يشمل تطبيقات التوصيل. • الخصم يشمل الفروع داخل السعودية في الرياض • لا يطبق العرض مع اي عروض اخرى ولا يمكن الجمع بين اكثر من عرض في نفس الوقت. • لا يسري العرض مع ايام المناسبات والاعياد والاجازات الرسمية مثال (اليوم الوطني – يوم التأ</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E24" s="5"/>
-      <x:c r="F24" s="5"/>
-      <x:c r="G24" s="5"/>
+      <x:c r="F24" s="5" t="n">
+        <x:v>45998.0</x:v>
+      </x:c>
+      <x:c r="G24" s="5" t="n">
+        <x:v>46346.0</x:v>
+      </x:c>
       <x:c r="H24" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16502,13 +17418,19 @@
       <x:c r="M24" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N24" s="4"/>
+      <x:c r="N24" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Kayzo-dec25</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O24" s="4"/>
       <x:c r="P24" s="4"/>
       <x:c r="Q24" s="4"/>
       <x:c r="R24" s="4"/>
       <x:c r="S24" s="4"/>
-      <x:c r="T24" s="5"/>
+      <x:c r="T24" s="5" t="n">
+        <x:v>46259.741513515</x:v>
+      </x:c>
       <x:c r="U24" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16517,12 +17439,28 @@
       <x:c r="A25" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B25" s="4"/>
-      <x:c r="C25" s="4"/>
-      <x:c r="D25" s="4"/>
+      <x:c r="B25" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C25" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بأجواء واستمتع بخصم 20% رائعة في ميازو</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D25" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بأجواء واستمتع بخصم 20% رائعة في ميازو الشروط والأحكام: • استمتع بأجواء رائعة في ميازو واستمتع بخصم 20% عند الدفع باستخدام بطاقات الكاش باك من الإنماء باي • يسري العرض من 7 ديسمبر 2025 و حتى 20 نوفمبر 2026. • خصم 20% عند الدفع باستخدام بطاقات الكاش باك للإنماء باي خلال الفترة المشار إليها على جميع الطلبات من قائمة الطعام الانتقائية ولا يسري على قائمة الطعام المجهز مسبقاً ( Set Menu) • يسري العرض من الاحد الى الخميس من الساعة 1 م الى الساعة 6 م. • العرض لا يشمل تطبيقات التوصيل. • الخصم يشمل الفروع داخل السعودية في الرياض • لا يطبق العرض مع اي عروض اخرى ولا يمكن الجمع بين اكثر من عرض في نفس الوقت. • لا يسري العرض مع ايام المناسبات والاعياد والاجازات الرسمية مثال (اليوم الوطني – يوم التأ</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E25" s="5"/>
-      <x:c r="F25" s="5"/>
-      <x:c r="G25" s="5"/>
+      <x:c r="F25" s="5" t="n">
+        <x:v>45998.0</x:v>
+      </x:c>
+      <x:c r="G25" s="5" t="n">
+        <x:v>46346.0</x:v>
+      </x:c>
       <x:c r="H25" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16535,13 +17473,19 @@
       <x:c r="M25" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N25" s="4"/>
+      <x:c r="N25" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/MYAZU-dec25</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O25" s="4"/>
       <x:c r="P25" s="4"/>
       <x:c r="Q25" s="4"/>
       <x:c r="R25" s="4"/>
       <x:c r="S25" s="4"/>
-      <x:c r="T25" s="5"/>
+      <x:c r="T25" s="5" t="n">
+        <x:v>46259.741513515</x:v>
+      </x:c>
       <x:c r="U25" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16550,12 +17494,28 @@
       <x:c r="A26" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B26" s="4"/>
-      <x:c r="C26" s="4"/>
-      <x:c r="D26" s="4"/>
+      <x:c r="B26" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C26" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بخصم 15% لدى المهيدب ريزدنس</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D26" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">• استمتع بخصم 15 % لدى المهيدب ريزدنس عند الدفع بأي من بطاقات الإنماء باي فيزا أو مدى. • يسري العرض من تاريخ 5 فبراير حتى 30 يناير 2027.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E26" s="5"/>
-      <x:c r="F26" s="5"/>
-      <x:c r="G26" s="5"/>
+      <x:c r="F26" s="5" t="n">
+        <x:v>46423.0</x:v>
+      </x:c>
+      <x:c r="G26" s="5" t="n">
+        <x:v>46417.0</x:v>
+      </x:c>
       <x:c r="H26" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16568,13 +17528,19 @@
       <x:c r="M26" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N26" s="4"/>
+      <x:c r="N26" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Al-Muhaidb-Offer---Feb-2026</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O26" s="4"/>
       <x:c r="P26" s="4"/>
       <x:c r="Q26" s="4"/>
       <x:c r="R26" s="4"/>
       <x:c r="S26" s="4"/>
-      <x:c r="T26" s="5"/>
+      <x:c r="T26" s="5" t="n">
+        <x:v>46259.82478451854</x:v>
+      </x:c>
       <x:c r="U26" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16583,12 +17549,28 @@
       <x:c r="A27" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B27" s="4"/>
-      <x:c r="C27" s="4"/>
-      <x:c r="D27" s="4"/>
+      <x:c r="B27" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C27" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بخصم 15% لدى فنادق إيواء</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D27" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">• استمتع بخصم 15 % لدى المهيدب ريزدنس عند الدفع بأي من بطاقات الإنماء باي فيزا أو مدى. • يسري العرض من تاريخ 5 فبراير حتى 30 يناير 2027.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E27" s="5"/>
-      <x:c r="F27" s="5"/>
-      <x:c r="G27" s="5"/>
+      <x:c r="F27" s="5" t="n">
+        <x:v>46423.0</x:v>
+      </x:c>
+      <x:c r="G27" s="5" t="n">
+        <x:v>46417.0</x:v>
+      </x:c>
       <x:c r="H27" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16601,13 +17583,19 @@
       <x:c r="M27" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N27" s="4"/>
+      <x:c r="N27" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/EWAA-Hotels-Offer---Feb-2026</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O27" s="4"/>
       <x:c r="P27" s="4"/>
       <x:c r="Q27" s="4"/>
       <x:c r="R27" s="4"/>
       <x:c r="S27" s="4"/>
-      <x:c r="T27" s="5"/>
+      <x:c r="T27" s="5" t="n">
+        <x:v>46259.741513515</x:v>
+      </x:c>
       <x:c r="U27" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16616,12 +17604,28 @@
       <x:c r="A28" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B28" s="4"/>
-      <x:c r="C28" s="4"/>
-      <x:c r="D28" s="4"/>
+      <x:c r="B28" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C28" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بخصم 15% لدى فنادق جراند بلازا</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D28" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">• استمتع بخصم 15 % لدى فنادق جراند بلازا عند الدفع بأي من بطاقات الإنماء باي فيزا أو مدى. • يسري العرض من تاريخ 5 فبراير حتى 30 يناير 2027.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E28" s="5"/>
-      <x:c r="F28" s="5"/>
-      <x:c r="G28" s="5"/>
+      <x:c r="F28" s="5" t="n">
+        <x:v>46423.0</x:v>
+      </x:c>
+      <x:c r="G28" s="5" t="n">
+        <x:v>46417.0</x:v>
+      </x:c>
       <x:c r="H28" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16634,13 +17638,19 @@
       <x:c r="M28" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N28" s="4"/>
+      <x:c r="N28" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Grand-Plaza-Hotels---Feb-2026</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O28" s="4"/>
       <x:c r="P28" s="4"/>
       <x:c r="Q28" s="4"/>
       <x:c r="R28" s="4"/>
       <x:c r="S28" s="4"/>
-      <x:c r="T28" s="5"/>
+      <x:c r="T28" s="5" t="n">
+        <x:v>46259.82478451854</x:v>
+      </x:c>
       <x:c r="U28" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16649,12 +17659,28 @@
       <x:c r="A29" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B29" s="4"/>
-      <x:c r="C29" s="4"/>
-      <x:c r="D29" s="4"/>
+      <x:c r="B29" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C29" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بخصم 30% لدى ستايلي</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D29" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">• استمتع بخصم 30% لدى ستايلي عند الدفع بأي من بطاقات الإنماء باي فيزا. • يسري العرض من تاريخ 5 فبراير حتى 30 ديسمبر 2026.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E29" s="5"/>
-      <x:c r="F29" s="5"/>
-      <x:c r="G29" s="5"/>
+      <x:c r="F29" s="5" t="n">
+        <x:v>46058.0</x:v>
+      </x:c>
+      <x:c r="G29" s="5" t="n">
+        <x:v>46386.0</x:v>
+      </x:c>
       <x:c r="H29" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16667,13 +17693,19 @@
       <x:c r="M29" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N29" s="4"/>
+      <x:c r="N29" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Stily-Offer---Feb-2026</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O29" s="4"/>
       <x:c r="P29" s="4"/>
       <x:c r="Q29" s="4"/>
       <x:c r="R29" s="4"/>
       <x:c r="S29" s="4"/>
-      <x:c r="T29" s="5"/>
+      <x:c r="T29" s="5" t="n">
+        <x:v>46259.82478451854</x:v>
+      </x:c>
       <x:c r="U29" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16682,12 +17714,28 @@
       <x:c r="A30" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B30" s="4"/>
-      <x:c r="C30" s="4"/>
-      <x:c r="D30" s="4"/>
+      <x:c r="B30" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C30" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">تسوّق من FARFETCH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D30" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بخصم يصل حتى 500 ريال لدى FARFETCH عند الدفع باستخدام أي من بطاقات الإنماء باي فيزا. يسري العرض من 15 يناير وحتى 31 ديسمبر 2026 .</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E30" s="5"/>
-      <x:c r="F30" s="5"/>
-      <x:c r="G30" s="5"/>
+      <x:c r="F30" s="5" t="n">
+        <x:v>46037.0</x:v>
+      </x:c>
+      <x:c r="G30" s="5" t="n">
+        <x:v>46387.0</x:v>
+      </x:c>
       <x:c r="H30" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16700,13 +17748,19 @@
       <x:c r="M30" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N30" s="4"/>
+      <x:c r="N30" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Shop-on-FARFETCH---Jan-2026</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O30" s="4"/>
       <x:c r="P30" s="4"/>
       <x:c r="Q30" s="4"/>
       <x:c r="R30" s="4"/>
       <x:c r="S30" s="4"/>
-      <x:c r="T30" s="5"/>
+      <x:c r="T30" s="5" t="n">
+        <x:v>46259.82478451854</x:v>
+      </x:c>
       <x:c r="U30" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16715,12 +17769,28 @@
       <x:c r="A31" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B31" s="4"/>
-      <x:c r="C31" s="4"/>
-      <x:c r="D31" s="4"/>
+      <x:c r="B31" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C31" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">خصم 20% لدى سيار</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D31" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بخصم 20% لدى سيار (Sayyar) عند الدفع باستخدام بطاقات الإنماء باي . يسري العرض من 1 يناير 2026 حتى 31 ديسمبر 2026 .</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E31" s="5"/>
-      <x:c r="F31" s="5"/>
-      <x:c r="G31" s="5"/>
+      <x:c r="F31" s="5" t="n">
+        <x:v>46023.0</x:v>
+      </x:c>
+      <x:c r="G31" s="5" t="n">
+        <x:v>46387.0</x:v>
+      </x:c>
       <x:c r="H31" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16733,13 +17803,19 @@
       <x:c r="M31" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N31" s="4"/>
+      <x:c r="N31" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Sayyar---April2026</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O31" s="4"/>
       <x:c r="P31" s="4"/>
       <x:c r="Q31" s="4"/>
       <x:c r="R31" s="4"/>
       <x:c r="S31" s="4"/>
-      <x:c r="T31" s="5"/>
+      <x:c r="T31" s="5" t="n">
+        <x:v>46259.741513515</x:v>
+      </x:c>
       <x:c r="U31" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16748,12 +17824,28 @@
       <x:c r="A32" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B32" s="4"/>
-      <x:c r="C32" s="4"/>
-      <x:c r="D32" s="4"/>
+      <x:c r="B32" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C32" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">عرض آيهيرب 40%</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D32" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بخصم 40% على مشترياتك من آيهيرب عند الدفع ببطاقات الإنماء باي فيزا . يسري العرض من 21 أغسطس 2026 حتى 4 سبتمبر 2026 .</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E32" s="5"/>
-      <x:c r="F32" s="5"/>
-      <x:c r="G32" s="5"/>
+      <x:c r="F32" s="5" t="n">
+        <x:v>46255.0</x:v>
+      </x:c>
+      <x:c r="G32" s="5" t="n">
+        <x:v>46269.0</x:v>
+      </x:c>
       <x:c r="H32" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16766,13 +17858,19 @@
       <x:c r="M32" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N32" s="4"/>
+      <x:c r="N32" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/iHerb_Aug_2026</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O32" s="4"/>
       <x:c r="P32" s="4"/>
       <x:c r="Q32" s="4"/>
       <x:c r="R32" s="4"/>
       <x:c r="S32" s="4"/>
-      <x:c r="T32" s="5"/>
+      <x:c r="T32" s="5" t="n">
+        <x:v>46259.82478451854</x:v>
+      </x:c>
       <x:c r="U32" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16781,12 +17879,28 @@
       <x:c r="A33" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B33" s="4"/>
-      <x:c r="C33" s="4"/>
-      <x:c r="D33" s="4"/>
+      <x:c r="B33" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Remittance</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C33" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">عرض اليمن: كاش باك 5 ريال</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D33" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">حوّل إلى اليمن عبر خدمة مباشر الإنماء باي واستمتع بكاش باك 5 ريال بعد إتمام 3 عمليات تحويل. استمتع بكاش باك 5 ريال بعد إتمام 3 عمليات تحويل إلى اليمن عبر خدمة مباشر الإنماء باي.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E33" s="5"/>
-      <x:c r="F33" s="5"/>
-      <x:c r="G33" s="5"/>
+      <x:c r="F33" s="5" t="n">
+        <x:v>46230.0</x:v>
+      </x:c>
+      <x:c r="G33" s="5" t="n">
+        <x:v>46261.0</x:v>
+      </x:c>
       <x:c r="H33" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16799,13 +17913,19 @@
       <x:c r="M33" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N33" s="4"/>
+      <x:c r="N33" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Yemen-Cashback-5SAR</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O33" s="4"/>
       <x:c r="P33" s="4"/>
       <x:c r="Q33" s="4"/>
       <x:c r="R33" s="4"/>
       <x:c r="S33" s="4"/>
-      <x:c r="T33" s="5"/>
+      <x:c r="T33" s="5" t="n">
+        <x:v>46259.82478451854</x:v>
+      </x:c>
       <x:c r="U33" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16814,12 +17934,28 @@
       <x:c r="A34" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B34" s="4"/>
-      <x:c r="C34" s="4"/>
-      <x:c r="D34" s="4"/>
+      <x:c r="B34" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Remittance</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C34" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">عرض رسوم تحويل اليمن 3 ريال</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D34" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بتحويلاتك إلى اليمن برسوم ثابتة 3 ريال فقط عبر خدمة alinmapay Direct ، بدون حد أدنى للتحويل. رسوم تحويل ثابتة بقيمة 3 ريال على التحويلات إلى 🇾🇪 اليمن .</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E34" s="5"/>
-      <x:c r="F34" s="5"/>
-      <x:c r="G34" s="5"/>
+      <x:c r="F34" s="5" t="n">
+        <x:v>46181.0</x:v>
+      </x:c>
+      <x:c r="G34" s="5" t="n">
+        <x:v>46387.0</x:v>
+      </x:c>
       <x:c r="H34" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16832,13 +17968,19 @@
       <x:c r="M34" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N34" s="4"/>
+      <x:c r="N34" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/SAR-3-Transfer-Fee-Yemen-Offer-June26</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O34" s="4"/>
       <x:c r="P34" s="4"/>
       <x:c r="Q34" s="4"/>
       <x:c r="R34" s="4"/>
       <x:c r="S34" s="4"/>
-      <x:c r="T34" s="5"/>
+      <x:c r="T34" s="5" t="n">
+        <x:v>46259.82478451854</x:v>
+      </x:c>
       <x:c r="U34" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16847,12 +17989,28 @@
       <x:c r="A35" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B35" s="4"/>
-      <x:c r="C35" s="4"/>
-      <x:c r="D35" s="4"/>
+      <x:c r="B35" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C35" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">عرض شي إن 20%</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D35" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بخصم 20% على مشترياتك من شي إن عند الدفع ببطاقات الإنماء باي فيزا . يسري العرض من 21 أغسطس 2026 حتى 4 سبتمبر 2026 .</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E35" s="5"/>
-      <x:c r="F35" s="5"/>
-      <x:c r="G35" s="5"/>
+      <x:c r="F35" s="5" t="n">
+        <x:v>46255.0</x:v>
+      </x:c>
+      <x:c r="G35" s="5" t="n">
+        <x:v>46269.0</x:v>
+      </x:c>
       <x:c r="H35" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16865,13 +18023,19 @@
       <x:c r="M35" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N35" s="4"/>
+      <x:c r="N35" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/SHEIN_Aug_2026</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O35" s="4"/>
       <x:c r="P35" s="4"/>
       <x:c r="Q35" s="4"/>
       <x:c r="R35" s="4"/>
       <x:c r="S35" s="4"/>
-      <x:c r="T35" s="5"/>
+      <x:c r="T35" s="5" t="n">
+        <x:v>46259.82478451854</x:v>
+      </x:c>
       <x:c r="U35" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16880,12 +18044,28 @@
       <x:c r="A36" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B36" s="4"/>
-      <x:c r="C36" s="4"/>
-      <x:c r="D36" s="4"/>
+      <x:c r="B36" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C36" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">عين لندن: خصم 15%</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D36" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بخصم 15% لدى عين لندن على التذاكر العادية عند الدفع بأي من بطاقات الإنماء باي فيزا . يسري العرض من 19 أغسطس حتى 30 سبتمبر 2026 .</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E36" s="5"/>
-      <x:c r="F36" s="5"/>
-      <x:c r="G36" s="5"/>
+      <x:c r="F36" s="5" t="n">
+        <x:v>46253.0</x:v>
+      </x:c>
+      <x:c r="G36" s="5" t="n">
+        <x:v>46295.0</x:v>
+      </x:c>
       <x:c r="H36" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16898,13 +18078,19 @@
       <x:c r="M36" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N36" s="4"/>
+      <x:c r="N36" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/LendonEye_2026</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O36" s="4"/>
       <x:c r="P36" s="4"/>
       <x:c r="Q36" s="4"/>
       <x:c r="R36" s="4"/>
       <x:c r="S36" s="4"/>
-      <x:c r="T36" s="5"/>
+      <x:c r="T36" s="5" t="n">
+        <x:v>46259.82478451854</x:v>
+      </x:c>
       <x:c r="U36" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16913,12 +18099,28 @@
       <x:c r="A37" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B37" s="4"/>
-      <x:c r="C37" s="4"/>
-      <x:c r="D37" s="4"/>
+      <x:c r="B37" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C37" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">كيمارت: خصم 70 ريال</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D37" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بخصم يصل حتى 70 ريالاً لدى كيمارت عند الدفع باستخدام أي من بطاقات الإنماء باي كاش باك . حالة العميل (جديد/حالي) تحدد حسب حساب المستخدم في تطبيق كيمارت</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E37" s="5"/>
-      <x:c r="F37" s="5"/>
-      <x:c r="G37" s="5"/>
+      <x:c r="F37" s="5" t="n">
+        <x:v>46254.0</x:v>
+      </x:c>
+      <x:c r="G37" s="5" t="n">
+        <x:v>46276.0</x:v>
+      </x:c>
       <x:c r="H37" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16931,13 +18133,19 @@
       <x:c r="M37" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N37" s="4"/>
+      <x:c r="N37" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Keemart_Aug_2026</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O37" s="4"/>
       <x:c r="P37" s="4"/>
       <x:c r="Q37" s="4"/>
       <x:c r="R37" s="4"/>
       <x:c r="S37" s="4"/>
-      <x:c r="T37" s="5"/>
+      <x:c r="T37" s="5" t="n">
+        <x:v>46259.82478451854</x:v>
+      </x:c>
       <x:c r="U37" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16946,12 +18154,28 @@
       <x:c r="A38" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B38" s="4"/>
-      <x:c r="C38" s="4"/>
-      <x:c r="D38" s="4"/>
+      <x:c r="B38" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C38" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ليجو لاند: خصم 15%</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D38" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بخصم 15% لدى ليجو لاند على تذاكر الدخول ليوم كامل عند الدفع بأي من بطاقات الإنماء باي فيزا . يسري العرض من 19 أغسطس حتى 30 سبتمبر 2026 .</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E38" s="5"/>
-      <x:c r="F38" s="5"/>
-      <x:c r="G38" s="5"/>
+      <x:c r="F38" s="5" t="n">
+        <x:v>46253.0</x:v>
+      </x:c>
+      <x:c r="G38" s="5" t="n">
+        <x:v>46295.0</x:v>
+      </x:c>
       <x:c r="H38" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16964,13 +18188,19 @@
       <x:c r="M38" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N38" s="4"/>
+      <x:c r="N38" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/LegoLand_2026</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O38" s="4"/>
       <x:c r="P38" s="4"/>
       <x:c r="Q38" s="4"/>
       <x:c r="R38" s="4"/>
       <x:c r="S38" s="4"/>
-      <x:c r="T38" s="5"/>
+      <x:c r="T38" s="5" t="n">
+        <x:v>46259.82478451854</x:v>
+      </x:c>
       <x:c r="U38" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16979,12 +18209,28 @@
       <x:c r="A39" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B39" s="4"/>
-      <x:c r="C39" s="4"/>
-      <x:c r="D39" s="4"/>
+      <x:c r="B39" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C39" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">مدام تيسو: خصم 15%</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D39" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">استمتع بخصم 15% لدى مدام تيسو على التذاكر العادية عند الدفع بأي من بطاقات الإنماء باي فيزا . يسري العرض من 19 أغسطس حتى 30 سبتمبر 2026 .</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E39" s="5"/>
-      <x:c r="F39" s="5"/>
-      <x:c r="G39" s="5"/>
+      <x:c r="F39" s="5" t="n">
+        <x:v>46253.0</x:v>
+      </x:c>
+      <x:c r="G39" s="5" t="n">
+        <x:v>46295.0</x:v>
+      </x:c>
       <x:c r="H39" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16997,13 +18243,19 @@
       <x:c r="M39" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N39" s="4"/>
+      <x:c r="N39" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/MADAME-TUSSAUDS_2026</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O39" s="4"/>
       <x:c r="P39" s="4"/>
       <x:c r="Q39" s="4"/>
       <x:c r="R39" s="4"/>
       <x:c r="S39" s="4"/>
-      <x:c r="T39" s="5"/>
+      <x:c r="T39" s="5" t="n">
+        <x:v>46259.82478451854</x:v>
+      </x:c>
       <x:c r="U39" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>

</xml_diff>

<commit_message>
chore: refresh competitor intelligence (stc-bank)
</commit_message>
<xml_diff>
--- a/competitor_campaigns_latest.xlsx
+++ b/competitor_campaigns_latest.xlsx
@@ -5944,7 +5944,7 @@
         </x:is>
       </x:c>
       <x:c r="T9" s="5" t="n">
-        <x:v>46240.0</x:v>
+        <x:v>46260.30139796085</x:v>
       </x:c>
       <x:c r="U9" s="35" t="str">
         <x:f t="shared" ref="U9:U53" si="3">IF(C9="","",IF(COUNTA(O9:R9)=0,"No direct social post verified",IF(O9&lt;&gt;"","Instagram","")&amp;IF(AND(O9&lt;&gt;"",OR(P9&lt;&gt;"",Q9&lt;&gt;"",R9&lt;&gt;"")),", ","")&amp;IF(P9&lt;&gt;"","X","")&amp;IF(AND(P9&lt;&gt;"",OR(Q9&lt;&gt;"",R9&lt;&gt;"")),", ","")&amp;IF(Q9&lt;&gt;"","Facebook","")&amp;IF(AND(Q9&lt;&gt;"",R9&lt;&gt;""),", ","")&amp;IF(R9&lt;&gt;"","TikTok","")))</x:f>
@@ -6173,7 +6173,7 @@
         </x:is>
       </x:c>
       <x:c r="T12" s="5" t="n">
-        <x:v>46240.0</x:v>
+        <x:v>46260.30139796085</x:v>
       </x:c>
       <x:c r="U12" s="35" t="str">
         <x:f t="shared" si="3">IF(C12="","",IF(COUNTA(O12:R12)=0,"No direct social post verified",IF(O12&lt;&gt;"","Instagram","")&amp;IF(AND(O12&lt;&gt;"",OR(P12&lt;&gt;"",Q12&lt;&gt;"",R12&lt;&gt;"")),", ","")&amp;IF(P12&lt;&gt;"","X","")&amp;IF(AND(P12&lt;&gt;"",OR(Q12&lt;&gt;"",R12&lt;&gt;"")),", ","")&amp;IF(Q12&lt;&gt;"","Facebook","")&amp;IF(AND(Q12&lt;&gt;"",R12&lt;&gt;""),", ","")&amp;IF(R12&lt;&gt;"","TikTok","")))</x:f>
@@ -6471,7 +6471,7 @@
         </x:is>
       </x:c>
       <x:c r="T16" s="5" t="n">
-        <x:v>46240.0</x:v>
+        <x:v>46260.30139796085</x:v>
       </x:c>
       <x:c r="U16" s="35" t="str">
         <x:f t="shared" si="3">IF(C16="","",IF(COUNTA(O16:R16)=0,"No direct social post verified",IF(O16&lt;&gt;"","Instagram","")&amp;IF(AND(O16&lt;&gt;"",OR(P16&lt;&gt;"",Q16&lt;&gt;"",R16&lt;&gt;"")),", ","")&amp;IF(P16&lt;&gt;"","X","")&amp;IF(AND(P16&lt;&gt;"",OR(Q16&lt;&gt;"",R16&lt;&gt;"")),", ","")&amp;IF(Q16&lt;&gt;"","Facebook","")&amp;IF(AND(Q16&lt;&gt;"",R16&lt;&gt;""),", ","")&amp;IF(R16&lt;&gt;"","TikTok","")))</x:f>
@@ -6545,7 +6545,7 @@
         </x:is>
       </x:c>
       <x:c r="T17" s="5" t="n">
-        <x:v>46240.0</x:v>
+        <x:v>46260.30139796085</x:v>
       </x:c>
       <x:c r="U17" s="35" t="str">
         <x:f t="shared" si="3">IF(C17="","",IF(COUNTA(O17:R17)=0,"No direct social post verified",IF(O17&lt;&gt;"","Instagram","")&amp;IF(AND(O17&lt;&gt;"",OR(P17&lt;&gt;"",Q17&lt;&gt;"",R17&lt;&gt;"")),", ","")&amp;IF(P17&lt;&gt;"","X","")&amp;IF(AND(P17&lt;&gt;"",OR(Q17&lt;&gt;"",R17&lt;&gt;"")),", ","")&amp;IF(Q17&lt;&gt;"","Facebook","")&amp;IF(AND(Q17&lt;&gt;"",R17&lt;&gt;""),", ","")&amp;IF(R17&lt;&gt;"","TikTok","")))</x:f>
@@ -6619,7 +6619,7 @@
         </x:is>
       </x:c>
       <x:c r="T18" s="5" t="n">
-        <x:v>46240.0</x:v>
+        <x:v>46260.30139796085</x:v>
       </x:c>
       <x:c r="U18" s="35" t="str">
         <x:f t="shared" si="3">IF(C18="","",IF(COUNTA(O18:R18)=0,"No direct social post verified",IF(O18&lt;&gt;"","Instagram","")&amp;IF(AND(O18&lt;&gt;"",OR(P18&lt;&gt;"",Q18&lt;&gt;"",R18&lt;&gt;"")),", ","")&amp;IF(P18&lt;&gt;"","X","")&amp;IF(AND(P18&lt;&gt;"",OR(Q18&lt;&gt;"",R18&lt;&gt;"")),", ","")&amp;IF(Q18&lt;&gt;"","Facebook","")&amp;IF(AND(Q18&lt;&gt;"",R18&lt;&gt;""),", ","")&amp;IF(R18&lt;&gt;"","TikTok","")))</x:f>
@@ -6693,7 +6693,7 @@
         </x:is>
       </x:c>
       <x:c r="T19" s="5" t="n">
-        <x:v>46240.0</x:v>
+        <x:v>46260.30139796085</x:v>
       </x:c>
       <x:c r="U19" s="35" t="str">
         <x:f t="shared" si="3">IF(C19="","",IF(COUNTA(O19:R19)=0,"No direct social post verified",IF(O19&lt;&gt;"","Instagram","")&amp;IF(AND(O19&lt;&gt;"",OR(P19&lt;&gt;"",Q19&lt;&gt;"",R19&lt;&gt;"")),", ","")&amp;IF(P19&lt;&gt;"","X","")&amp;IF(AND(P19&lt;&gt;"",OR(Q19&lt;&gt;"",R19&lt;&gt;"")),", ","")&amp;IF(Q19&lt;&gt;"","Facebook","")&amp;IF(AND(Q19&lt;&gt;"",R19&lt;&gt;""),", ","")&amp;IF(R19&lt;&gt;"","TikTok","")))</x:f>
@@ -6767,7 +6767,7 @@
         </x:is>
       </x:c>
       <x:c r="T20" s="5" t="n">
-        <x:v>46240.0</x:v>
+        <x:v>46260.30139796085</x:v>
       </x:c>
       <x:c r="U20" s="35" t="str">
         <x:f t="shared" si="3">IF(C20="","",IF(COUNTA(O20:R20)=0,"No direct social post verified",IF(O20&lt;&gt;"","Instagram","")&amp;IF(AND(O20&lt;&gt;"",OR(P20&lt;&gt;"",Q20&lt;&gt;"",R20&lt;&gt;"")),", ","")&amp;IF(P20&lt;&gt;"","X","")&amp;IF(AND(P20&lt;&gt;"",OR(Q20&lt;&gt;"",R20&lt;&gt;"")),", ","")&amp;IF(Q20&lt;&gt;"","Facebook","")&amp;IF(AND(Q20&lt;&gt;"",R20&lt;&gt;""),", ","")&amp;IF(R20&lt;&gt;"","TikTok","")))</x:f>
@@ -6841,7 +6841,7 @@
         </x:is>
       </x:c>
       <x:c r="T21" s="5" t="n">
-        <x:v>46240.0</x:v>
+        <x:v>46260.30139796085</x:v>
       </x:c>
       <x:c r="U21" s="35" t="str">
         <x:f t="shared" si="3">IF(C21="","",IF(COUNTA(O21:R21)=0,"No direct social post verified",IF(O21&lt;&gt;"","Instagram","")&amp;IF(AND(O21&lt;&gt;"",OR(P21&lt;&gt;"",Q21&lt;&gt;"",R21&lt;&gt;"")),", ","")&amp;IF(P21&lt;&gt;"","X","")&amp;IF(AND(P21&lt;&gt;"",OR(Q21&lt;&gt;"",R21&lt;&gt;"")),", ","")&amp;IF(Q21&lt;&gt;"","Facebook","")&amp;IF(AND(Q21&lt;&gt;"",R21&lt;&gt;""),", ","")&amp;IF(R21&lt;&gt;"","TikTok","")))</x:f>
@@ -7007,7 +7007,7 @@
         </x:is>
       </x:c>
       <x:c r="T23" s="5" t="n">
-        <x:v>46240.0</x:v>
+        <x:v>46260.30139796085</x:v>
       </x:c>
       <x:c r="U23" s="35" t="str">
         <x:f t="shared" si="3">IF(C23="","",IF(COUNTA(O23:R23)=0,"No direct social post verified",IF(O23&lt;&gt;"","Instagram","")&amp;IF(AND(O23&lt;&gt;"",OR(P23&lt;&gt;"",Q23&lt;&gt;"",R23&lt;&gt;"")),", ","")&amp;IF(P23&lt;&gt;"","X","")&amp;IF(AND(P23&lt;&gt;"",OR(Q23&lt;&gt;"",R23&lt;&gt;"")),", ","")&amp;IF(Q23&lt;&gt;"","Facebook","")&amp;IF(AND(Q23&lt;&gt;"",R23&lt;&gt;""),", ","")&amp;IF(R23&lt;&gt;"","TikTok","")))</x:f>
@@ -7019,12 +7019,26 @@
         <x:f t="shared" si="0">IF(C24="","",ROW()-8)</x:f>
         <x:v>16</x:v>
       </x:c>
-      <x:c r="B24" s="4"/>
-      <x:c r="C24" s="4"/>
-      <x:c r="D24" s="4"/>
+      <x:c r="B24" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Merchant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C24" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Polish and protect your car with a 20% discount from Dettaglioauto!</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D24" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Enjoy a 20% discount at Dettaglioauto branches around KSA, using any STC Bank card.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E24" s="5"/>
       <x:c r="F24" s="5"/>
-      <x:c r="G24" s="5"/>
+      <x:c r="G24" s="5" t="n">
+        <x:v>46314.0</x:v>
+      </x:c>
       <x:c r="H24" s="7" t="n">
         <x:f t="shared" si="1">IF(OR(C24="",G24=""),"",G24-TODAY())</x:f>
         <x:v>57</x:v>
@@ -7040,13 +7054,19 @@
         <x:f t="shared" si="4">IF(C24="","",IF(N24&lt;&gt;"",N24,IF(O24&lt;&gt;"",O24,IF(P24&lt;&gt;"",P24,IF(Q24&lt;&gt;"",Q24,IF(R24&lt;&gt;"",R24,""))))))</x:f>
         <x:v>https://stcbank.com.sa/en/web/guest/w/blt-cash</x:v>
       </x:c>
-      <x:c r="N24" s="4"/>
+      <x:c r="N24" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/dettaglioauto-offer</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O24" s="4"/>
       <x:c r="P24" s="4"/>
       <x:c r="Q24" s="4"/>
       <x:c r="R24" s="4"/>
       <x:c r="S24" s="4"/>
-      <x:c r="T24" s="5"/>
+      <x:c r="T24" s="5" t="n">
+        <x:v>46260.30139796085</x:v>
+      </x:c>
       <x:c r="U24" s="35" t="str">
         <x:f t="shared" si="3">IF(C24="","",IF(COUNTA(O24:R24)=0,"No direct social post verified",IF(O24&lt;&gt;"","Instagram","")&amp;IF(AND(O24&lt;&gt;"",OR(P24&lt;&gt;"",Q24&lt;&gt;"",R24&lt;&gt;"")),", ","")&amp;IF(P24&lt;&gt;"","X","")&amp;IF(AND(P24&lt;&gt;"",OR(Q24&lt;&gt;"",R24&lt;&gt;"")),", ","")&amp;IF(Q24&lt;&gt;"","Facebook","")&amp;IF(AND(Q24&lt;&gt;"",R24&lt;&gt;""),", ","")&amp;IF(R24&lt;&gt;"","TikTok","")))</x:f>
         <x:v>No direct social post verified</x:v>
@@ -7056,12 +7076,26 @@
       <x:c r="A25" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B25" s="4"/>
-      <x:c r="C25" s="4"/>
-      <x:c r="D25" s="4"/>
+      <x:c r="B25" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Remittance</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C25" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Transfer internationally and enter the draw</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D25" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Make an international transfer of any amount to any country through the app and get a chance to enter the draw to win a car every week and ⃁ 1,000 for 10 winners daily.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E25" s="5"/>
       <x:c r="F25" s="5"/>
-      <x:c r="G25" s="5"/>
+      <x:c r="G25" s="5" t="n">
+        <x:v>46314.0</x:v>
+      </x:c>
       <x:c r="H25" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -7074,13 +7108,23 @@
       <x:c r="M25" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N25" s="4"/>
+      <x:c r="N25" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://stcbank.com.sa/en/web/guest/w/transfer-internationally-and-enter-the-draw</x:t>
+        </x:is>
+      </x:c>
       <x:c r="O25" s="4"/>
       <x:c r="P25" s="4"/>
-      <x:c r="Q25" s="4"/>
+      <x:c r="Q25" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">https://m.facebook.com/stcbank/posts/pfbid0A7CQGcMTqxF47NMhKYT4TXgNUycHgbn27me4FwmVPMf8EU6wCZ922d62Pnq19ZYrl</x:t>
+        </x:is>
+      </x:c>
       <x:c r="R25" s="4"/>
       <x:c r="S25" s="4"/>
-      <x:c r="T25" s="5"/>
+      <x:c r="T25" s="5" t="n">
+        <x:v>46260.30139796085</x:v>
+      </x:c>
       <x:c r="U25" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -8738,21 +8782,9 @@
       <x:c r="A15" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B15" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C15" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Crazy Pizza offer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D15" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Terms and Conditions Offer • Enjoy a 20% discount at Crazy Pizza Tahlia, Oud Square, north yard and Khobar when paying with barq Visa cards.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B15" s="4"/>
+      <x:c r="C15" s="4"/>
+      <x:c r="D15" s="4"/>
       <x:c r="E15" s="5"/>
       <x:c r="F15" s="5"/>
       <x:c r="G15" s="5"/>
@@ -8768,19 +8800,13 @@
       <x:c r="M15" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N15" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://barq.com/offers/crazy-pizza/</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N15" s="4"/>
       <x:c r="O15" s="4"/>
       <x:c r="P15" s="4"/>
       <x:c r="Q15" s="4"/>
       <x:c r="R15" s="4"/>
       <x:c r="S15" s="4"/>
-      <x:c r="T15" s="5" t="n">
-        <x:v>46260.08078116647</x:v>
-      </x:c>
+      <x:c r="T15" s="5"/>
       <x:c r="U15" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -8789,25 +8815,11 @@
       <x:c r="A16" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B16" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Other</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C16" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">حملة الصيف \ مارثون برق</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D16" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">تستمر الحملة لمدة تسعة و اربعون (49) يومًا تقويميًا. الأسبوع الأول: ابتداءً من يوم الاحد 24 مايو 2026 الساعة 12:00 مساءً وحتى يوم الاحد 31 مايو 2026 الساعة 11:00 مساءً.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B16" s="4"/>
+      <x:c r="C16" s="4"/>
+      <x:c r="D16" s="4"/>
       <x:c r="E16" s="5"/>
-      <x:c r="F16" s="5" t="n">
-        <x:v>46166.0</x:v>
-      </x:c>
+      <x:c r="F16" s="5"/>
       <x:c r="G16" s="5"/>
       <x:c r="H16" s="7" t="str">
         <x:f t="shared" si="1"/>
@@ -8821,19 +8833,13 @@
       <x:c r="M16" s="9" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
-      <x:c r="N16" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://barq.com/ar/offers/%d8%ad%d9%85%d9%84%d8%a9-%d8%a7%d9%84%d8%b5%d9%8a%d9%81/</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N16" s="4"/>
       <x:c r="O16" s="4"/>
       <x:c r="P16" s="4"/>
       <x:c r="Q16" s="4"/>
       <x:c r="R16" s="4"/>
       <x:c r="S16" s="4"/>
-      <x:c r="T16" s="5" t="n">
-        <x:v>46260.29939116185</x:v>
-      </x:c>
+      <x:c r="T16" s="5"/>
       <x:c r="U16" s="35" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
@@ -10139,7 +10145,7 @@
         </x:is>
       </x:c>
       <x:c r="T10" s="5" t="n">
-        <x:v>46260.11321182853</x:v>
+        <x:v>46240.0</x:v>
       </x:c>
       <x:c r="U10" s="35" t="str">
         <x:f t="shared" si="4">IF(C10="","",IF(COUNTA(O10:R10)=0,"No direct social post verified",IF(O10&lt;&gt;"","Instagram","")&amp;IF(AND(O10&lt;&gt;"",OR(P10&lt;&gt;"",Q10&lt;&gt;"",R10&lt;&gt;"")),", ","")&amp;IF(P10&lt;&gt;"","X","")&amp;IF(AND(P10&lt;&gt;"",OR(Q10&lt;&gt;"",R10&lt;&gt;"")),", ","")&amp;IF(Q10&lt;&gt;"","Facebook","")&amp;IF(AND(Q10&lt;&gt;"",R10&lt;&gt;""),", ","")&amp;IF(R10&lt;&gt;"","TikTok","")))</x:f>
@@ -10469,28 +10475,12 @@
       <x:c r="A15" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B15" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Other</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C15" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10 SAR CASHBACK</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D15" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">The offer is valid from 5 Jan until 30 Aug 2026. Share your promo code with your friends to get SAR 5 Cashback, and them get SAR 5 Cashback.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B15" s="4"/>
+      <x:c r="C15" s="4"/>
+      <x:c r="D15" s="4"/>
       <x:c r="E15" s="5"/>
-      <x:c r="F15" s="5" t="n">
-        <x:v>46027.0</x:v>
-      </x:c>
-      <x:c r="G15" s="5" t="n">
-        <x:v>46264.0</x:v>
-      </x:c>
+      <x:c r="F15" s="5"/>
+      <x:c r="G15" s="5"/>
       <x:c r="H15" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -10503,19 +10493,13 @@
       <x:c r="M15" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N15" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-26.html</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N15" s="4"/>
       <x:c r="O15" s="4"/>
       <x:c r="P15" s="4"/>
       <x:c r="Q15" s="4"/>
       <x:c r="R15" s="4"/>
       <x:c r="S15" s="4"/>
-      <x:c r="T15" s="5" t="n">
-        <x:v>46260.20266816726</x:v>
-      </x:c>
+      <x:c r="T15" s="5"/>
       <x:c r="U15" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -10524,28 +10508,12 @@
       <x:c r="A16" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B16" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C16" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">AL MABAT HOTEL</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D16" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Offer is valid from 10 July 2025 to 30 Nov 2026. 15% discount with no limit on your full hotel experience — buffet service excluded.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B16" s="4"/>
+      <x:c r="C16" s="4"/>
+      <x:c r="D16" s="4"/>
       <x:c r="E16" s="5"/>
-      <x:c r="F16" s="5" t="n">
-        <x:v>45848.0</x:v>
-      </x:c>
-      <x:c r="G16" s="5" t="n">
-        <x:v>46356.0</x:v>
-      </x:c>
+      <x:c r="F16" s="5"/>
+      <x:c r="G16" s="5"/>
       <x:c r="H16" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -10558,19 +10526,13 @@
       <x:c r="M16" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N16" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/en/offers/offer-13.html</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N16" s="4"/>
       <x:c r="O16" s="4"/>
       <x:c r="P16" s="4"/>
       <x:c r="Q16" s="4"/>
       <x:c r="R16" s="4"/>
       <x:c r="S16" s="4"/>
-      <x:c r="T16" s="5" t="n">
-        <x:v>46260.20266816726</x:v>
-      </x:c>
+      <x:c r="T16" s="5"/>
       <x:c r="U16" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -10579,28 +10541,12 @@
       <x:c r="A17" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B17" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Other</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C17" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">EARN MILES WITH ALL MOBILY PAY SERVICES</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D17" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Offer is valid from 1 Feb 2025 until 30 Sep 2026. Offer includes only the services specified in the Miles Earning Schedule when using Mobily Pay App</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B17" s="4"/>
+      <x:c r="C17" s="4"/>
+      <x:c r="D17" s="4"/>
       <x:c r="E17" s="5"/>
-      <x:c r="F17" s="5" t="n">
-        <x:v>45689.0</x:v>
-      </x:c>
-      <x:c r="G17" s="5" t="n">
-        <x:v>46295.0</x:v>
-      </x:c>
+      <x:c r="F17" s="5"/>
+      <x:c r="G17" s="5"/>
       <x:c r="H17" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -10613,19 +10559,13 @@
       <x:c r="M17" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N17" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-7.html</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N17" s="4"/>
       <x:c r="O17" s="4"/>
       <x:c r="P17" s="4"/>
       <x:c r="Q17" s="4"/>
       <x:c r="R17" s="4"/>
       <x:c r="S17" s="4"/>
-      <x:c r="T17" s="5" t="n">
-        <x:v>46260.20266816726</x:v>
-      </x:c>
+      <x:c r="T17" s="5"/>
       <x:c r="U17" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -10634,28 +10574,12 @@
       <x:c r="A18" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B18" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C18" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">FANOS LIGHTING</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D18" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Offer is valid from 22 Oct 2025 until 20 Oct 2026. 12% discount without limit on all products except establishment products.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B18" s="4"/>
+      <x:c r="C18" s="4"/>
+      <x:c r="D18" s="4"/>
       <x:c r="E18" s="5"/>
-      <x:c r="F18" s="5" t="n">
-        <x:v>45952.0</x:v>
-      </x:c>
-      <x:c r="G18" s="5" t="n">
-        <x:v>46315.0</x:v>
-      </x:c>
+      <x:c r="F18" s="5"/>
+      <x:c r="G18" s="5"/>
       <x:c r="H18" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -10668,19 +10592,13 @@
       <x:c r="M18" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N18" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/en/offers/offer-19.html</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N18" s="4"/>
       <x:c r="O18" s="4"/>
       <x:c r="P18" s="4"/>
       <x:c r="Q18" s="4"/>
       <x:c r="R18" s="4"/>
       <x:c r="S18" s="4"/>
-      <x:c r="T18" s="5" t="n">
-        <x:v>46260.20266816726</x:v>
-      </x:c>
+      <x:c r="T18" s="5"/>
       <x:c r="U18" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -10689,25 +10607,11 @@
       <x:c r="A19" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B19" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Remittance</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C19" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">INTERNATIONAL TRANSFER TO PAKISTAN IS FREE</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D19" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Offer is valid from 8 Nov 2023 No fees are applied to international transfers to bank accounts or digital wallets in Pakistan.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B19" s="4"/>
+      <x:c r="C19" s="4"/>
+      <x:c r="D19" s="4"/>
       <x:c r="E19" s="5"/>
-      <x:c r="F19" s="5" t="n">
-        <x:v>45238.0</x:v>
-      </x:c>
+      <x:c r="F19" s="5"/>
       <x:c r="G19" s="5"/>
       <x:c r="H19" s="7" t="str">
         <x:f t="shared" si="1"/>
@@ -10721,19 +10625,13 @@
       <x:c r="M19" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N19" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-2.html</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N19" s="4"/>
       <x:c r="O19" s="4"/>
       <x:c r="P19" s="4"/>
       <x:c r="Q19" s="4"/>
       <x:c r="R19" s="4"/>
       <x:c r="S19" s="4"/>
-      <x:c r="T19" s="5" t="n">
-        <x:v>46260.24731988846</x:v>
-      </x:c>
+      <x:c r="T19" s="5"/>
       <x:c r="U19" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -10742,28 +10640,12 @@
       <x:c r="A20" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B20" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C20" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Maintaining your car is easier with MisMar</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D20" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Offer is valid from 12 May 2025 until 10 May 2027. 75% discount with no minimum on maintenance and malfunction service fees.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B20" s="4"/>
+      <x:c r="C20" s="4"/>
+      <x:c r="D20" s="4"/>
       <x:c r="E20" s="5"/>
-      <x:c r="F20" s="5" t="n">
-        <x:v>45789.0</x:v>
-      </x:c>
-      <x:c r="G20" s="5" t="n">
-        <x:v>46517.0</x:v>
-      </x:c>
+      <x:c r="F20" s="5"/>
+      <x:c r="G20" s="5"/>
       <x:c r="H20" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -10776,19 +10658,13 @@
       <x:c r="M20" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N20" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/en/offers/offer-9.html</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N20" s="4"/>
       <x:c r="O20" s="4"/>
       <x:c r="P20" s="4"/>
       <x:c r="Q20" s="4"/>
       <x:c r="R20" s="4"/>
       <x:c r="S20" s="4"/>
-      <x:c r="T20" s="5" t="n">
-        <x:v>46260.24731988846</x:v>
-      </x:c>
+      <x:c r="T20" s="5"/>
       <x:c r="U20" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -10797,28 +10673,12 @@
       <x:c r="A21" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B21" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C21" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">RASEEL GIFT</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D21" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Offer valid from 15 Oct 2025 until 14 Oct 2026 30% Discount on the first order, up to a maximum of 100 SAR when using promo code MPay30 , The offer can be used once per customer.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B21" s="4"/>
+      <x:c r="C21" s="4"/>
+      <x:c r="D21" s="4"/>
       <x:c r="E21" s="5"/>
-      <x:c r="F21" s="5" t="n">
-        <x:v>45945.0</x:v>
-      </x:c>
-      <x:c r="G21" s="5" t="n">
-        <x:v>46309.0</x:v>
-      </x:c>
+      <x:c r="F21" s="5"/>
+      <x:c r="G21" s="5"/>
       <x:c r="H21" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -10831,19 +10691,13 @@
       <x:c r="M21" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N21" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/en/offers/offer-18.html</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N21" s="4"/>
       <x:c r="O21" s="4"/>
       <x:c r="P21" s="4"/>
       <x:c r="Q21" s="4"/>
       <x:c r="R21" s="4"/>
       <x:c r="S21" s="4"/>
-      <x:c r="T21" s="5" t="n">
-        <x:v>46260.21978412851</x:v>
-      </x:c>
+      <x:c r="T21" s="5"/>
       <x:c r="U21" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -10852,28 +10706,12 @@
       <x:c r="A22" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B22" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C22" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SWEATER</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D22" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Offer valid from 26 Oct 2025 until 30 Dec 2026 40% discount on single wash only from 9:00 AM to 2 PM when using promo code MobilyPay40</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B22" s="4"/>
+      <x:c r="C22" s="4"/>
+      <x:c r="D22" s="4"/>
       <x:c r="E22" s="5"/>
-      <x:c r="F22" s="5" t="n">
-        <x:v>45956.0</x:v>
-      </x:c>
-      <x:c r="G22" s="5" t="n">
-        <x:v>46386.0</x:v>
-      </x:c>
+      <x:c r="F22" s="5"/>
+      <x:c r="G22" s="5"/>
       <x:c r="H22" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -10886,19 +10724,13 @@
       <x:c r="M22" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N22" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/en/offers/offer-20.html</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N22" s="4"/>
       <x:c r="O22" s="4"/>
       <x:c r="P22" s="4"/>
       <x:c r="Q22" s="4"/>
       <x:c r="R22" s="4"/>
       <x:c r="S22" s="4"/>
-      <x:c r="T22" s="5" t="n">
-        <x:v>46260.20266816726</x:v>
-      </x:c>
+      <x:c r="T22" s="5"/>
       <x:c r="U22" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -10907,28 +10739,12 @@
       <x:c r="A23" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B23" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Other</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C23" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Trips For hotel and flight reservations</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D23" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Offer is valid from 16 Aug until 31 Aug 2026. 5% discount on hotels and 5% cashback on domestic and international airlines with no maximum discount or cashback.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B23" s="4"/>
+      <x:c r="C23" s="4"/>
+      <x:c r="D23" s="4"/>
       <x:c r="E23" s="5"/>
-      <x:c r="F23" s="5" t="n">
-        <x:v>46250.0</x:v>
-      </x:c>
-      <x:c r="G23" s="5" t="n">
-        <x:v>46265.0</x:v>
-      </x:c>
+      <x:c r="F23" s="5"/>
+      <x:c r="G23" s="5"/>
       <x:c r="H23" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -10941,19 +10757,13 @@
       <x:c r="M23" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N23" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-57.html</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N23" s="4"/>
       <x:c r="O23" s="4"/>
       <x:c r="P23" s="4"/>
       <x:c r="Q23" s="4"/>
       <x:c r="R23" s="4"/>
       <x:c r="S23" s="4"/>
-      <x:c r="T23" s="5" t="n">
-        <x:v>46260.20266816726</x:v>
-      </x:c>
+      <x:c r="T23" s="5"/>
       <x:c r="U23" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -10962,28 +10772,12 @@
       <x:c r="A24" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B24" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C24" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Vogacloset</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D24" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Offer valid from 19 April to 30 September 2026. Offer is valid on all purchases when using a Mobily Pay card (Platinum &amp; Signature) with promo code "VISA10".</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B24" s="4"/>
+      <x:c r="C24" s="4"/>
+      <x:c r="D24" s="4"/>
       <x:c r="E24" s="5"/>
-      <x:c r="F24" s="5" t="n">
-        <x:v>46131.0</x:v>
-      </x:c>
-      <x:c r="G24" s="5" t="n">
-        <x:v>46295.0</x:v>
-      </x:c>
+      <x:c r="F24" s="5"/>
+      <x:c r="G24" s="5"/>
       <x:c r="H24" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -10996,19 +10790,13 @@
       <x:c r="M24" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N24" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/en/offers/offer-49.html</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N24" s="4"/>
       <x:c r="O24" s="4"/>
       <x:c r="P24" s="4"/>
       <x:c r="Q24" s="4"/>
       <x:c r="R24" s="4"/>
       <x:c r="S24" s="4"/>
-      <x:c r="T24" s="5" t="n">
-        <x:v>46260.20266816726</x:v>
-      </x:c>
+      <x:c r="T24" s="5"/>
       <x:c r="U24" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -11017,28 +10805,12 @@
       <x:c r="A25" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B25" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C25" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">أيهيرب</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D25" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">يسري العرض من 1 أبريل حتى 30 سبتمبر 2026. احصل على خصم %25 على أول طلب لك من أيهيرب، أو خصم %10 إذا كنت عميلاً حالياً.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B25" s="4"/>
+      <x:c r="C25" s="4"/>
+      <x:c r="D25" s="4"/>
       <x:c r="E25" s="5"/>
-      <x:c r="F25" s="5" t="n">
-        <x:v>46113.0</x:v>
-      </x:c>
-      <x:c r="G25" s="5" t="n">
-        <x:v>46295.0</x:v>
-      </x:c>
+      <x:c r="F25" s="5"/>
+      <x:c r="G25" s="5"/>
       <x:c r="H25" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -11051,19 +10823,13 @@
       <x:c r="M25" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N25" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://mobilypay.sa/ar/offers/offer-50.html</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N25" s="4"/>
       <x:c r="O25" s="4"/>
       <x:c r="P25" s="4"/>
       <x:c r="Q25" s="4"/>
       <x:c r="R25" s="4"/>
       <x:c r="S25" s="4"/>
-      <x:c r="T25" s="5" t="n">
-        <x:v>46260.11321182853</x:v>
-      </x:c>
+      <x:c r="T25" s="5"/>
       <x:c r="U25" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -15994,28 +15760,12 @@
       <x:c r="A14" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B14" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C14" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء رائعة بخصم 20% في اجو</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D14" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء رائعة بخصم 20% في اجو الشروط والأحكام: • استمتع بأجواء رائعة في اجو واستمتع بخصم 20% عند الدفع باستخدام بطاقات الكاش باك من الإنماء باي. • يسري العرض من 7 ديسمبر 2025 و حتى 20 نوفمبر 2026. • خصم 20% عند الدفع باستخدام بطاقات الكاش باك للإنماء باي خلال الفترة المشار إليها على جميع الطلبات من قائمة الطعام الانتقائية ولا يسري على قائمة الطعام المجهز مسبقاً ( Set Menu) • يسري العرض من الاحد الى الخميس من الساعة 1 م الى الساعة 6 م. • العرض لا يشمل تطبيقات التوصيل. • الخصم يشمل الفروع داخل السعودية في الرياض • لا يطبق العرض مع اي عروض اخرى ولا يمكن الجمع بين اكثر من عرض في نفس الوقت. • لا يسري العرض مع ايام المناسبات والاعياد والاجازات الرسمية مثال (اليوم الوطني – يوم التأسيس – ويوم </x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B14" s="4"/>
+      <x:c r="C14" s="4"/>
+      <x:c r="D14" s="4"/>
       <x:c r="E14" s="5"/>
-      <x:c r="F14" s="5" t="n">
-        <x:v>45998.0</x:v>
-      </x:c>
-      <x:c r="G14" s="5" t="n">
-        <x:v>46346.0</x:v>
-      </x:c>
+      <x:c r="F14" s="5"/>
+      <x:c r="G14" s="5"/>
       <x:c r="H14" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16028,19 +15778,13 @@
       <x:c r="M14" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N14" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Agio-dec25</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N14" s="4"/>
       <x:c r="O14" s="4"/>
       <x:c r="P14" s="4"/>
       <x:c r="Q14" s="4"/>
       <x:c r="R14" s="4"/>
       <x:c r="S14" s="4"/>
-      <x:c r="T14" s="5" t="n">
-        <x:v>46260.29939116185</x:v>
-      </x:c>
+      <x:c r="T14" s="5"/>
       <x:c r="U14" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16049,28 +15793,12 @@
       <x:c r="A15" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B15" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C15" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء رائعة واحصل على خصم 15% في أيرث كافيه</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D15" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء رائعة واحصل على خصم 15% في أيرث كافيه الشروط والأحكام : • استمتع بأجواء رائعة في أيرث كافيه وحصل على خصم 15% عند الدفع باستخدام ب طاقات الكاش باك للإنماء باي • يسري العرض حتى 20-11-2026. • خصم 15% عند الدفع باستخدام بطاقات الكاش باي للإنماء خلال الفترة المشار إليها على جميع الطلبات من قائمة الطعام الانتقائية ولا يسري على قائمة الطعام المجهز مسبقاً ( Set Menu) • يسري العرض من الاحد الى الخميس من الساعة 7 ص الى الساعة 6 م. • العرض لا يشمل تطبيقات التوصيل. • الخصم يشمل الفروع داخل السعودية في الرياض و جدة و الخبر . • لا يطبق العرض مع اي عروض اخرى ولا يمكن الجمع بين اكثر من عرض في نفس الوقت. • لا يسري العرض مع ايام المناسبات والاعياد والاجازات الرسمية مثال (اليوم الوطني – يوم التأس</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B15" s="4"/>
+      <x:c r="C15" s="4"/>
+      <x:c r="D15" s="4"/>
       <x:c r="E15" s="5"/>
-      <x:c r="F15" s="5" t="n">
-        <x:v>45998.0</x:v>
-      </x:c>
-      <x:c r="G15" s="5" t="n">
-        <x:v>46346.0</x:v>
-      </x:c>
+      <x:c r="F15" s="5"/>
+      <x:c r="G15" s="5"/>
       <x:c r="H15" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16083,19 +15811,13 @@
       <x:c r="M15" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N15" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Urth-Cafe-dec25</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N15" s="4"/>
       <x:c r="O15" s="4"/>
       <x:c r="P15" s="4"/>
       <x:c r="Q15" s="4"/>
       <x:c r="R15" s="4"/>
       <x:c r="S15" s="4"/>
-      <x:c r="T15" s="5" t="n">
-        <x:v>46260.29939116185</x:v>
-      </x:c>
+      <x:c r="T15" s="5"/>
       <x:c r="U15" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16104,28 +15826,12 @@
       <x:c r="A16" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B16" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C16" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء رائعة واستمتع بخصم 20% في بيف بار</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D16" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء رائعة واستمتع بخصم 20% في بيف بار الشروط والأحكام: • استمتع بأجواء رائعة في بيف بار واستمتع بخصم 20% عند الدفع باستخدام بطاقات الكاش باك من الإنماء باي • يسري العرض من 7 ديسمبر 2025 و حتى 20 نوفمبر 2026. • خصم 20% عند الدفع باستخدام بطاقات الكاش باك للإنماء باي خلال الفترة المشار إليها على جميع الطلبات من قائمة الطعام الانتقائية ولا يسري على قائمة الطعام المجهز مسبقاً ( Set Menu) • يسري العرض من الاحد الى الخميس من الساعة 1 م الى الساعة 6 م. • العرض لا يشمل تطبيقات التوصيل. • الخصم يشمل الفروع داخل السعودية في الرياض • لا يطبق العرض مع اي عروض اخرى ولا يمكن الجمع بين اكثر من عرض في نفس الوقت. • لا يسري العرض مع ايام المناسبات والاعياد والاجازات الرسمية مثال (اليوم الوطني – يوم </x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B16" s="4"/>
+      <x:c r="C16" s="4"/>
+      <x:c r="D16" s="4"/>
       <x:c r="E16" s="5"/>
-      <x:c r="F16" s="5" t="n">
-        <x:v>45998.0</x:v>
-      </x:c>
-      <x:c r="G16" s="5" t="n">
-        <x:v>46346.0</x:v>
-      </x:c>
+      <x:c r="F16" s="5"/>
+      <x:c r="G16" s="5"/>
       <x:c r="H16" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16138,19 +15844,13 @@
       <x:c r="M16" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N16" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Beefbar-dec25</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N16" s="4"/>
       <x:c r="O16" s="4"/>
       <x:c r="P16" s="4"/>
       <x:c r="Q16" s="4"/>
       <x:c r="R16" s="4"/>
       <x:c r="S16" s="4"/>
-      <x:c r="T16" s="5" t="n">
-        <x:v>46260.29939116185</x:v>
-      </x:c>
+      <x:c r="T16" s="5"/>
       <x:c r="U16" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16159,28 +15859,12 @@
       <x:c r="A17" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B17" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C17" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء رائعة واستمتع بخصم 20% في روباتا</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D17" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء رائعة واستمتع بخصم 20% في روباتا الشروط والأحكام: • استمتع بأجواء رائعة في روباتا واستمتع بخصم 20% عند الدفع باستخدام بطاقات الكاش باك من الإنماء باي. • يسري العرض من 7 ديسمبر 2025 و حتى 20 نوفمبر 2026. • خصم 20% عند الدفع باستخدام بطاقات الكاش باك للإنماء باي خلال الفترة المشار إليها على جميع الطلبات من قائمة الطعام الانتقائية ولا يسري على قائمة الطعام المجهز مسبقاً ( Set Menu) • يسري العرض من الاحد الى الخميس من الساعة 1 م الى الساعة 6 م. • العرض لا يشمل تطبيقات التوصيل. • الخصم يشمل الفروع داخل السعودية في الرياض • لا يطبق العرض مع اي عروض اخرى ولا يمكن الجمع بين اكثر من عرض في نفس الوقت. • لا يسري العرض مع ايام المناسبات والاعياد والاجازات الرسمية مثال (اليوم الوطني – يوم ا</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B17" s="4"/>
+      <x:c r="C17" s="4"/>
+      <x:c r="D17" s="4"/>
       <x:c r="E17" s="5"/>
-      <x:c r="F17" s="5" t="n">
-        <x:v>45998.0</x:v>
-      </x:c>
-      <x:c r="G17" s="5" t="n">
-        <x:v>46346.0</x:v>
-      </x:c>
+      <x:c r="F17" s="5"/>
+      <x:c r="G17" s="5"/>
       <x:c r="H17" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16193,19 +15877,13 @@
       <x:c r="M17" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N17" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Robata-dec25</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N17" s="4"/>
       <x:c r="O17" s="4"/>
       <x:c r="P17" s="4"/>
       <x:c r="Q17" s="4"/>
       <x:c r="R17" s="4"/>
       <x:c r="S17" s="4"/>
-      <x:c r="T17" s="5" t="n">
-        <x:v>46260.29939116185</x:v>
-      </x:c>
+      <x:c r="T17" s="5"/>
       <x:c r="U17" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16214,28 +15892,12 @@
       <x:c r="A18" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B18" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C18" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء رائعة واستمتع بخصم 20% في كريزي بيتزا</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D18" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء رائعة واستمتع بخصم 20% في كريزي بيتزا الشروط والأحكام: • استمتع بأجواء رائعة في كريزي بيتزا واستمتع بخصم 20% عند الدفع باستخدام بطاقات الكاش باك من الإنماء باي • يسري العرض من 7 ديسمبر 2025 و حتى 20 نوفمبر 2026. • خصم 20% عند الدفع باستخدام بطاقات الكاش باك للإنماء باي خلال الفترة المشار إليها على جميع الطلبات من قائمة الطعام الانتقائية ولا يسري على قائمة الطعام المجهز مسبقاً ( Set Menu) • يسري العرض من الاحد الى الخميس من الساعة 1 م الى الساعة 6 م. • العرض لا يشمل تطبيقات التوصيل. • الخصم يشمل الفروع داخل السعودية: • الرياض فرع شارع التحلية طوال أيام الأسبوع وطوال اليوم • الرياض فرع عود سكوير من الأحد الى الخميس من 1 م حتى 6 م • الرياض فرع نورث يارد من الأحد الى الخميس من 1 م </x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B18" s="4"/>
+      <x:c r="C18" s="4"/>
+      <x:c r="D18" s="4"/>
       <x:c r="E18" s="5"/>
-      <x:c r="F18" s="5" t="n">
-        <x:v>45998.0</x:v>
-      </x:c>
-      <x:c r="G18" s="5" t="n">
-        <x:v>46346.0</x:v>
-      </x:c>
+      <x:c r="F18" s="5"/>
+      <x:c r="G18" s="5"/>
       <x:c r="H18" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16248,19 +15910,13 @@
       <x:c r="M18" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N18" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Crazy-Pizza-dec25</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N18" s="4"/>
       <x:c r="O18" s="4"/>
       <x:c r="P18" s="4"/>
       <x:c r="Q18" s="4"/>
       <x:c r="R18" s="4"/>
       <x:c r="S18" s="4"/>
-      <x:c r="T18" s="5" t="n">
-        <x:v>46260.29939116185</x:v>
-      </x:c>
+      <x:c r="T18" s="5"/>
       <x:c r="U18" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16269,28 +15925,12 @@
       <x:c r="A19" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B19" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C19" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء رائعة واستمتع بخصم 20% في كويا</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D19" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء رائعة واستمتع بخصم 20% في كويا الشروط والأحكام: • استمتع بأجواء رائعة في كويا واستمتع بخصم 20% عند الدفع باستخدام بطاقات الكاش باك من الإنماء باي • يسري العرض من 7 ديسمبر 2025 و حتى 20 نوفمبر 2026. • خصم 20% عند الدفع باستخدام بطاقات الكاش باك للإنماء باي خلال الفترة المشار إليها على جميع الطلبات من قائمة الطعام الانتقائية ولا يسري على قائمة الطعام المجهز مسبقاً ( Set Menu) • يسري العرض من الاحد الى الخميس من الساعة 1 م الى الساعة 6 م. • العرض لا يشمل تطبيقات التوصيل. • الخصم يشمل الفروع داخل السعودية في الرياض • لا يطبق العرض مع اي عروض اخرى ولا يمكن الجمع بين اكثر من عرض في نفس الوقت. • لا يسري العرض مع ايام المناسبات والاعياد والاجازات الرسمية مثال (اليوم الوطني – يوم التأسي</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B19" s="4"/>
+      <x:c r="C19" s="4"/>
+      <x:c r="D19" s="4"/>
       <x:c r="E19" s="5"/>
-      <x:c r="F19" s="5" t="n">
-        <x:v>45998.0</x:v>
-      </x:c>
-      <x:c r="G19" s="5" t="n">
-        <x:v>46346.0</x:v>
-      </x:c>
+      <x:c r="F19" s="5"/>
+      <x:c r="G19" s="5"/>
       <x:c r="H19" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16303,19 +15943,13 @@
       <x:c r="M19" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N19" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Coya-dec25</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N19" s="4"/>
       <x:c r="O19" s="4"/>
       <x:c r="P19" s="4"/>
       <x:c r="Q19" s="4"/>
       <x:c r="R19" s="4"/>
       <x:c r="S19" s="4"/>
-      <x:c r="T19" s="5" t="n">
-        <x:v>46260.29939116185</x:v>
-      </x:c>
+      <x:c r="T19" s="5"/>
       <x:c r="U19" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16324,28 +15958,12 @@
       <x:c r="A20" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B20" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C20" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء واستمتع بخصم 20% رائعة في سان كارلو شيكيتي</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D20" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء واستمتع بخصم 20% رائعة في سان كارلو شيكيتي الشروط والأحكام: • استمتع بأجواء رائعة في سان كارلو شيكيتي واستمتع بخصم 20% عند الدفع باستخدام بطاقات الكاش باك من الإنماء باي • يسري العرض من 7 ديسمبر 2025 و حتى 20 نوفمبر 2026. • خصم 20% عند الدفع باستخدام بطاقات الكاش باك للإنماء باي خلال الفترة المشار إليها على جميع الطلبات من قائمة الطعام الانتقائية ولا يسري على قائمة الطعام المجهز مسبقاً ( Set Menu) • يسري العرض من الاحد الى الخميس من الساعة 1 م الى الساعة 6 م. • العرض لا يشمل تطبيقات التوصيل. • الخصم يشمل الفروع داخل السعودية في الرياض وجده والخبر • لا يطبق العرض مع اي عروض اخرى ولا يمكن الجمع بين اكثر من عرض في نفس الوقت. • لا يسري العرض مع ايام المناسبات والاعياد والاجازات الر</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B20" s="4"/>
+      <x:c r="C20" s="4"/>
+      <x:c r="D20" s="4"/>
       <x:c r="E20" s="5"/>
-      <x:c r="F20" s="5" t="n">
-        <x:v>45998.0</x:v>
-      </x:c>
-      <x:c r="G20" s="5" t="n">
-        <x:v>46346.0</x:v>
-      </x:c>
+      <x:c r="F20" s="5"/>
+      <x:c r="G20" s="5"/>
       <x:c r="H20" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16358,19 +15976,13 @@
       <x:c r="M20" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N20" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/San-Carlo-Cicchetti-dec25</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N20" s="4"/>
       <x:c r="O20" s="4"/>
       <x:c r="P20" s="4"/>
       <x:c r="Q20" s="4"/>
       <x:c r="R20" s="4"/>
       <x:c r="S20" s="4"/>
-      <x:c r="T20" s="5" t="n">
-        <x:v>46260.29939116185</x:v>
-      </x:c>
+      <x:c r="T20" s="5"/>
       <x:c r="U20" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16379,28 +15991,12 @@
       <x:c r="A21" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B21" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C21" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء واستمتع بخصم 20% رائعة في سينيور ساسي</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D21" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء واستمتع بخصم 20% رائعة في سينيور ساسي الشروط والأحكام: • استمتع بأجواء رائعة في سينيور ساسي واستمتع بخصم 20% عند الدفع باستخدام بطاقات الكاش باك من الإنماء باي • يسري العرض من 7 ديسمبر 2025 و حتى 20 نوفمبر 2026. • خصم 20% عند الدفع باستخدام بطاقات الكاش باك للإنماء باي خلال الفترة المشار إليها على جميع الطلبات من قائمة الطعام الانتقائية ولا يسري على قائمة الطعام المجهز مسبقاً ( (Set Menu • يسري العرض من الاحد الى الخميس من الساعة 1 م الى الساعة 6 م. • العرض لا يشمل تطبيقات التوصيل. • الخصم يشمل الفروع داخل السعودية في الرياض • لا يطبق العرض مع اي عروض اخرى ولا يمكن الجمع بين اكثر من عرض في نفس الوقت. • لا يسري العرض مع ايام المناسبات والاعياد والاجازات الرسمية مثال (اليوم الوطن</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B21" s="4"/>
+      <x:c r="C21" s="4"/>
+      <x:c r="D21" s="4"/>
       <x:c r="E21" s="5"/>
-      <x:c r="F21" s="5" t="n">
-        <x:v>45998.0</x:v>
-      </x:c>
-      <x:c r="G21" s="5" t="n">
-        <x:v>46346.0</x:v>
-      </x:c>
+      <x:c r="F21" s="5"/>
+      <x:c r="G21" s="5"/>
       <x:c r="H21" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16413,19 +16009,13 @@
       <x:c r="M21" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N21" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Signor-Sassi-dec25</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N21" s="4"/>
       <x:c r="O21" s="4"/>
       <x:c r="P21" s="4"/>
       <x:c r="Q21" s="4"/>
       <x:c r="R21" s="4"/>
       <x:c r="S21" s="4"/>
-      <x:c r="T21" s="5" t="n">
-        <x:v>46260.29939116185</x:v>
-      </x:c>
+      <x:c r="T21" s="5"/>
       <x:c r="U21" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16434,28 +16024,12 @@
       <x:c r="A22" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B22" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C22" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء واستمتع بخصم 20% رائعة في كايزو</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D22" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء واستمتع بخصم 20% رائعة في كايزو الشروط والأحكام: • استمتع بأجواء رائعة في كايزو واستمتع بخصم 20% عند الدفع باستخدام بطاقات الكاش باك من الإنماء باي • يسري العرض من 7 ديسمبر 2025 و حتى 20 نوفمبر 2026. • خصم 20% عند الدفع باستخدام بطاقات الكاش باك للإنماء باي خلال الفترة المشار إليها على جميع الطلبات من قائمة الطعام الانتقائية ولا يسري على قائمة الطعام المجهز مسبقاً ( Set Menu) • يسري العرض من الاحد الى الخميس من الساعة 1 م الى الساعة 6 م. • العرض لا يشمل تطبيقات التوصيل. • الخصم يشمل الفروع داخل السعودية في الرياض • لا يطبق العرض مع اي عروض اخرى ولا يمكن الجمع بين اكثر من عرض في نفس الوقت. • لا يسري العرض مع ايام المناسبات والاعياد والاجازات الرسمية مثال (اليوم الوطني – يوم التأ</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B22" s="4"/>
+      <x:c r="C22" s="4"/>
+      <x:c r="D22" s="4"/>
       <x:c r="E22" s="5"/>
-      <x:c r="F22" s="5" t="n">
-        <x:v>45998.0</x:v>
-      </x:c>
-      <x:c r="G22" s="5" t="n">
-        <x:v>46346.0</x:v>
-      </x:c>
+      <x:c r="F22" s="5"/>
+      <x:c r="G22" s="5"/>
       <x:c r="H22" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16468,19 +16042,13 @@
       <x:c r="M22" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N22" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Kayzo-dec25</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N22" s="4"/>
       <x:c r="O22" s="4"/>
       <x:c r="P22" s="4"/>
       <x:c r="Q22" s="4"/>
       <x:c r="R22" s="4"/>
       <x:c r="S22" s="4"/>
-      <x:c r="T22" s="5" t="n">
-        <x:v>46260.29939116185</x:v>
-      </x:c>
+      <x:c r="T22" s="5"/>
       <x:c r="U22" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16489,28 +16057,12 @@
       <x:c r="A23" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B23" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C23" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء واستمتع بخصم 20% رائعة في ميازو</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D23" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بأجواء واستمتع بخصم 20% رائعة في ميازو الشروط والأحكام: • استمتع بأجواء رائعة في ميازو واستمتع بخصم 20% عند الدفع باستخدام بطاقات الكاش باك من الإنماء باي • يسري العرض من 7 ديسمبر 2025 و حتى 20 نوفمبر 2026. • خصم 20% عند الدفع باستخدام بطاقات الكاش باك للإنماء باي خلال الفترة المشار إليها على جميع الطلبات من قائمة الطعام الانتقائية ولا يسري على قائمة الطعام المجهز مسبقاً ( Set Menu) • يسري العرض من الاحد الى الخميس من الساعة 1 م الى الساعة 6 م. • العرض لا يشمل تطبيقات التوصيل. • الخصم يشمل الفروع داخل السعودية في الرياض • لا يطبق العرض مع اي عروض اخرى ولا يمكن الجمع بين اكثر من عرض في نفس الوقت. • لا يسري العرض مع ايام المناسبات والاعياد والاجازات الرسمية مثال (اليوم الوطني – يوم التأ</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B23" s="4"/>
+      <x:c r="C23" s="4"/>
+      <x:c r="D23" s="4"/>
       <x:c r="E23" s="5"/>
-      <x:c r="F23" s="5" t="n">
-        <x:v>45998.0</x:v>
-      </x:c>
-      <x:c r="G23" s="5" t="n">
-        <x:v>46346.0</x:v>
-      </x:c>
+      <x:c r="F23" s="5"/>
+      <x:c r="G23" s="5"/>
       <x:c r="H23" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16523,19 +16075,13 @@
       <x:c r="M23" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N23" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/MYAZU-dec25</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N23" s="4"/>
       <x:c r="O23" s="4"/>
       <x:c r="P23" s="4"/>
       <x:c r="Q23" s="4"/>
       <x:c r="R23" s="4"/>
       <x:c r="S23" s="4"/>
-      <x:c r="T23" s="5" t="n">
-        <x:v>46260.29939116185</x:v>
-      </x:c>
+      <x:c r="T23" s="5"/>
       <x:c r="U23" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16544,28 +16090,12 @@
       <x:c r="A24" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B24" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C24" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بخصم 15% لدى المهيدب ريزدنس</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D24" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">• استمتع بخصم 15 % لدى المهيدب ريزدنس عند الدفع بأي من بطاقات الإنماء باي فيزا أو مدى. • يسري العرض من تاريخ 5 فبراير حتى 30 يناير 2027.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B24" s="4"/>
+      <x:c r="C24" s="4"/>
+      <x:c r="D24" s="4"/>
       <x:c r="E24" s="5"/>
-      <x:c r="F24" s="5" t="n">
-        <x:v>46423.0</x:v>
-      </x:c>
-      <x:c r="G24" s="5" t="n">
-        <x:v>46417.0</x:v>
-      </x:c>
+      <x:c r="F24" s="5"/>
+      <x:c r="G24" s="5"/>
       <x:c r="H24" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16578,19 +16108,13 @@
       <x:c r="M24" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N24" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Al-Muhaidb-Offer---Feb-2026</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N24" s="4"/>
       <x:c r="O24" s="4"/>
       <x:c r="P24" s="4"/>
       <x:c r="Q24" s="4"/>
       <x:c r="R24" s="4"/>
       <x:c r="S24" s="4"/>
-      <x:c r="T24" s="5" t="n">
-        <x:v>46260.29939116185</x:v>
-      </x:c>
+      <x:c r="T24" s="5"/>
       <x:c r="U24" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16599,28 +16123,12 @@
       <x:c r="A25" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B25" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C25" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بخصم 15% لدى فنادق إيواء</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D25" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">• استمتع بخصم 15 % لدى المهيدب ريزدنس عند الدفع بأي من بطاقات الإنماء باي فيزا أو مدى. يسري العرض من تاريخ 5 فبراير حتى 30 يناير 2027.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B25" s="4"/>
+      <x:c r="C25" s="4"/>
+      <x:c r="D25" s="4"/>
       <x:c r="E25" s="5"/>
-      <x:c r="F25" s="5" t="n">
-        <x:v>46423.0</x:v>
-      </x:c>
-      <x:c r="G25" s="5" t="n">
-        <x:v>46417.0</x:v>
-      </x:c>
+      <x:c r="F25" s="5"/>
+      <x:c r="G25" s="5"/>
       <x:c r="H25" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16633,19 +16141,13 @@
       <x:c r="M25" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N25" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/EWAA-Hotels-Offer---Feb-2026</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N25" s="4"/>
       <x:c r="O25" s="4"/>
       <x:c r="P25" s="4"/>
       <x:c r="Q25" s="4"/>
       <x:c r="R25" s="4"/>
       <x:c r="S25" s="4"/>
-      <x:c r="T25" s="5" t="n">
-        <x:v>46260.29939116185</x:v>
-      </x:c>
+      <x:c r="T25" s="5"/>
       <x:c r="U25" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16654,28 +16156,12 @@
       <x:c r="A26" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B26" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C26" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بخصم 15% لدى فنادق جراند بلازا</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D26" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">• استمتع بخصم 15 % لدى فنادق جراند بلازا عند الدفع بأي من بطاقات الإنماء باي فيزا أو مدى. • يسري العرض من تاريخ 5 فبراير حتى 30 يناير 2027.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B26" s="4"/>
+      <x:c r="C26" s="4"/>
+      <x:c r="D26" s="4"/>
       <x:c r="E26" s="5"/>
-      <x:c r="F26" s="5" t="n">
-        <x:v>46423.0</x:v>
-      </x:c>
-      <x:c r="G26" s="5" t="n">
-        <x:v>46417.0</x:v>
-      </x:c>
+      <x:c r="F26" s="5"/>
+      <x:c r="G26" s="5"/>
       <x:c r="H26" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16688,19 +16174,13 @@
       <x:c r="M26" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N26" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Grand-Plaza-Hotels---Feb-2026</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N26" s="4"/>
       <x:c r="O26" s="4"/>
       <x:c r="P26" s="4"/>
       <x:c r="Q26" s="4"/>
       <x:c r="R26" s="4"/>
       <x:c r="S26" s="4"/>
-      <x:c r="T26" s="5" t="n">
-        <x:v>46260.29939116185</x:v>
-      </x:c>
+      <x:c r="T26" s="5"/>
       <x:c r="U26" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16709,28 +16189,12 @@
       <x:c r="A27" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B27" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C27" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بخصم 30% لدى ستايلي</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D27" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">• استمتع بخصم 30% لدى ستايلي عند الدفع بأي من بطاقات الإنماء باي فيزا. • يسري العرض من تاريخ 5 فبراير حتى 30 ديسمبر 2026.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B27" s="4"/>
+      <x:c r="C27" s="4"/>
+      <x:c r="D27" s="4"/>
       <x:c r="E27" s="5"/>
-      <x:c r="F27" s="5" t="n">
-        <x:v>46058.0</x:v>
-      </x:c>
-      <x:c r="G27" s="5" t="n">
-        <x:v>46386.0</x:v>
-      </x:c>
+      <x:c r="F27" s="5"/>
+      <x:c r="G27" s="5"/>
       <x:c r="H27" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16743,19 +16207,13 @@
       <x:c r="M27" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N27" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Stily-Offer---Feb-2026</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N27" s="4"/>
       <x:c r="O27" s="4"/>
       <x:c r="P27" s="4"/>
       <x:c r="Q27" s="4"/>
       <x:c r="R27" s="4"/>
       <x:c r="S27" s="4"/>
-      <x:c r="T27" s="5" t="n">
-        <x:v>46260.29939116185</x:v>
-      </x:c>
+      <x:c r="T27" s="5"/>
       <x:c r="U27" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16764,28 +16222,12 @@
       <x:c r="A28" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B28" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C28" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">تسوّق من FARFETCH</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D28" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بخصم يصل حتى 500 ريال لدى FARFETCH عند الدفع باستخدام أي من بطاقات الإنماء باي فيزا. يسري العرض من 15 يناير وحتى 31 ديسمبر 2026 .</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B28" s="4"/>
+      <x:c r="C28" s="4"/>
+      <x:c r="D28" s="4"/>
       <x:c r="E28" s="5"/>
-      <x:c r="F28" s="5" t="n">
-        <x:v>46037.0</x:v>
-      </x:c>
-      <x:c r="G28" s="5" t="n">
-        <x:v>46387.0</x:v>
-      </x:c>
+      <x:c r="F28" s="5"/>
+      <x:c r="G28" s="5"/>
       <x:c r="H28" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16798,19 +16240,13 @@
       <x:c r="M28" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N28" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Shop-on-FARFETCH---Jan-2026</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N28" s="4"/>
       <x:c r="O28" s="4"/>
       <x:c r="P28" s="4"/>
       <x:c r="Q28" s="4"/>
       <x:c r="R28" s="4"/>
       <x:c r="S28" s="4"/>
-      <x:c r="T28" s="5" t="n">
-        <x:v>46259.82478451854</x:v>
-      </x:c>
+      <x:c r="T28" s="5"/>
       <x:c r="U28" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16819,28 +16255,12 @@
       <x:c r="A29" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B29" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C29" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">خصم 20% لدى سيار</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D29" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بخصم 20% لدى سيار (Sayyar) عند الدفع باستخدام بطاقات الإنماء باي . يسري العرض من 1 يناير 2026 حتى 31 ديسمبر 2026 .</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B29" s="4"/>
+      <x:c r="C29" s="4"/>
+      <x:c r="D29" s="4"/>
       <x:c r="E29" s="5"/>
-      <x:c r="F29" s="5" t="n">
-        <x:v>46023.0</x:v>
-      </x:c>
-      <x:c r="G29" s="5" t="n">
-        <x:v>46387.0</x:v>
-      </x:c>
+      <x:c r="F29" s="5"/>
+      <x:c r="G29" s="5"/>
       <x:c r="H29" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16853,19 +16273,13 @@
       <x:c r="M29" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N29" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Sayyar---April2026</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N29" s="4"/>
       <x:c r="O29" s="4"/>
       <x:c r="P29" s="4"/>
       <x:c r="Q29" s="4"/>
       <x:c r="R29" s="4"/>
       <x:c r="S29" s="4"/>
-      <x:c r="T29" s="5" t="n">
-        <x:v>46260.29939116185</x:v>
-      </x:c>
+      <x:c r="T29" s="5"/>
       <x:c r="U29" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16874,28 +16288,12 @@
       <x:c r="A30" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B30" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Card</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C30" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">صفر رسوم على المشتريات الدولية</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D30" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بصفر رسوم على مشترياتك الدولية مع بطاقة الإنماء باي كاش باك صفر رسوم على عمليات الشراء الدولية عبر نقاط البيع خارج المملكة العربية السعودية.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B30" s="4"/>
+      <x:c r="C30" s="4"/>
+      <x:c r="D30" s="4"/>
       <x:c r="E30" s="5"/>
-      <x:c r="F30" s="5" t="n">
-        <x:v>46197.0</x:v>
-      </x:c>
-      <x:c r="G30" s="5" t="n">
-        <x:v>46265.0</x:v>
-      </x:c>
+      <x:c r="F30" s="5"/>
+      <x:c r="G30" s="5"/>
       <x:c r="H30" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16908,19 +16306,13 @@
       <x:c r="M30" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N30" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/OIF-JUN2026</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N30" s="4"/>
       <x:c r="O30" s="4"/>
       <x:c r="P30" s="4"/>
       <x:c r="Q30" s="4"/>
       <x:c r="R30" s="4"/>
       <x:c r="S30" s="4"/>
-      <x:c r="T30" s="5" t="n">
-        <x:v>46259.82478451854</x:v>
-      </x:c>
+      <x:c r="T30" s="5"/>
       <x:c r="U30" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16929,28 +16321,12 @@
       <x:c r="A31" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B31" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C31" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">عرض آيهيرب 40%</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D31" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بخصم 40% على مشترياتك من آيهيرب عند الدفع ببطاقات الإنماء باي فيزا . يسري العرض من 21 أغسطس 2026 حتى 4 سبتمبر 2026 .</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B31" s="4"/>
+      <x:c r="C31" s="4"/>
+      <x:c r="D31" s="4"/>
       <x:c r="E31" s="5"/>
-      <x:c r="F31" s="5" t="n">
-        <x:v>46255.0</x:v>
-      </x:c>
-      <x:c r="G31" s="5" t="n">
-        <x:v>46269.0</x:v>
-      </x:c>
+      <x:c r="F31" s="5"/>
+      <x:c r="G31" s="5"/>
       <x:c r="H31" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -16963,19 +16339,13 @@
       <x:c r="M31" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N31" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/iHerb_Aug_2026</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N31" s="4"/>
       <x:c r="O31" s="4"/>
       <x:c r="P31" s="4"/>
       <x:c r="Q31" s="4"/>
       <x:c r="R31" s="4"/>
       <x:c r="S31" s="4"/>
-      <x:c r="T31" s="5" t="n">
-        <x:v>46259.82478451854</x:v>
-      </x:c>
+      <x:c r="T31" s="5"/>
       <x:c r="U31" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -16984,28 +16354,12 @@
       <x:c r="A32" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B32" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Other</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C32" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">عرض الهند على رسوم التحويلات الدولية</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D32" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">حوّل دولياً إلى الهند برسوم ثابتة 5 ريال فقط عبر خدمة alinmapay Direct ، إلى الهند. رسوم تحويل دولية ثابتة بقيمة 5 ريال عبر خدمة alinmapay Direct .</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B32" s="4"/>
+      <x:c r="C32" s="4"/>
+      <x:c r="D32" s="4"/>
       <x:c r="E32" s="5"/>
-      <x:c r="F32" s="5" t="n">
-        <x:v>46242.0</x:v>
-      </x:c>
-      <x:c r="G32" s="5" t="n">
-        <x:v>46387.0</x:v>
-      </x:c>
+      <x:c r="F32" s="5"/>
+      <x:c r="G32" s="5"/>
       <x:c r="H32" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -17018,23 +16372,13 @@
       <x:c r="M32" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N32" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/India-Transfer-Fee-Offer-Aug26</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N32" s="4"/>
       <x:c r="O32" s="4"/>
       <x:c r="P32" s="4"/>
       <x:c r="Q32" s="4"/>
-      <x:c r="R32" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.tiktok.com/@alinmapay/video/7586667265882443024</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="R32" s="4"/>
       <x:c r="S32" s="4"/>
-      <x:c r="T32" s="5" t="n">
-        <x:v>46259.82478451854</x:v>
-      </x:c>
+      <x:c r="T32" s="5"/>
       <x:c r="U32" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -17043,28 +16387,12 @@
       <x:c r="A33" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B33" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Other</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C33" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">عرض اليمن: كاش باك 5 ريال</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D33" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">حوّل إلى اليمن عبر خدمة مباشر الإنماء باي واستمتع بكاش باك 5 ريال بعد إتمام 3 عمليات تحويل. استمتع بكاش باك 5 ريال بعد إتمام 3 عمليات تحويل إلى اليمن عبر خدمة مباشر الإنماء باي.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B33" s="4"/>
+      <x:c r="C33" s="4"/>
+      <x:c r="D33" s="4"/>
       <x:c r="E33" s="5"/>
-      <x:c r="F33" s="5" t="n">
-        <x:v>46230.0</x:v>
-      </x:c>
-      <x:c r="G33" s="5" t="n">
-        <x:v>46261.0</x:v>
-      </x:c>
+      <x:c r="F33" s="5"/>
+      <x:c r="G33" s="5"/>
       <x:c r="H33" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -17077,19 +16405,13 @@
       <x:c r="M33" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N33" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Yemen-Cashback-5SAR</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N33" s="4"/>
       <x:c r="O33" s="4"/>
       <x:c r="P33" s="4"/>
       <x:c r="Q33" s="4"/>
       <x:c r="R33" s="4"/>
       <x:c r="S33" s="4"/>
-      <x:c r="T33" s="5" t="n">
-        <x:v>46259.82478451854</x:v>
-      </x:c>
+      <x:c r="T33" s="5"/>
       <x:c r="U33" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -17098,28 +16420,12 @@
       <x:c r="A34" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B34" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C34" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">عرض شي إن 20%</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D34" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بخصم 20% على مشترياتك من شي إن عند الدفع ببطاقات الإنماء باي فيزا . يسري العرض من 21 أغسطس 2026 حتى 4 سبتمبر 2026 .</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B34" s="4"/>
+      <x:c r="C34" s="4"/>
+      <x:c r="D34" s="4"/>
       <x:c r="E34" s="5"/>
-      <x:c r="F34" s="5" t="n">
-        <x:v>46255.0</x:v>
-      </x:c>
-      <x:c r="G34" s="5" t="n">
-        <x:v>46269.0</x:v>
-      </x:c>
+      <x:c r="F34" s="5"/>
+      <x:c r="G34" s="5"/>
       <x:c r="H34" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -17132,19 +16438,13 @@
       <x:c r="M34" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N34" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/SHEIN_Aug_2026</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N34" s="4"/>
       <x:c r="O34" s="4"/>
       <x:c r="P34" s="4"/>
       <x:c r="Q34" s="4"/>
       <x:c r="R34" s="4"/>
       <x:c r="S34" s="4"/>
-      <x:c r="T34" s="5" t="n">
-        <x:v>46259.82478451854</x:v>
-      </x:c>
+      <x:c r="T34" s="5"/>
       <x:c r="U34" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -17153,28 +16453,12 @@
       <x:c r="A35" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B35" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C35" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">عين لندن: خصم 15%</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D35" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بخصم 15% لدى عين لندن على التذاكر العادية عند الدفع بأي من بطاقات الإنماء باي فيزا . يسري العرض من 19 أغسطس حتى 30 سبتمبر 2026 .</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B35" s="4"/>
+      <x:c r="C35" s="4"/>
+      <x:c r="D35" s="4"/>
       <x:c r="E35" s="5"/>
-      <x:c r="F35" s="5" t="n">
-        <x:v>46253.0</x:v>
-      </x:c>
-      <x:c r="G35" s="5" t="n">
-        <x:v>46295.0</x:v>
-      </x:c>
+      <x:c r="F35" s="5"/>
+      <x:c r="G35" s="5"/>
       <x:c r="H35" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -17187,19 +16471,13 @@
       <x:c r="M35" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N35" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/LendonEye_2026</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N35" s="4"/>
       <x:c r="O35" s="4"/>
       <x:c r="P35" s="4"/>
       <x:c r="Q35" s="4"/>
       <x:c r="R35" s="4"/>
       <x:c r="S35" s="4"/>
-      <x:c r="T35" s="5" t="n">
-        <x:v>46259.82478451854</x:v>
-      </x:c>
+      <x:c r="T35" s="5"/>
       <x:c r="U35" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -17208,26 +16486,12 @@
       <x:c r="A36" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B36" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Musaned</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C36" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">كاش باك 100% على رواتب عمالتك المنزلية</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D36" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">حوّل راتب العمالة المنزلية بنجاح عبر خدمة مساند في تطبيق الإنماء باي ، وادخل السحب الشهري تلقائياً لتسترجع قيمة الراتب بالكامل في محفظتك! تبدأ الحملة من 28 يوليو 2026م وحتى 28 ديسمبر 2026م .</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B36" s="4"/>
+      <x:c r="C36" s="4"/>
+      <x:c r="D36" s="4"/>
       <x:c r="E36" s="5"/>
       <x:c r="F36" s="5"/>
-      <x:c r="G36" s="5" t="n">
-        <x:v>46384.0</x:v>
-      </x:c>
+      <x:c r="G36" s="5"/>
       <x:c r="H36" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -17240,31 +16504,13 @@
       <x:c r="M36" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N36" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Musaned-Cashback</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O36" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.instagram.com/p/DbqaY05mm9E</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P36" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://x.com/alinmapay/status/2082127730972176680</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q36" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://m.facebook.com/AlinmaPaySA/posts/pfbid02qzFxmfE6Ajm5LhhKy4EVeNqAVycQERoEyiAKqjyHfBhKQ13AdTQGqE9Wcrs39Fucl</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N36" s="4"/>
+      <x:c r="O36" s="4"/>
+      <x:c r="P36" s="4"/>
+      <x:c r="Q36" s="4"/>
       <x:c r="R36" s="4"/>
       <x:c r="S36" s="4"/>
-      <x:c r="T36" s="5" t="n">
-        <x:v>46259.82478451854</x:v>
-      </x:c>
+      <x:c r="T36" s="5"/>
       <x:c r="U36" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -17273,28 +16519,12 @@
       <x:c r="A37" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B37" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C37" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">كيمارت: خصم 70 ريال</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D37" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بخصم يصل حتى 70 ريالاً لدى كيمارت عند الدفع باستخدام أي من بطاقات الإنماء باي كاش باك . حالة العميل (جديد/حالي) تحدد حسب حساب المستخدم في تطبيق كيمارت</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B37" s="4"/>
+      <x:c r="C37" s="4"/>
+      <x:c r="D37" s="4"/>
       <x:c r="E37" s="5"/>
-      <x:c r="F37" s="5" t="n">
-        <x:v>46254.0</x:v>
-      </x:c>
-      <x:c r="G37" s="5" t="n">
-        <x:v>46276.0</x:v>
-      </x:c>
+      <x:c r="F37" s="5"/>
+      <x:c r="G37" s="5"/>
       <x:c r="H37" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -17307,19 +16537,13 @@
       <x:c r="M37" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N37" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/Keemart_Aug_2026</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N37" s="4"/>
       <x:c r="O37" s="4"/>
       <x:c r="P37" s="4"/>
       <x:c r="Q37" s="4"/>
       <x:c r="R37" s="4"/>
       <x:c r="S37" s="4"/>
-      <x:c r="T37" s="5" t="n">
-        <x:v>46259.82478451854</x:v>
-      </x:c>
+      <x:c r="T37" s="5"/>
       <x:c r="U37" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -17328,28 +16552,12 @@
       <x:c r="A38" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B38" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C38" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">ليجو لاند: خصم 15%</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D38" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بخصم 15% لدى ليجو لاند على تذاكر الدخول ليوم كامل عند الدفع بأي من بطاقات الإنماء باي فيزا . يسري العرض من 19 أغسطس حتى 30 سبتمبر 2026 .</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B38" s="4"/>
+      <x:c r="C38" s="4"/>
+      <x:c r="D38" s="4"/>
       <x:c r="E38" s="5"/>
-      <x:c r="F38" s="5" t="n">
-        <x:v>46253.0</x:v>
-      </x:c>
-      <x:c r="G38" s="5" t="n">
-        <x:v>46295.0</x:v>
-      </x:c>
+      <x:c r="F38" s="5"/>
+      <x:c r="G38" s="5"/>
       <x:c r="H38" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -17362,19 +16570,13 @@
       <x:c r="M38" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N38" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/LegoLand_2026</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N38" s="4"/>
       <x:c r="O38" s="4"/>
       <x:c r="P38" s="4"/>
       <x:c r="Q38" s="4"/>
       <x:c r="R38" s="4"/>
       <x:c r="S38" s="4"/>
-      <x:c r="T38" s="5" t="n">
-        <x:v>46259.82478451854</x:v>
-      </x:c>
+      <x:c r="T38" s="5"/>
       <x:c r="U38" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>
@@ -17383,28 +16585,12 @@
       <x:c r="A39" s="8" t="str">
         <x:f t="shared" si="0"/>
       </x:c>
-      <x:c r="B39" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Merchant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C39" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">مدام تيسو: خصم 15%</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D39" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">استمتع بخصم 15% لدى مدام تيسو على التذاكر العادية عند الدفع بأي من بطاقات الإنماء باي فيزا . يسري العرض من 19 أغسطس حتى 30 سبتمبر 2026 .</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B39" s="4"/>
+      <x:c r="C39" s="4"/>
+      <x:c r="D39" s="4"/>
       <x:c r="E39" s="5"/>
-      <x:c r="F39" s="5" t="n">
-        <x:v>46253.0</x:v>
-      </x:c>
-      <x:c r="G39" s="5" t="n">
-        <x:v>46295.0</x:v>
-      </x:c>
+      <x:c r="F39" s="5"/>
+      <x:c r="G39" s="5"/>
       <x:c r="H39" s="7" t="str">
         <x:f t="shared" si="1"/>
       </x:c>
@@ -17417,19 +16603,13 @@
       <x:c r="M39" s="9" t="str">
         <x:f t="shared" si="3"/>
       </x:c>
-      <x:c r="N39" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.alinmapay.com.sa/Offers/MADAME-TUSSAUDS_2026</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="N39" s="4"/>
       <x:c r="O39" s="4"/>
       <x:c r="P39" s="4"/>
       <x:c r="Q39" s="4"/>
       <x:c r="R39" s="4"/>
       <x:c r="S39" s="4"/>
-      <x:c r="T39" s="5" t="n">
-        <x:v>46259.82478451854</x:v>
-      </x:c>
+      <x:c r="T39" s="5"/>
       <x:c r="U39" s="35" t="str">
         <x:f t="shared" si="4"/>
       </x:c>

</xml_diff>